<commit_message>
Permite foto em qualquer nó, não só em quem tem perfil completo
Adiciona 4 colunas opcionais na aba Nodes (Foto, Crédito, Link da
fonte, Nota) para colocar foto numa pessoa mesmo sem perfil pesquisado
na aba Perfis. Quando há perfil completo, a foto da aba Perfis
continua prevalecendo. Refatora a geração de HTML da foto num helper
único (photoHtml) reaproveitado nos dois casos.

Nenhuma linha usa esse campo ainda — só a infraestrutura, sem mudança
visual no site por enquanto.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -3499,7 +3499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -3539,6 +3539,26 @@
       <c r="F1" s="44" t="inlineStr">
         <is>
           <t>Degree</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Foto (arquivo)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Crédito da foto</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Link da fonte da foto</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Nota da foto (opcional)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fotos para instituições/empresas/bens + corrige foco preso após reset
Fotos (26 novas, via colunas de foto da aba Nodes):
- Fotos reais de sede/prédio para instituições e empresas identificáveis
  (TSE, STF, PF, PGR, Abin, Receita, Santander, CPI).
- Fotos ilustrativas (genéricas, licença livre) para bens privados sem
  imagem pública real (mansão, apartamento, triplex, jato, casa, fábrica,
  banco, etc.) — sempre com aviso "Imagem ilustrativa" visível no cartão,
  nunca apresentadas como o imóvel/objeto real.
- photos/CREDITS.md documenta fonte e licença de cada uma.

Bug: "Mostrar tudo" limpava os filtros de grupo mas não o nó selecionado,
então o mapa continuava mostrando só os vizinhos de quem estava focado
(resto meio apagado) em vez de voltar à visão geral de verdade. Agora
também limpa a seleção.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -3541,22 +3541,22 @@
           <t>Degree</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>Foto (arquivo)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>Crédito da foto</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>Link da fonte da foto</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>Nota da foto (opcional)</t>
         </is>
@@ -3592,6 +3592,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A2)+COUNTIF(Edges!$B$2:$B$120,A2)</f>
         <v/>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>assoc.jpg</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata a sede real</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="23.25" customHeight="1" s="25">
       <c r="A3" s="45" t="inlineStr">
@@ -3778,6 +3798,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A8)+COUNTIF(Edges!$B$2:$B$120,A8)</f>
         <v/>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>sala.jpg</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata a sede real</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="25">
       <c r="A9" s="45" t="inlineStr">
@@ -3809,6 +3849,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A9)+COUNTIF(Edges!$B$2:$B$120,A9)</f>
         <v/>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>bravo.jpg</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Samuel Zeller · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Assembly_Line_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — linha de produção genérica, não retrata a fábrica real</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="25">
       <c r="A10" s="45" t="inlineStr">
@@ -3871,6 +3931,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A11)+COUNTIF(Edges!$B$2:$B$120,A11)</f>
         <v/>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>escw.jpg</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata a sede real</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
       <c r="A12" s="45" t="inlineStr">
@@ -3902,6 +3982,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A12)+COUNTIF(Edges!$B$2:$B$120,A12)</f>
         <v/>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>bets.jpg</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Maximo Betman · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Mesa-de-ruleta-casino-ciudad-de-mexico25-04-2023.jpg</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — mesa de cassino genérica, não retrata a empresa real</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="45" t="inlineStr">
@@ -3964,6 +4064,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A14)+COUNTIF(Edges!$B$2:$B$120,A14)</f>
         <v/>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>wt.jpg</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata a sede real</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="45" t="inlineStr">
@@ -3995,6 +4115,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A15)+COUNTIF(Edges!$B$2:$B$120,A15)</f>
         <v/>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>alcazar.jpg</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata a sede real</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
       <c r="A16" s="45" t="inlineStr">
@@ -4026,6 +4166,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A16)+COUNTIF(Edges!$B$2:$B$120,A16)</f>
         <v/>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>santander.jpg</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Simplus Menegati · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Agencia_Banco_Santander_de_Telemaco_Borba.jpg</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
       <c r="A17" s="45" t="inlineStr">
@@ -4057,6 +4213,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A17)+COUNTIF(Edges!$B$2:$B$120,A17)</f>
         <v/>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>cpi.jpg</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Agência Senado · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:CPIPANDEMIA_-_Comiss%C3%A3o_Parlamentar_de_Inqu%C3%A9rito_da_Pandemia_(1).jpg</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="45" t="inlineStr">
@@ -4212,6 +4384,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A22)+COUNTIF(Edges!$B$2:$B$120,A22)</f>
         <v/>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>escf.jpg</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata a sede real</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
       <c r="A23" s="45" t="inlineStr">
@@ -4243,6 +4435,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A23)+COUNTIF(Edges!$B$2:$B$120,A23)</f>
         <v/>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ong.jpg</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata a sede real</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
       <c r="A24" s="45" t="inlineStr">
@@ -4460,6 +4672,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A30)+COUNTIF(Edges!$B$2:$B$120,A30)</f>
         <v/>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>master.jpg</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Anthony Esau · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Farm_Credit_Bank_Building_2016_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — agência bancária genérica, não retrata o Banco Master</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
       <c r="A31" s="45" t="inlineStr">
@@ -4553,6 +4785,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A33)+COUNTIF(Edges!$B$2:$B$120,A33)</f>
         <v/>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>primeu.jpg</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata a sede real</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
       <c r="A34" s="45" t="inlineStr">
@@ -4584,6 +4836,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A34)+COUNTIF(Edges!$B$2:$B$120,A34)</f>
         <v/>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>luri.jpg</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata a sede real</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="23.25" customHeight="1" s="25">
       <c r="A35" s="45" t="inlineStr">
@@ -4708,6 +4980,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A38)+COUNTIF(Edges!$B$2:$B$120,A38)</f>
         <v/>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>angra.jpg</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Tim Gouw · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Drone_pool_and_deck_chairs_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata o imóvel real</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
       <c r="A39" s="45" t="inlineStr">
@@ -4739,6 +5031,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A39)+COUNTIF(Edges!$B$2:$B$120,A39)</f>
         <v/>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>aptosp.jpg</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Grant Lemons · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Modern_apartment_building_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata o imóvel real</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
       <c r="A40" s="45" t="inlineStr">
@@ -4770,6 +5082,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A40)+COUNTIF(Edges!$B$2:$B$120,A40)</f>
         <v/>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>triplex.jpg</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Grant Lemons · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Modern_apartment_building_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata o imóvel real</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="23.25" customHeight="1" s="25">
       <c r="A41" s="45" t="inlineStr">
@@ -4801,6 +5133,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A41)+COUNTIF(Edges!$B$2:$B$120,A41)</f>
         <v/>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>jato.jpg</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Checkerberry · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Flexjet_Embraer_EMB-545_Praetor_500_(N446FX)_Landing_Runway_22_at_KLEX.jpg</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — jato executivo genérico, não retrata a aeronave real</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
       <c r="A42" s="45" t="inlineStr">
@@ -4832,6 +5184,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A42)+COUNTIF(Edges!$B$2:$B$120,A42)</f>
         <v/>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>atibaia.jpg</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Ritchie Valens · CC0 (Unsplash via Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Cozy_Cottage_Home_(Unsplash).jpg</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — não retrata o imóvel real</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
       <c r="A43" s="45" t="inlineStr">
@@ -5018,6 +5390,26 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A48)+COUNTIF(Edges!$B$2:$B$120,A48)</f>
         <v/>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>coaf.jpg</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>frankieleon · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Scales_of_Justice_(3285348799).jpg</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Imagem ilustrativa — símbolo da justiça, não retrata o caso real</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
       <c r="A49" s="45" t="inlineStr">
@@ -5142,6 +5534,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A52)+COUNTIF(Edges!$B$2:$B$120,A52)</f>
         <v/>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>abin.jpg</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Antonio Cruz/Agência Brasil · CC BY 3.0 BR</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Pr%C3%A9dio_da_Abin.jpg</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
       <c r="A53" s="45" t="inlineStr">
@@ -5173,6 +5581,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A53)+COUNTIF(Edges!$B$2:$B$120,A53)</f>
         <v/>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>receita.jpg</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Academia de Letras de Campo Maior · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Ag%C3%AAncia_da_Receita_Federal_de_Campo_Maior,_Piau%C3%AD,_Brasil.JPG</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
       <c r="A54" s="45" t="inlineStr">
@@ -5204,6 +5628,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A54)+COUNTIF(Edges!$B$2:$B$120,A54)</f>
         <v/>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>pf.jpg</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Agência Senado · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Sede_da_Pol%C3%ADcia_Federal_(52830107256).jpg</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
       <c r="A55" s="45" t="inlineStr">
@@ -5235,6 +5675,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A55)+COUNTIF(Edges!$B$2:$B$120,A55)</f>
         <v/>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>pgr.jpg</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Webysther · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Webysther_20180212174501_-_PGR_-_Procuradoria_Geral_da_Rep%C3%BAblica.jpg</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56" ht="23.25" customHeight="1" s="25">
       <c r="A56" s="45" t="inlineStr">
@@ -5297,6 +5753,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A57)+COUNTIF(Edges!$B$2:$B$120,A57)</f>
         <v/>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>stf.jpg</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Daderot · CC0 (domínio público)</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Supremo_Tribunal_Federal_building_in_Brasilia_-_DSC00288.JPG</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
       <c r="A58" s="45" t="inlineStr">
@@ -5328,6 +5800,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A58)+COUNTIF(Edges!$B$2:$B$120,A58)</f>
         <v/>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>tse.jpg</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Alexandresena · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Sede_do_Tribunal_Superior_Eleitoral,_em_Bras%C3%ADlia.jpg</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F58"/>

</xml_diff>

<commit_message>
Troca fotos ilustrativas por logo real da Blaze; remove o resto
A Blaze agora usa o logo oficial (domínio público, simples demais pra
direito autoral) em vez de uma foto genérica de cassino. CSS ajustado
pra logos PNG usarem object-fit: contain, senão o wordmark cortava.

As outras 17 fotos ilustrativas (mansão, jato, triplex, apartamento,
casa, fábrica, escritórios genéricos, Banco Master etc.) saem — não
representavam o imóvel/objeto real e distorciam mais do que ajudavam.
Ficam só as fotos reais e verificadas (TSE, STF, PF, PGR, Abin,
Receita, Santander, CPI, Blaze), com CREDITS.md atualizado.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -3592,26 +3592,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A2)+COUNTIF(Edges!$B$2:$B$120,A2)</f>
         <v/>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>assoc.jpg</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata a sede real</t>
-        </is>
-      </c>
+      <c r="G2" s="24" t="n"/>
+      <c r="H2" s="24" t="n"/>
+      <c r="I2" s="24" t="n"/>
+      <c r="J2" s="24" t="n"/>
     </row>
     <row r="3" ht="23.25" customHeight="1" s="25">
       <c r="A3" s="45" t="inlineStr">
@@ -3798,26 +3782,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A8)+COUNTIF(Edges!$B$2:$B$120,A8)</f>
         <v/>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>sala.jpg</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata a sede real</t>
-        </is>
-      </c>
+      <c r="G8" s="24" t="n"/>
+      <c r="H8" s="24" t="n"/>
+      <c r="I8" s="24" t="n"/>
+      <c r="J8" s="24" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="25">
       <c r="A9" s="45" t="inlineStr">
@@ -3849,26 +3817,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A9)+COUNTIF(Edges!$B$2:$B$120,A9)</f>
         <v/>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>bravo.jpg</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Samuel Zeller · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Assembly_Line_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — linha de produção genérica, não retrata a fábrica real</t>
-        </is>
-      </c>
+      <c r="G9" s="24" t="n"/>
+      <c r="H9" s="24" t="n"/>
+      <c r="I9" s="24" t="n"/>
+      <c r="J9" s="24" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="25">
       <c r="A10" s="45" t="inlineStr">
@@ -3931,26 +3883,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A11)+COUNTIF(Edges!$B$2:$B$120,A11)</f>
         <v/>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>escw.jpg</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata a sede real</t>
-        </is>
-      </c>
+      <c r="G11" s="24" t="n"/>
+      <c r="H11" s="24" t="n"/>
+      <c r="I11" s="24" t="n"/>
+      <c r="J11" s="24" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
       <c r="A12" s="45" t="inlineStr">
@@ -3982,26 +3918,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A12)+COUNTIF(Edges!$B$2:$B$120,A12)</f>
         <v/>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>bets.jpg</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Maximo Betman · CC BY-SA 4.0</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Mesa-de-ruleta-casino-ciudad-de-mexico25-04-2023.jpg</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — mesa de cassino genérica, não retrata a empresa real</t>
-        </is>
-      </c>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>bets.png</t>
+        </is>
+      </c>
+      <c r="H12" s="24" t="inlineStr">
+        <is>
+          <t>blaze.com · domínio público (logo simples, sem direito autoral)</t>
+        </is>
+      </c>
+      <c r="I12" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Blaze_apostas_logo.png</t>
+        </is>
+      </c>
+      <c r="J12" s="24" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="45" t="inlineStr">
@@ -4064,26 +3996,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A14)+COUNTIF(Edges!$B$2:$B$120,A14)</f>
         <v/>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>wt.jpg</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata a sede real</t>
-        </is>
-      </c>
+      <c r="G14" s="24" t="n"/>
+      <c r="H14" s="24" t="n"/>
+      <c r="I14" s="24" t="n"/>
+      <c r="J14" s="24" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="45" t="inlineStr">
@@ -4115,26 +4031,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A15)+COUNTIF(Edges!$B$2:$B$120,A15)</f>
         <v/>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>alcazar.jpg</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata a sede real</t>
-        </is>
-      </c>
+      <c r="G15" s="24" t="n"/>
+      <c r="H15" s="24" t="n"/>
+      <c r="I15" s="24" t="n"/>
+      <c r="J15" s="24" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
       <c r="A16" s="45" t="inlineStr">
@@ -4166,22 +4066,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A16)+COUNTIF(Edges!$B$2:$B$120,A16)</f>
         <v/>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="24" t="inlineStr">
         <is>
           <t>santander.jpg</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="24" t="inlineStr">
         <is>
           <t>Simplus Menegati · CC BY-SA 4.0</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="24" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Agencia_Banco_Santander_de_Telemaco_Borba.jpg</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" s="24" t="inlineStr"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
       <c r="A17" s="45" t="inlineStr">
@@ -4213,22 +4113,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A17)+COUNTIF(Edges!$B$2:$B$120,A17)</f>
         <v/>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="24" t="inlineStr">
         <is>
           <t>cpi.jpg</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="24" t="inlineStr">
         <is>
           <t>Agência Senado · CC BY 2.0</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="24" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:CPIPANDEMIA_-_Comiss%C3%A3o_Parlamentar_de_Inqu%C3%A9rito_da_Pandemia_(1).jpg</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" s="24" t="inlineStr"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="45" t="inlineStr">
@@ -4384,26 +4284,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A22)+COUNTIF(Edges!$B$2:$B$120,A22)</f>
         <v/>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>escf.jpg</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata a sede real</t>
-        </is>
-      </c>
+      <c r="G22" s="24" t="n"/>
+      <c r="H22" s="24" t="n"/>
+      <c r="I22" s="24" t="n"/>
+      <c r="J22" s="24" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
       <c r="A23" s="45" t="inlineStr">
@@ -4435,26 +4319,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A23)+COUNTIF(Edges!$B$2:$B$120,A23)</f>
         <v/>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>ong.jpg</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata a sede real</t>
-        </is>
-      </c>
+      <c r="G23" s="24" t="n"/>
+      <c r="H23" s="24" t="n"/>
+      <c r="I23" s="24" t="n"/>
+      <c r="J23" s="24" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
       <c r="A24" s="45" t="inlineStr">
@@ -4672,26 +4540,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A30)+COUNTIF(Edges!$B$2:$B$120,A30)</f>
         <v/>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>master.jpg</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Anthony Esau · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Farm_Credit_Bank_Building_2016_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — agência bancária genérica, não retrata o Banco Master</t>
-        </is>
-      </c>
+      <c r="G30" s="24" t="n"/>
+      <c r="H30" s="24" t="n"/>
+      <c r="I30" s="24" t="n"/>
+      <c r="J30" s="24" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
       <c r="A31" s="45" t="inlineStr">
@@ -4785,26 +4637,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A33)+COUNTIF(Edges!$B$2:$B$120,A33)</f>
         <v/>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>primeu.jpg</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata a sede real</t>
-        </is>
-      </c>
+      <c r="G33" s="24" t="n"/>
+      <c r="H33" s="24" t="n"/>
+      <c r="I33" s="24" t="n"/>
+      <c r="J33" s="24" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
       <c r="A34" s="45" t="inlineStr">
@@ -4836,26 +4672,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A34)+COUNTIF(Edges!$B$2:$B$120,A34)</f>
         <v/>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>luri.jpg</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Riku Lu · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Office_district_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata a sede real</t>
-        </is>
-      </c>
+      <c r="G34" s="24" t="n"/>
+      <c r="H34" s="24" t="n"/>
+      <c r="I34" s="24" t="n"/>
+      <c r="J34" s="24" t="n"/>
     </row>
     <row r="35" ht="23.25" customHeight="1" s="25">
       <c r="A35" s="45" t="inlineStr">
@@ -4980,26 +4800,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A38)+COUNTIF(Edges!$B$2:$B$120,A38)</f>
         <v/>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>angra.jpg</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Tim Gouw · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Drone_pool_and_deck_chairs_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata o imóvel real</t>
-        </is>
-      </c>
+      <c r="G38" s="24" t="n"/>
+      <c r="H38" s="24" t="n"/>
+      <c r="I38" s="24" t="n"/>
+      <c r="J38" s="24" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
       <c r="A39" s="45" t="inlineStr">
@@ -5031,26 +4835,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A39)+COUNTIF(Edges!$B$2:$B$120,A39)</f>
         <v/>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>aptosp.jpg</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Grant Lemons · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Modern_apartment_building_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata o imóvel real</t>
-        </is>
-      </c>
+      <c r="G39" s="24" t="n"/>
+      <c r="H39" s="24" t="n"/>
+      <c r="I39" s="24" t="n"/>
+      <c r="J39" s="24" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
       <c r="A40" s="45" t="inlineStr">
@@ -5082,26 +4870,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A40)+COUNTIF(Edges!$B$2:$B$120,A40)</f>
         <v/>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>triplex.jpg</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Grant Lemons · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Modern_apartment_building_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata o imóvel real</t>
-        </is>
-      </c>
+      <c r="G40" s="24" t="n"/>
+      <c r="H40" s="24" t="n"/>
+      <c r="I40" s="24" t="n"/>
+      <c r="J40" s="24" t="n"/>
     </row>
     <row r="41" ht="23.25" customHeight="1" s="25">
       <c r="A41" s="45" t="inlineStr">
@@ -5133,26 +4905,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A41)+COUNTIF(Edges!$B$2:$B$120,A41)</f>
         <v/>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>jato.jpg</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Checkerberry · CC BY-SA 4.0</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Flexjet_Embraer_EMB-545_Praetor_500_(N446FX)_Landing_Runway_22_at_KLEX.jpg</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — jato executivo genérico, não retrata a aeronave real</t>
-        </is>
-      </c>
+      <c r="G41" s="24" t="n"/>
+      <c r="H41" s="24" t="n"/>
+      <c r="I41" s="24" t="n"/>
+      <c r="J41" s="24" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
       <c r="A42" s="45" t="inlineStr">
@@ -5184,26 +4940,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A42)+COUNTIF(Edges!$B$2:$B$120,A42)</f>
         <v/>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>atibaia.jpg</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Ritchie Valens · CC0 (Unsplash via Wikimedia Commons)</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Cozy_Cottage_Home_(Unsplash).jpg</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — não retrata o imóvel real</t>
-        </is>
-      </c>
+      <c r="G42" s="24" t="n"/>
+      <c r="H42" s="24" t="n"/>
+      <c r="I42" s="24" t="n"/>
+      <c r="J42" s="24" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
       <c r="A43" s="45" t="inlineStr">
@@ -5390,26 +5130,10 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A48)+COUNTIF(Edges!$B$2:$B$120,A48)</f>
         <v/>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>coaf.jpg</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>frankieleon · CC BY 2.0</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/wiki/File:Scales_of_Justice_(3285348799).jpg</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>Imagem ilustrativa — símbolo da justiça, não retrata o caso real</t>
-        </is>
-      </c>
+      <c r="G48" s="24" t="n"/>
+      <c r="H48" s="24" t="n"/>
+      <c r="I48" s="24" t="n"/>
+      <c r="J48" s="24" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
       <c r="A49" s="45" t="inlineStr">
@@ -5534,22 +5258,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A52)+COUNTIF(Edges!$B$2:$B$120,A52)</f>
         <v/>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G52" s="24" t="inlineStr">
         <is>
           <t>abin.jpg</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H52" s="24" t="inlineStr">
         <is>
           <t>Antonio Cruz/Agência Brasil · CC BY 3.0 BR</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I52" s="24" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Pr%C3%A9dio_da_Abin.jpg</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
+      <c r="J52" s="24" t="inlineStr"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
       <c r="A53" s="45" t="inlineStr">
@@ -5581,22 +5305,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A53)+COUNTIF(Edges!$B$2:$B$120,A53)</f>
         <v/>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="24" t="inlineStr">
         <is>
           <t>receita.jpg</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H53" s="24" t="inlineStr">
         <is>
           <t>Academia de Letras de Campo Maior · CC BY-SA 4.0</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I53" s="24" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Ag%C3%AAncia_da_Receita_Federal_de_Campo_Maior,_Piau%C3%AD,_Brasil.JPG</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
+      <c r="J53" s="24" t="inlineStr"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
       <c r="A54" s="45" t="inlineStr">
@@ -5628,22 +5352,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A54)+COUNTIF(Edges!$B$2:$B$120,A54)</f>
         <v/>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G54" s="24" t="inlineStr">
         <is>
           <t>pf.jpg</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H54" s="24" t="inlineStr">
         <is>
           <t>Agência Senado · CC BY 2.0</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I54" s="24" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Sede_da_Pol%C3%ADcia_Federal_(52830107256).jpg</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
+      <c r="J54" s="24" t="inlineStr"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
       <c r="A55" s="45" t="inlineStr">
@@ -5675,22 +5399,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A55)+COUNTIF(Edges!$B$2:$B$120,A55)</f>
         <v/>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G55" s="24" t="inlineStr">
         <is>
           <t>pgr.jpg</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="H55" s="24" t="inlineStr">
         <is>
           <t>Webysther · CC BY-SA 4.0</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="I55" s="24" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Webysther_20180212174501_-_PGR_-_Procuradoria_Geral_da_Rep%C3%BAblica.jpg</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
+      <c r="J55" s="24" t="inlineStr"/>
     </row>
     <row r="56" ht="23.25" customHeight="1" s="25">
       <c r="A56" s="45" t="inlineStr">
@@ -5753,22 +5477,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A57)+COUNTIF(Edges!$B$2:$B$120,A57)</f>
         <v/>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="24" t="inlineStr">
         <is>
           <t>stf.jpg</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H57" s="24" t="inlineStr">
         <is>
           <t>Daderot · CC0 (domínio público)</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I57" s="24" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Supremo_Tribunal_Federal_building_in_Brasilia_-_DSC00288.JPG</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
+      <c r="J57" s="24" t="inlineStr"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
       <c r="A58" s="45" t="inlineStr">
@@ -5800,22 +5524,22 @@
         <f>COUNTIF(Edges!$A$2:$A$120,A58)+COUNTIF(Edges!$B$2:$B$120,A58)</f>
         <v/>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G58" s="24" t="inlineStr">
         <is>
           <t>tse.jpg</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="H58" s="24" t="inlineStr">
         <is>
           <t>Alexandresena · CC BY-SA 4.0</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="I58" s="24" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Sede_do_Tribunal_Superior_Eleitoral,_em_Bras%C3%ADlia.jpg</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
+      <c r="J58" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F58"/>

</xml_diff>

<commit_message>
Corrige grafia de nomes: Willer Tomaz, Frederick Wassef, Fabiano Zettel, Kássio Nunes Marques, Sérgio Moro
Confirmado com fontes externas (CNN Brasil, Correio da Manhã, Money Times,
documento do Senado) que os nomes no Nodes/Perfis estavam com grafia
divergente da imprensa ou entre as próprias abas da planilha.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -1608,12 +1608,12 @@
       </c>
       <c r="B7" s="38" t="inlineStr">
         <is>
-          <t>Willer Tomaz (planilha: "Tomás")</t>
+          <t>Willer Tomaz</t>
         </is>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="D7" s="37" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="J7" s="37" t="inlineStr">
         <is>
-          <t>Grafia na imprensa é "Tomaz".</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K7" s="37" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="C8" s="37" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="D8" s="37" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="D9" s="37" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="B14" s="38" t="inlineStr">
         <is>
-          <t>Frederick Wassef (planilha: "Frederico")</t>
+          <t>Frederick Wassef</t>
         </is>
       </c>
       <c r="C14" s="37" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J14" s="37" t="inlineStr">
         <is>
-          <t>Grafia correta é "Frederick". Não confirmei a resposta da PGR após julho.</t>
+          <t>Não confirmei a resposta da PGR após julho.</t>
         </is>
       </c>
       <c r="K14" s="37" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="B18" s="38" t="inlineStr">
         <is>
-          <t>Fabiano Campos Zettel (planilha: "Zetel")</t>
+          <t>Fabiano Campos Zettel</t>
         </is>
       </c>
       <c r="C18" s="37" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="J18" s="37" t="inlineStr">
         <is>
-          <t>Grafia na imprensa: "Zettel". Não achei a venda do apartamento à WT nas fontes que abri.</t>
+          <t>Não achei a venda do apartamento à WT nas fontes que abri.</t>
         </is>
       </c>
       <c r="K18" s="37" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="B26" s="38" t="inlineStr">
         <is>
-          <t>Kassio Nunes Marques</t>
+          <t>Kássio Nunes Marques</t>
         </is>
       </c>
       <c r="C26" s="37" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="B30" s="38" t="inlineStr">
         <is>
-          <t>Sergio Fernando Moro</t>
+          <t>Sérgio Fernando Moro</t>
         </is>
       </c>
       <c r="C30" s="37" t="inlineStr">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="B10" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás</t>
+          <t>Willer Tomaz</t>
         </is>
       </c>
       <c r="C10" s="45" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="D10" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="E10" s="45" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="E11" s="45" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="D12" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="E12" s="45" t="inlineStr">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="D13" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="E13" s="45" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="D14" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="E14" s="45" t="inlineStr">
@@ -4019,7 +4019,7 @@
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="E15" s="45" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="D16" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="E16" s="45" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="D17" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="E17" s="45" t="inlineStr">
@@ -4148,7 +4148,7 @@
       </c>
       <c r="D18" s="45" t="inlineStr">
         <is>
-          <t>Willer Tomás e sua rede</t>
+          <t>Willer Tomaz e sua rede</t>
         </is>
       </c>
       <c r="E18" s="45" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="B26" s="45" t="inlineStr">
         <is>
-          <t>Frederico Wassef</t>
+          <t>Frederick Wassef</t>
         </is>
       </c>
       <c r="C26" s="45" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="B31" s="45" t="inlineStr">
         <is>
-          <t>Fabiano Zetel</t>
+          <t>Fabiano Zettel</t>
         </is>
       </c>
       <c r="C31" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Checagem final da importação do acervo
Corrige rótulos conferidos contra as fontes: Zettel foi o 2º doador de Jair;
advogado morto em 2024 representava a WT, não Richarlison; posse no STJ não
confirmada; uma reunião Mendonça–Vorcaro confirmada (14/03/2025); voo de
Marçal pago pela Prime You. Adiciona respostas dos citados e troca link
quebrado da CNN.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011rQv2fzfb4Xj3f3AYjm2Yf
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -971,7 +971,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="25">
       <c r="A4" s="28" t="inlineStr">
         <is>
@@ -1080,23 +1079,6 @@
         <v/>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
     <row r="28" ht="15" customHeight="1" s="25">
       <c r="A28" s="35" t="inlineStr">
         <is>
@@ -1902,7 +1884,7 @@
       </c>
       <c r="K10" s="37" t="inlineStr">
         <is>
-          <t>Wikipedia pt https://pt.wikipedia.org/wiki/Fl%C3%A1vio_Bolsonaro | Tribuna do Sertão (link acima) | O Povo 23/07/2026 https://www.opovo.com.br/noticias/politica/2026/07/23/amp/andre-mendonca-autoriza-inquerito-sobre-repasses-para-dark-horse-filme-sobre-jair-bolsonaro.html | Resultado do 1º turno https://portaldeprefeitura.com.br/bastidores-da-politica/eleicoes-2026-com-100-das-secoes-totalizadas-flavio-tem-4703-e/633498/ | Wikipedia (Banco Master scandal) https://en.wikipedia.org/wiki/Banco_Master_scandal | JB 12/10/2026 https://www.jb.com.br/brasil/justica/2026/10/1061206-moraes-autoriza-flavio-bolsonaro-a-visitar-jair-bolsonaro-em-prisao-domiciliar.html | A investigação sobre o financiamento de Dark Horse (bbc.com) https://www.bbc.com/portuguese/articles/c4g5ky0r25jo | A investigação sobre o financiamento de Dark Horse (em.com.br) https://www.em.com.br/politica/2026/09/7498387-flavio-bolsonaro-vira-investigado-do-dark-horse-que-segue-sob-sigilo.html | O acordo de R$ 134 milhões para o filme (intercept.com.br) https://www.intercept.com.br/2026/05/13/audio-flavio-negociou-vorcaro-milhoes/ | A checagem de declarações sobre Vorcaro (aosfatos.org) https://www.aosfatos.org/noticias/flavio-mentiu-ao-menos-43-vezes-sobre-envolvimento-com-vorcaro/ | Os registros de contato no celular do banqueiro (piaui.uol.com.br) https://piaui.uol.com.br/web/mensagens-celular-flavio-vorcaro/ | As menções a encontros presenciais (estadao.com.br) https://www.estadao.com.br/politica/celular-de-vorcaro-tinha-tres-meses-de-conversa-com-flavio-bolsonaro-e-mencao-a-seis-encontros/ | O voo no jato de Vorcaro em janeiro de 2025 (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-viajou-em-jato-de-vorcaro/ | O apartamento de Fabiano Zettel e Willer Tomaz (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-zettel-tomaz-imovel-vila-nova-conceicao-sao-paulo/ | O aniversário em uma mansão gerida por empresa de Vorcaro (iclnoticias.com.br) https://iclnoticias.com.br/flavio-bolsonaro-aniversario-da-filha-em-mansao/ | E-mails sobre vínculo bancário com Willer Tomaz (noticias.uol.com.br) https://noticias.uol.com.br/colunas/fabio-serapiao/2026/10/10/flavio-dividia-conta-com-suspeito-de-lavar-dinheiro-do-inss-indicam-emails.htm | Endereço e contabilidade compartilhados em Brasília (iclnoticias.com.br) https://iclnoticias.com.br/empresas-de-flavio-bolsonaro-e-careca-do-inss/ | Cargo na Câmara, faculdade e estágio no Rio (bbc.com) https://www.bbc.com/portuguese/brasil-46828487 | A acusação de rachadinhas na Alerj (valor.globo.com) https://valor.globo.com/politica/eleicoes-2026/noticia/2026/09/01/flavio-bolsonaro-relembre-o-processo-da-rachadinha.ghtml | A acusação de rachadinhas na Alerj (folhadelondrina.com.br) https://www.folhadelondrina.com.br/ultimas-noticias/entenda-quais-provas-da-rachadinha-contra-flavio-bolsonaro-ainda-valem-3131387e.html | A investigação da loja Kopenhagen (oglobo.globo.com) https://oglobo.globo.com/politica/alvo-de-investigacao-das-rachadinhas-loja-de-flavio-bolsonaro-no-rio-vendida-1-24867874 | Imóveis comprados pela família e investigações (g1.globo.com) https://g1.globo.com/jornal-nacional/noticia/2022/08/31/reportagem-do-uol-revela-que-51-imoveis-comprados-pela-familia-bolsonaro-foram-pagos-em-dinheiro-vivo.ghtml | Imóveis comprados pela família e investigações (noticias.uol.com.br) https://noticias.uol.com.br/politica/ultimas-noticias/2022/08/30/imoveis-cla-bolsonaro-objeto-de-investigacao-suspeita-dinheiro-vivo.htm | Imóveis comprados pela família e investigações (estadao.com.br) https://www.estadao.com.br/politica/investigacao-sobre-flaviobolsonaro-alcanca-37-imoveis/ | A compra e a quitação da mansão em Brasília (oglobo.globo.com) https://oglobo.globo.com/politica/eleicoes-2026/noticia/2026/08/14/video-mansao-que-fez-patrimonio-de-flavio-disparar-fica-em-terreno-de-2400-m-e-foi-quitada-27-anos-antes-do-previsto.ghtml | A análise do MPF sobre 37 transações imobiliárias (cnnbrasil.com.br) https://www.cnnbrasil.com.br/politica/o-mpf-ve-fortes-indicios-de-lavagem-de-dinheiro-em-bens-de-flavio-bolsonaro/a | A acusação do MP-RJ sobre organização criminosa (g1.globo.com) https://g1.globo.com/rj/rio-de-janeiro/noticia/2019/12/19/mp-do-rj-detalha-suposto-esquema-de-corrupcao-envolvendo-entao-deputado-flavio-bolsonaro.ghtml?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=g1 | Destinação de emendas e entidades questionadas (revistaforum.com.br) https://revistaforum.com.br/politica/flavio-bolsonaro-emendas-ong-fantasma-e-instituto-de-miliciano/</t>
+          <t>Wikipedia pt https://pt.wikipedia.org/wiki/Fl%C3%A1vio_Bolsonaro | Tribuna do Sertão (link acima) | O Povo 23/07/2026 https://www.opovo.com.br/noticias/politica/2026/07/23/amp/andre-mendonca-autoriza-inquerito-sobre-repasses-para-dark-horse-filme-sobre-jair-bolsonaro.html | Resultado do 1º turno https://portaldeprefeitura.com.br/bastidores-da-politica/eleicoes-2026-com-100-das-secoes-totalizadas-flavio-tem-4703-e/633498/ | Wikipedia (Banco Master scandal) https://en.wikipedia.org/wiki/Banco_Master_scandal | JB 12/10/2026 https://www.jb.com.br/brasil/justica/2026/10/1061206-moraes-autoriza-flavio-bolsonaro-a-visitar-jair-bolsonaro-em-prisao-domiciliar.html | A investigação sobre o financiamento de Dark Horse (bbc.com) https://www.bbc.com/portuguese/articles/c4g5ky0r25jo | A investigação sobre o financiamento de Dark Horse (em.com.br) https://www.em.com.br/politica/2026/09/7498387-flavio-bolsonaro-vira-investigado-do-dark-horse-que-segue-sob-sigilo.html | O acordo de R$ 134 milhões para o filme (intercept.com.br) https://www.intercept.com.br/2026/05/13/audio-flavio-negociou-vorcaro-milhoes/ | A checagem de declarações sobre Vorcaro (aosfatos.org) https://www.aosfatos.org/noticias/flavio-mentiu-ao-menos-43-vezes-sobre-envolvimento-com-vorcaro/ | Os registros de contato no celular do banqueiro (piaui.uol.com.br) https://piaui.uol.com.br/web/mensagens-celular-flavio-vorcaro/ | As menções a encontros presenciais (estadao.com.br) https://www.estadao.com.br/politica/celular-de-vorcaro-tinha-tres-meses-de-conversa-com-flavio-bolsonaro-e-mencao-a-seis-encontros/ | O voo no jato de Vorcaro em janeiro de 2025 (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-viajou-em-jato-de-vorcaro/ | O apartamento de Fabiano Zettel e Willer Tomaz (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-zettel-tomaz-imovel-vila-nova-conceicao-sao-paulo/ | O aniversário em uma mansão gerida por empresa de Vorcaro (iclnoticias.com.br) https://iclnoticias.com.br/flavio-bolsonaro-aniversario-da-filha-em-mansao/ | E-mails sobre vínculo bancário com Willer Tomaz (noticias.uol.com.br) https://noticias.uol.com.br/colunas/fabio-serapiao/2026/10/10/flavio-dividia-conta-com-suspeito-de-lavar-dinheiro-do-inss-indicam-emails.htm | Endereço e contabilidade compartilhados em Brasília (iclnoticias.com.br) https://iclnoticias.com.br/empresas-de-flavio-bolsonaro-e-careca-do-inss/ | Cargo na Câmara, faculdade e estágio no Rio (bbc.com) https://www.bbc.com/portuguese/brasil-46828487 | A acusação de rachadinhas na Alerj (valor.globo.com) https://valor.globo.com/politica/eleicoes-2026/noticia/2026/09/01/flavio-bolsonaro-relembre-o-processo-da-rachadinha.ghtml | A acusação de rachadinhas na Alerj (folhadelondrina.com.br) https://www.folhadelondrina.com.br/ultimas-noticias/entenda-quais-provas-da-rachadinha-contra-flavio-bolsonaro-ainda-valem-3131387e.html | A investigação da loja Kopenhagen (oglobo.globo.com) https://oglobo.globo.com/politica/alvo-de-investigacao-das-rachadinhas-loja-de-flavio-bolsonaro-no-rio-vendida-1-24867874 | Imóveis comprados pela família e investigações (g1.globo.com) https://g1.globo.com/jornal-nacional/noticia/2022/08/31/reportagem-do-uol-revela-que-51-imoveis-comprados-pela-familia-bolsonaro-foram-pagos-em-dinheiro-vivo.ghtml | Imóveis comprados pela família e investigações (noticias.uol.com.br) https://noticias.uol.com.br/politica/ultimas-noticias/2022/08/30/imoveis-cla-bolsonaro-objeto-de-investigacao-suspeita-dinheiro-vivo.htm | Imóveis comprados pela família e investigações (estadao.com.br) https://www.estadao.com.br/politica/investigacao-sobre-flaviobolsonaro-alcanca-37-imoveis/ | A compra e a quitação da mansão em Brasília (oglobo.globo.com) https://oglobo.globo.com/politica/eleicoes-2026/noticia/2026/08/14/video-mansao-que-fez-patrimonio-de-flavio-disparar-fica-em-terreno-de-2400-m-e-foi-quitada-27-anos-antes-do-previsto.ghtml | A análise do MPF sobre 37 transações imobiliárias (cnnbrasil.com.br) https://www.maisgoias.com.br/politica/procurador-aponta-fortes-indicios-de-lavagem-de-dinheiro-em-bens-de-flavio-bolsonaro/ | A acusação do MP-RJ sobre organização criminosa (g1.globo.com) https://g1.globo.com/rj/rio-de-janeiro/noticia/2019/12/19/mp-do-rj-detalha-suposto-esquema-de-corrupcao-envolvendo-entao-deputado-flavio-bolsonaro.ghtml?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=g1 | Destinação de emendas e entidades questionadas (revistaforum.com.br) https://revistaforum.com.br/politica/flavio-bolsonaro-emendas-ong-fantasma-e-instituto-de-miliciano/</t>
         </is>
       </c>
       <c r="L10" s="37" t="inlineStr">
@@ -2925,7 +2907,7 @@
       </c>
       <c r="J24" s="37" t="inlineStr">
         <is>
-          <t>Em jun/2026 uma advogada publicou e retirou um vídeo sobre o caso, retratando-se por imprecisões. Acervo a verdade.: o advogado dele na disputa pela casa foi morto em 2024 no Rio. Nada nas fontes liga Flávio ou Willer ao homicídio. O PDF diz que a mansão é gerida por empresa de Vorcaro; o mapa a registra como da WT.</t>
+          <t>Em jun/2026 uma advogada publicou e retirou um vídeo sobre o caso, retratando-se por imprecisões. Acervo a verdade.: o PDF diz que o advogado morto em fev/2024 no Rio era de Richarlison, mas a ICL informa que Rodrigo Crespo representava a WT, do lado de Willer (que nega que ele tenha atuado). Nada nas fontes liga Flávio ou Willer ao homicídio. O PDF diz que a mansão é gerida por empresa de Vorcaro; o mapa a registra como da WT.</t>
         </is>
       </c>
       <c r="K24" s="37" t="inlineStr">
@@ -3761,7 +3743,7 @@
       </c>
       <c r="J35" s="37" t="inlineStr">
         <is>
-          <t>O PDF original diz que ele “é investigado”; isso está desatualizado desde o arquivamento (Folha e UOL, 06/10/2026).</t>
+          <t>A PGR também pediu o arquivamento; ele diz que a acusação é falsa e move ações contra quem a levou adiante. O PDF original diz que ele “é investigado”; isso está desatualizado desde o arquivamento (Folha e UOL, 06/10/2026).</t>
         </is>
       </c>
       <c r="K35" s="37" t="inlineStr">
@@ -5967,7 +5949,7 @@
       </c>
       <c r="E62" s="45" t="inlineStr">
         <is>
-          <t>Deputado; presente na reunião Mendonça–Vorcaro (fev/2025); alvo de operação autorizada por Dino</t>
+          <t>Deputado federal; ajudou a articular a reunião Mendonça–Vorcaro de mar/2025; alvo de operação autorizada por Dino</t>
         </is>
       </c>
       <c r="F62" s="45">
@@ -6282,7 +6264,7 @@
       </c>
       <c r="E71" s="45" t="inlineStr">
         <is>
-          <t>Voo internacional de R$ 1 mi pago por empresa da qual Vorcaro era sócio</t>
+          <t>Ex-coach; voo de R$ 1,17 mi pago pela Prime You, de que Vorcaro era sócio; confirmou o uso</t>
         </is>
       </c>
       <c r="F71" s="45">
@@ -6387,7 +6369,7 @@
       </c>
       <c r="E74" s="45" t="inlineStr">
         <is>
-          <t>Avaliada em R$ 6 mi; terreno de 2.400 m²; quitada 27 anos antes do previsto</t>
+          <t>R$ 6 mi, 2.400 m², Setor de Mansões Dom Bosco; R$ 3,1 mi financiados pelo BRB</t>
         </is>
       </c>
       <c r="F74" s="45">
@@ -6597,7 +6579,7 @@
       </c>
       <c r="E80" s="45" t="inlineStr">
         <is>
-          <t>Condenado no caso Marielle; negociou emenda com assessora de Flávio</t>
+          <t>Robson Calixto, PM da reserva condenado no caso Marielle; PF diz que intermediou emenda de Flávio</t>
         </is>
       </c>
       <c r="F80" s="45">
@@ -6632,7 +6614,7 @@
       </c>
       <c r="E81" s="45" t="inlineStr">
         <is>
-          <t>Recebeu emenda de Flávio; PF apura desvios</t>
+          <t>Instituto Ifop (Taquara, RJ); PF suspeita de ligação com os Brazão; a ONG nega</t>
         </is>
       </c>
       <c r="F81" s="45">
@@ -6702,7 +6684,7 @@
       </c>
       <c r="E83" s="45" t="inlineStr">
         <is>
-          <t>Pastor de Flávio; defendeu em livro retirar o título de padroeira de N. Sra. Aparecida</t>
+          <t>Bispo da Comunidade das Nações; defendeu em livro retirar o título de padroeira de N. Sra. Aparecida</t>
         </is>
       </c>
       <c r="F83" s="45">
@@ -10477,7 +10459,7 @@
       </c>
       <c r="C124" s="45" t="inlineStr">
         <is>
-          <t>Empréstimo para a mansão com juros abaixo do mercado; PF investiga</t>
+          <t>Empréstimo de R$ 3,1 mi a 3,71% a.a., abaixo da média do banco; PF investiga. Ele diz que a Justiça já atestou a regularidade e que o empréstimo está quitado</t>
         </is>
       </c>
       <c r="D124" s="45" t="inlineStr">
@@ -10537,7 +10519,7 @@
       </c>
       <c r="C126" s="45" t="inlineStr">
         <is>
-          <t>Comprou; ele diz pagar com renda de advogado</t>
+          <t>Comprou em 2021 por R$ 6 mi</t>
         </is>
       </c>
       <c r="D126" s="45" t="inlineStr">
@@ -10567,7 +10549,7 @@
       </c>
       <c r="C127" s="45" t="inlineStr">
         <is>
-          <t>Maior doador da campanha de 2022 (R$ 3 mi)</t>
+          <t>Doou R$ 3 mi à campanha de 2022, 2º maior doador depois do PL (CNN/TSE)</t>
         </is>
       </c>
       <c r="D127" s="45" t="inlineStr">
@@ -10597,7 +10579,7 @@
       </c>
       <c r="C128" s="45" t="inlineStr">
         <is>
-          <t>Doou R$ 2 mi à campanha de 2022</t>
+          <t>Doou R$ 2 mi à campanha de 2022, a maior doação de pessoa física (CNN/TSE)</t>
         </is>
       </c>
       <c r="D128" s="45" t="inlineStr">
@@ -10807,7 +10789,7 @@
       </c>
       <c r="C135" s="45" t="inlineStr">
         <is>
-          <t>Reuniões em 19/02 e 14/03/2025 fora da agenda oficial</t>
+          <t>Reunião reservada de 2 h em 14/03/2025, fora da agenda, no ITER (mensagens); não há prova de que tenha agido pelo Master</t>
         </is>
       </c>
       <c r="D135" s="45" t="inlineStr">
@@ -10897,7 +10879,7 @@
       </c>
       <c r="C138" s="45" t="inlineStr">
         <is>
-          <t>Na reunião de fev/2025; teria aproximado ministro e banqueiro</t>
+          <t>Ajudou a articular a reunião com Vorcaro de mar/2025 (mensagens)</t>
         </is>
       </c>
       <c r="D138" s="45" t="inlineStr">
@@ -11047,7 +11029,7 @@
       </c>
       <c r="C143" s="45" t="inlineStr">
         <is>
-          <t>Afastou o diretor-geral sem ouvir a PGR (set/2026); AGU vê usurpação de competência</t>
+          <t>Afastou o diretor-geral sem ouvir a PGR (08/09/2026), alegando monitoramento ilegal; AGU vê usurpação de competência</t>
         </is>
       </c>
       <c r="D143" s="45" t="inlineStr">
@@ -11347,7 +11329,7 @@
       </c>
       <c r="C153" s="45" t="inlineStr">
         <is>
-          <t>PF: mesada de R$ 300 mil a 500 mil e viagens pagas, incluindo Courchevel</t>
+          <t>PF: pagamentos mensais de R$ 300 mil a 500 mil e viagens pagas, incluindo Courchevel (~R$ 2 mi); ele nega ilicitude</t>
         </is>
       </c>
       <c r="D153" s="45" t="inlineStr">
@@ -11467,7 +11449,7 @@
       </c>
       <c r="C157" s="45" t="inlineStr">
         <is>
-          <t>PF: articulador dele em Brasília; empresa ligada ao banqueiro pagou R$ 67,5 mi por projeto de Faria</t>
+          <t>PF: articulador dele em Brasília; Vorcaro pagou R$ 67,5 mi por projeto eólico de Faria, que defende o valor</t>
         </is>
       </c>
       <c r="D157" s="45" t="inlineStr">
@@ -11637,7 +11619,7 @@
     <row r="163">
       <c r="A163" s="45" t="inlineStr">
         <is>
-          <t>vorcaro</t>
+          <t>primeu</t>
         </is>
       </c>
       <c r="B163" s="45" t="inlineStr">
@@ -11647,12 +11629,12 @@
       </c>
       <c r="C163" s="45" t="inlineStr">
         <is>
-          <t>Empresa da qual Vorcaro era sócio pagou voo de R$ 1 mi</t>
+          <t>Pagou voo SP–EUA de R$ 1,17 mi (2025); Marçal confirmou o uso (Valor)</t>
         </is>
       </c>
       <c r="D163" s="45" t="inlineStr">
         <is>
-          <t>Alegado ou contestado</t>
+          <t>Documentado</t>
         </is>
       </c>
       <c r="E163" s="45">
@@ -11737,7 +11719,7 @@
       </c>
       <c r="C166" s="45" t="inlineStr">
         <is>
-          <t>Flávio foi batizado na igreja dele (Folha)</t>
+          <t>Flávio foi batizado na Comunidade das Nações, igreja dele, em jan/2024 (Folha)</t>
         </is>
       </c>
       <c r="D166" s="45" t="inlineStr">
@@ -11797,7 +11779,7 @@
       </c>
       <c r="C168" s="45" t="inlineStr">
         <is>
-          <t>Ex-sócio na Kopenhagen cita lobby dele com Nunes (Brasil de Fato)</t>
+          <t>Ex-sócio cita lobby dele com Nunes em favor de cliente; sem comprovação independente (PlatôBR)</t>
         </is>
       </c>
       <c r="D168" s="45" t="inlineStr">
@@ -12067,7 +12049,7 @@
       </c>
       <c r="C177" s="45" t="inlineStr">
         <is>
-          <t>Emenda para a ONG; PF apura</t>
+          <t>Emenda de R$ 199 mil (nov/2023); PF apura. Ele diz que não cabe ao parlamentar auditar o uso</t>
         </is>
       </c>
       <c r="D177" s="45" t="inlineStr">
@@ -12097,7 +12079,7 @@
       </c>
       <c r="C178" s="45" t="inlineStr">
         <is>
-          <t>Negociou emenda com assessora dele (Estadão)</t>
+          <t>PF: intermediou a emenda com o gabinete dele (O Globo, Estadão)</t>
         </is>
       </c>
       <c r="D178" s="45" t="inlineStr">
@@ -12157,7 +12139,7 @@
       </c>
       <c r="C180" s="45" t="inlineStr">
         <is>
-          <t>Atuou como advogado dele; recurso no STJ reverteu decisão</t>
+          <t>Advogado dele no STJ (2024); recurso reverteu a ida a júri popular (coluna no iG)</t>
         </is>
       </c>
       <c r="D180" s="45" t="inlineStr">
@@ -12187,7 +12169,7 @@
       </c>
       <c r="C181" s="45" t="inlineStr">
         <is>
-          <t>Obteve a posse na Justiça; STJ reconheceu em 2025</t>
+          <t>Obteve a posse na Justiça na disputa com Richarlison</t>
         </is>
       </c>
       <c r="D181" s="45" t="inlineStr">
@@ -12248,7 +12230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="110" customWidth="1" style="24" min="1" max="1"/>
@@ -12325,30 +12307,37 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>21/10/2026: importados 26 nós, 62 conexões e 4 perfis do acervo a verdade. (https://bolsomaster.site, PDF em https://bolsomaster.site/documento-original.pdf). As fontes de cada item são as do acervo e não foram reverificadas uma a uma.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>Na importação, foi marcado como “Documentado” só o que é ato público ou fato noticiado sem disputa (indicação, doação registrada, homenagem, decisão judicial, contrato público). Suspeitas, mensagens, relatórios da PF sobre condutas e afirmações de ex-sócios ficaram como “Alegado ou contestado”.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Correções do próprio acervo aplicadas: honorários de até R$ 427 mi não são recebimento pessoal de Nunes; o caso do vice Alfredo Gaspar foi arquivado; números do celular de Vorcaro (Piauí × Estadão) não se somam; contratos do ITER são dois levantamentos diferentes.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>Registros do acervo deixados de fora: registro-3 (comparação retórica do PDF; o próprio acervo diz que não comprova a origem do dinheiro); registro-5 (afirmação de exclusividade não verificada pelo acervo); registro-7 (comparação de valores entre casos diferentes); registro-8 (comparação de valores entre casos diferentes); registro-22 (hipótese do PDF sobre o esquema, com fonte em vídeo); registro-27 (já no mapa (Nunes preside o TSE)); registro-41 (pessoa não identificada com clareza); registro-87 (sem pessoa ou conexão específica); registro-88 (só título de reportagem); registro-91 (projeto de lei sem ligação direta com o mapa); registro-93 (post de Nikolas Ferreira sem ligação com o mapa); registro-126 (padrinho não identificado no texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Checagem final (21/10/2026): 111 links testados (91 abrem; 19 bloqueiam robôs, como UOL, Intercept e Folha; 1 link da CNN quebrado foi trocado por Mais Goiás). Conferidas contra a fonte 22 matérias das conexões mais sensíveis. Corrigidos: Zettel foi o 2º doador de Jair, não o maior; o advogado morto em 2024 representava a WT, não Richarlison; a posse de Willer reconhecida pelo STJ não foi confirmada; Mendonça teve uma reunião reservada confirmada (14/03/2025), não duas; o voo de Marçal foi pago pela Prime You (R$ 1,17 mi). Respostas dos citados foram adicionadas (Flávio sobre o BRB e a emenda, Ciro, Faria, Marçal, Gaspar).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rodada UOL News: Best Bet/Cathedral, Rio Pag, hangar, Weverton Rocha
+7 nós, +16 conexões, perfil novo de Weverton Rocha e atualização dos perfis
de Willer e Flávio. Só entraram itens com reportagem escrita (piauí, Folha,
O Globo, Estadão, Poder360); festa no hangar, rancho e origem em Taguatinga
ficaram de fora. Divergência sobre a data de saída de Willer do país
registrada nas ressalvas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011rQv2fzfb4Xj3f3AYjm2Yf
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfis'!$A$1:$P$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfis'!$A$1:$P$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Nodes'!$A$1:$F$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Edges'!$A$1:$F$120</definedName>
   </definedNames>
@@ -971,6 +971,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="25">
       <c r="A4" s="28" t="inlineStr">
         <is>
@@ -995,7 +996,7 @@
         </is>
       </c>
       <c r="B5" s="24">
-        <f>COUNTIF(Perfis!$H$2:$H$35,A5)</f>
+        <f>COUNTIF(Perfis!$H$2:$H$36,A5)</f>
         <v/>
       </c>
       <c r="C5" s="30" t="inlineStr">
@@ -1011,7 +1012,7 @@
         </is>
       </c>
       <c r="B6" s="24">
-        <f>COUNTIF(Perfis!$H$2:$H$35,A6)</f>
+        <f>COUNTIF(Perfis!$H$2:$H$36,A6)</f>
         <v/>
       </c>
       <c r="C6" s="30" t="inlineStr">
@@ -1027,12 +1028,12 @@
         </is>
       </c>
       <c r="B7" s="24">
-        <f>COUNTIF(Perfis!$H$2:$H$35,A7)</f>
+        <f>COUNTIF(Perfis!$H$2:$H$36,A7)</f>
         <v/>
       </c>
       <c r="C7" s="30" t="inlineStr">
         <is>
-          <t>Fábio Luís Lula da Silva; Roberta Moreira Luchsinger; Willer Tomaz; Flávio Bolsonaro; Carlos Bolsonaro; Frederick Wassef; Ciro Nogueira; Mario Frias</t>
+          <t>Fábio Luís Lula da Silva; Roberta Moreira Luchsinger; Willer Tomaz; Flávio Bolsonaro; Carlos Bolsonaro; Frederick Wassef; Ciro Nogueira; Mario Frias; Weverton Rocha</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1044,7 @@
         </is>
       </c>
       <c r="B8" s="24">
-        <f>COUNTIF(Perfis!$H$2:$H$35,A8)</f>
+        <f>COUNTIF(Perfis!$H$2:$H$36,A8)</f>
         <v/>
       </c>
       <c r="C8" s="30" t="inlineStr">
@@ -1059,7 +1060,7 @@
         </is>
       </c>
       <c r="B9" s="24">
-        <f>COUNTIF(Perfis!$H$2:$H$35,A9)</f>
+        <f>COUNTIF(Perfis!$H$2:$H$36,A9)</f>
         <v/>
       </c>
       <c r="C9" s="30" t="inlineStr">
@@ -1079,6 +1080,23 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
     <row r="28" ht="15" customHeight="1" s="25">
       <c r="A28" s="35" t="inlineStr">
         <is>
@@ -1150,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -1618,7 +1636,7 @@
       </c>
       <c r="D7" s="37" t="inlineStr">
         <is>
-          <t>Advogado em Brasília. Preso em 2017 sob suspeita de tentar interferir na Operação Greenfield (fundos de pensão). Alvo de busca em ago/2026 na Operação Sem Desconto (caso ligado ao senador Weverton Rocha). O inquérito sobre ele e Flávio (suposta lavagem via bets, Rede Loto) chegou ao STF em 08/10/2026 (relator Moraes) e foi revelado em 18–19/10. A PF diz que uma conta dele movimentou ~R$ 130 mi entre mar e mai/2025. Dono de empresas como WT, Alcazar e Cathedral.</t>
+          <t>Advogado em Brasília. Preso em 2017 sob suspeita de tentar interferir na Operação Greenfield (fundos de pensão). Alvo de busca em ago/2026 na Operação Sem Desconto (caso ligado ao senador Weverton Rocha). O inquérito sobre ele e Flávio (suposta lavagem via bets, Rede Loto) chegou ao STF em 08/10/2026 (relator Moraes) e foi revelado em 18–19/10. A PF diz que uma conta dele movimentou ~R$ 130 mi entre mar e mai/2025. Dono de empresas como WT, Alcazar e Cathedral. Segundo a piauí (20/10/2026), criou em jan/2023 a offshore Cathedral, única acionista da Rede Loto (Best Bet), licenciada pela Loterj. Um e-mail achado pela PF mostra que ele se apresentou como sócio da Rio Pag, que processava pagamentos da Loterj; depois admitiu participação indireta. A PF achou sala oculta, sem dinheiro, em hangares de empresas dele no Aeroporto de Brasília. Na Operação Sem Desconto, a PF o descreve como “hub financeiro” do senador Weverton Rocha. Confirmou ao Metrópoles que viajou ao exterior com a família.</t>
         </is>
       </c>
       <c r="E7" s="37" t="inlineStr">
@@ -1633,7 +1651,7 @@
       </c>
       <c r="G7" s="37" t="inlineStr">
         <is>
-          <t>Investigado; nega irregularidades e fala em "pescaria probatória". Nas fontes não há denúncia nem condenação.</t>
+          <t>Investigado; nega irregularidades e fala em "pescaria probatória". Nas fontes não há denúncia nem condenação. Diz que não há sócios ocultos nem contas não declaradas, que a sala do hangar serve a empresas de transporte de valores e que não tem restrição judicial para viajar.</t>
         </is>
       </c>
       <c r="H7" s="41" t="inlineStr">
@@ -1648,22 +1666,22 @@
       </c>
       <c r="J7" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Data da saída do país não confirmada: o UOL News citou registros da PF de 21/08/2026 (chegada aos EUA em 22/08), mas a Fórum/Metrópoles (19/10) fala em viagem na semana anterior. A defesa diz que a Rede Loto nunca chegou a operar.</t>
         </is>
       </c>
       <c r="K7" s="37" t="inlineStr">
         <is>
-          <t>A Tarde https://atarde.com.br/eleicoes/quem-e-willer-tomaz-advogado-suspeito-de-ligacao-com-flavio-bolsonaro-1406358 | Tribuna do Sertão 19/10/2026 https://www.tribunadosertao.com.br/poder-e-governo/2026/10/19/1000284-flavio-bolsonaro-e-investigado-pela-pf-por-suspeita-de-lavagem-de-dinheiro-com-advogado-willer-tomaz | CartaCapital 18/10/2026 https://www.cartacapital.com.br/politica/flavio-bolsonaro-e-alvo-de-segundo-inquerito-no-stf-por-suspeita-de-lavagem-de-dinheiro/ | CNN Brasil https://www.cnnbrasil.com.br/politica/advogado-amigo-de-flavio-movimentou-r-130-milhoes-em-tres-meses-diz-pf/ | O voo no jato de Vorcaro em janeiro de 2025 (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-viajou-em-jato-de-vorcaro/ | E-mails sobre vínculo bancário com Willer Tomaz (noticias.uol.com.br) https://noticias.uol.com.br/colunas/fabio-serapiao/2026/10/10/flavio-dividia-conta-com-suspeito-de-lavar-dinheiro-do-inss-indicam-emails.htm | A disputa pelo imóvel comprado por Richarlison (iclnoticias.com.br) https://iclnoticias.com.br/advogado-defendia-amigo-de-flavio-bolsonaro/ | A disputa pelo imóvel comprado por Richarlison (iclnoticias.com.br) https://iclnoticias.com.br/pf-e-acionada-flavio-bolsonaro-richarlisson/</t>
+          <t>A Tarde https://atarde.com.br/eleicoes/quem-e-willer-tomaz-advogado-suspeito-de-ligacao-com-flavio-bolsonaro-1406358 | Tribuna do Sertão 19/10/2026 https://www.tribunadosertao.com.br/poder-e-governo/2026/10/19/1000284-flavio-bolsonaro-e-investigado-pela-pf-por-suspeita-de-lavagem-de-dinheiro-com-advogado-willer-tomaz | CartaCapital 18/10/2026 https://www.cartacapital.com.br/politica/flavio-bolsonaro-e-alvo-de-segundo-inquerito-no-stf-por-suspeita-de-lavagem-de-dinheiro/ | CNN Brasil https://www.cnnbrasil.com.br/politica/advogado-amigo-de-flavio-movimentou-r-130-milhoes-em-tres-meses-diz-pf/ | O voo no jato de Vorcaro em janeiro de 2025 (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-viajou-em-jato-de-vorcaro/ | E-mails sobre vínculo bancário com Willer Tomaz (noticias.uol.com.br) https://noticias.uol.com.br/colunas/fabio-serapiao/2026/10/10/flavio-dividia-conta-com-suspeito-de-lavar-dinheiro-do-inss-indicam-emails.htm | A disputa pelo imóvel comprado por Richarlison (iclnoticias.com.br) https://iclnoticias.com.br/advogado-defendia-amigo-de-flavio-bolsonaro/ | A disputa pelo imóvel comprado por Richarlison (iclnoticias.com.br) https://iclnoticias.com.br/pf-e-acionada-flavio-bolsonaro-richarlisson/ | Portal Porque (resume piauí, 20/10/2026) https://www.portalporque.com.br/brasil/revista-piaui-aponta-que-flavio-bolsonaro-foi-socio-indireto-de-bet/ | Correio da Manhã (via O Globo, Malu Gaspar) https://www.correiodamanha.com.br/politica/2026/10/328716-aliado-de-flavio-bolsonaro-admitiu-ser-socio-de-empresa-da-loterj-apos-negar-ligacao-revela-e-mail.html | Goiás 246 (via Estadão) https://www.goias246.com.br/noticia/34906/politica/pf-aponta-sala-estruturada-para-guardar-valores-em-hangar-de-empresas-do-advogado-willer-tomaz.html | Poder360 04/08/2026 https://www.poder360.com.br/poder-justica/pf-investiga-advogado-amigo-de-flavio-em-operacao-sobre-o-inss/ | Revista Fórum (via Metrópoles, 19/10/2026) https://revistaforum.com.br/politica/willer-tomaz-flavio-bolsonaro-viaja-preocupa-pf/</t>
         </is>
       </c>
       <c r="L7" s="37" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="M7" s="37" t="inlineStr">
         <is>
-          <t>Data de entrada no STF (08/10/2026), valores e confirmação da busca de ago/2026. 21/10/2026: importado do acervo a verdade. (bolsomaster.site).</t>
+          <t>Data de entrada no STF (08/10/2026), valores e confirmação da busca de ago/2026. 21/10/2026: importado do acervo a verdade. (bolsomaster.site). 22/10/2026: rodada UOL News (bets, Loterj, hangar, Weverton).</t>
         </is>
       </c>
       <c r="N7" s="24" t="inlineStr">
@@ -1849,7 +1867,7 @@
       </c>
       <c r="D10" s="37" t="inlineStr">
         <is>
-          <t>Nascido em 30/04/1981, Resende (RJ). Advogado e empresário; deputado estadual desde 2003, senador pelo RJ desde 2019. Candidato do PL à Presidência: no 1º turno (04/10/2026) teve 47,03% dos votos válidos contra 45,16% de Lula; o 2º turno é em 25/10/2026. Rachadinha: denunciado pelo MPRJ em out/2020 com Queiroz e outros 15; provas anuladas pelo STJ/STF em nov/2021; denúncia rejeitada e caso arquivado em 2022. Hoje há dois inquéritos no STF: (1) Dark Horse, autorizado por Mendonça em 23/07/2026 (~US$ 24 mi negociados; Coaf/piauí apontam ~US$ 12,3 mi repassados por Vorcaro ao fundo Havengate); em 10/09 a PF fez a Operação Make Up (49 mandados; alvos incluem a produtora Karina Gama e o deputado Mário Frias). (2) lavagem com Willer Tomaz, chegou ao STF em 08/10/2026 (relator Moraes). Em 12/10 Moraes liberou as visitas dele ao pai, suspensas desde julho por ele ter publicado uma carta de Jair.</t>
+          <t>Nascido em 30/04/1981, Resende (RJ). Advogado e empresário; deputado estadual desde 2003, senador pelo RJ desde 2019. Candidato do PL à Presidência: no 1º turno (04/10/2026) teve 47,03% dos votos válidos contra 45,16% de Lula; o 2º turno é em 25/10/2026. Rachadinha: denunciado pelo MPRJ em out/2020 com Queiroz e outros 15; provas anuladas pelo STJ/STF em nov/2021; denúncia rejeitada e caso arquivado em 2022. Hoje há dois inquéritos no STF: (1) Dark Horse, autorizado por Mendonça em 23/07/2026 (~US$ 24 mi negociados; Coaf/piauí apontam ~US$ 12,3 mi repassados por Vorcaro ao fundo Havengate); em 10/09 a PF fez a Operação Make Up (49 mandados; alvos incluem a produtora Karina Gama e o deputado Mário Frias). (2) lavagem com Willer Tomaz, chegou ao STF em 08/10/2026 (relator Moraes). Em 12/10 Moraes liberou as visitas dele ao pai, suspensas desde julho por ele ter publicado uma carta de Jair. Out/2026: a piauí aponta, com documentos da PF, que ele pode ter sido sócio oculto da Best Bet, de Willer, por ter sido “usuário master” da conta da offshore Alcazar (excluído por e-mail de 22/05/2025). A Folha revelou voos dele na Europa em 2025 com canhotos em nome da Cathedral, dona da bet.</t>
         </is>
       </c>
       <c r="E10" s="37" t="inlineStr">
@@ -1864,7 +1882,7 @@
       </c>
       <c r="G10" s="37" t="inlineStr">
         <is>
-          <t>Nega: chama o 2º inquérito de politicamente motivado e a relação com Willer de amizade entre famílias; diz que o filme foi patrocínio. Sem denúncia nova nem condenação.</t>
+          <t>Nega: chama o 2º inquérito de politicamente motivado e a relação com Willer de amizade entre famílias; diz que o filme foi patrocínio. Sem denúncia nova nem condenação. Sobre a bet e os voos: diz que nunca teve acesso a contas de empresas de Willer e que a relação é “exclusivamente de amizade”; chama a associação de “mera ilação”.</t>
         </is>
       </c>
       <c r="H10" s="41" t="inlineStr">
@@ -1884,17 +1902,17 @@
       </c>
       <c r="K10" s="37" t="inlineStr">
         <is>
-          <t>Wikipedia pt https://pt.wikipedia.org/wiki/Fl%C3%A1vio_Bolsonaro | Tribuna do Sertão (link acima) | O Povo 23/07/2026 https://www.opovo.com.br/noticias/politica/2026/07/23/amp/andre-mendonca-autoriza-inquerito-sobre-repasses-para-dark-horse-filme-sobre-jair-bolsonaro.html | Resultado do 1º turno https://portaldeprefeitura.com.br/bastidores-da-politica/eleicoes-2026-com-100-das-secoes-totalizadas-flavio-tem-4703-e/633498/ | Wikipedia (Banco Master scandal) https://en.wikipedia.org/wiki/Banco_Master_scandal | JB 12/10/2026 https://www.jb.com.br/brasil/justica/2026/10/1061206-moraes-autoriza-flavio-bolsonaro-a-visitar-jair-bolsonaro-em-prisao-domiciliar.html | A investigação sobre o financiamento de Dark Horse (bbc.com) https://www.bbc.com/portuguese/articles/c4g5ky0r25jo | A investigação sobre o financiamento de Dark Horse (em.com.br) https://www.em.com.br/politica/2026/09/7498387-flavio-bolsonaro-vira-investigado-do-dark-horse-que-segue-sob-sigilo.html | O acordo de R$ 134 milhões para o filme (intercept.com.br) https://www.intercept.com.br/2026/05/13/audio-flavio-negociou-vorcaro-milhoes/ | A checagem de declarações sobre Vorcaro (aosfatos.org) https://www.aosfatos.org/noticias/flavio-mentiu-ao-menos-43-vezes-sobre-envolvimento-com-vorcaro/ | Os registros de contato no celular do banqueiro (piaui.uol.com.br) https://piaui.uol.com.br/web/mensagens-celular-flavio-vorcaro/ | As menções a encontros presenciais (estadao.com.br) https://www.estadao.com.br/politica/celular-de-vorcaro-tinha-tres-meses-de-conversa-com-flavio-bolsonaro-e-mencao-a-seis-encontros/ | O voo no jato de Vorcaro em janeiro de 2025 (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-viajou-em-jato-de-vorcaro/ | O apartamento de Fabiano Zettel e Willer Tomaz (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-zettel-tomaz-imovel-vila-nova-conceicao-sao-paulo/ | O aniversário em uma mansão gerida por empresa de Vorcaro (iclnoticias.com.br) https://iclnoticias.com.br/flavio-bolsonaro-aniversario-da-filha-em-mansao/ | E-mails sobre vínculo bancário com Willer Tomaz (noticias.uol.com.br) https://noticias.uol.com.br/colunas/fabio-serapiao/2026/10/10/flavio-dividia-conta-com-suspeito-de-lavar-dinheiro-do-inss-indicam-emails.htm | Endereço e contabilidade compartilhados em Brasília (iclnoticias.com.br) https://iclnoticias.com.br/empresas-de-flavio-bolsonaro-e-careca-do-inss/ | Cargo na Câmara, faculdade e estágio no Rio (bbc.com) https://www.bbc.com/portuguese/brasil-46828487 | A acusação de rachadinhas na Alerj (valor.globo.com) https://valor.globo.com/politica/eleicoes-2026/noticia/2026/09/01/flavio-bolsonaro-relembre-o-processo-da-rachadinha.ghtml | A acusação de rachadinhas na Alerj (folhadelondrina.com.br) https://www.folhadelondrina.com.br/ultimas-noticias/entenda-quais-provas-da-rachadinha-contra-flavio-bolsonaro-ainda-valem-3131387e.html | A investigação da loja Kopenhagen (oglobo.globo.com) https://oglobo.globo.com/politica/alvo-de-investigacao-das-rachadinhas-loja-de-flavio-bolsonaro-no-rio-vendida-1-24867874 | Imóveis comprados pela família e investigações (g1.globo.com) https://g1.globo.com/jornal-nacional/noticia/2022/08/31/reportagem-do-uol-revela-que-51-imoveis-comprados-pela-familia-bolsonaro-foram-pagos-em-dinheiro-vivo.ghtml | Imóveis comprados pela família e investigações (noticias.uol.com.br) https://noticias.uol.com.br/politica/ultimas-noticias/2022/08/30/imoveis-cla-bolsonaro-objeto-de-investigacao-suspeita-dinheiro-vivo.htm | Imóveis comprados pela família e investigações (estadao.com.br) https://www.estadao.com.br/politica/investigacao-sobre-flaviobolsonaro-alcanca-37-imoveis/ | A compra e a quitação da mansão em Brasília (oglobo.globo.com) https://oglobo.globo.com/politica/eleicoes-2026/noticia/2026/08/14/video-mansao-que-fez-patrimonio-de-flavio-disparar-fica-em-terreno-de-2400-m-e-foi-quitada-27-anos-antes-do-previsto.ghtml | A análise do MPF sobre 37 transações imobiliárias (cnnbrasil.com.br) https://www.maisgoias.com.br/politica/procurador-aponta-fortes-indicios-de-lavagem-de-dinheiro-em-bens-de-flavio-bolsonaro/ | A acusação do MP-RJ sobre organização criminosa (g1.globo.com) https://g1.globo.com/rj/rio-de-janeiro/noticia/2019/12/19/mp-do-rj-detalha-suposto-esquema-de-corrupcao-envolvendo-entao-deputado-flavio-bolsonaro.ghtml?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=g1 | Destinação de emendas e entidades questionadas (revistaforum.com.br) https://revistaforum.com.br/politica/flavio-bolsonaro-emendas-ong-fantasma-e-instituto-de-miliciano/</t>
+          <t>Wikipedia pt https://pt.wikipedia.org/wiki/Fl%C3%A1vio_Bolsonaro | Tribuna do Sertão (link acima) | O Povo 23/07/2026 https://www.opovo.com.br/noticias/politica/2026/07/23/amp/andre-mendonca-autoriza-inquerito-sobre-repasses-para-dark-horse-filme-sobre-jair-bolsonaro.html | Resultado do 1º turno https://portaldeprefeitura.com.br/bastidores-da-politica/eleicoes-2026-com-100-das-secoes-totalizadas-flavio-tem-4703-e/633498/ | Wikipedia (Banco Master scandal) https://en.wikipedia.org/wiki/Banco_Master_scandal | JB 12/10/2026 https://www.jb.com.br/brasil/justica/2026/10/1061206-moraes-autoriza-flavio-bolsonaro-a-visitar-jair-bolsonaro-em-prisao-domiciliar.html | A investigação sobre o financiamento de Dark Horse (bbc.com) https://www.bbc.com/portuguese/articles/c4g5ky0r25jo | A investigação sobre o financiamento de Dark Horse (em.com.br) https://www.em.com.br/politica/2026/09/7498387-flavio-bolsonaro-vira-investigado-do-dark-horse-que-segue-sob-sigilo.html | O acordo de R$ 134 milhões para o filme (intercept.com.br) https://www.intercept.com.br/2026/05/13/audio-flavio-negociou-vorcaro-milhoes/ | A checagem de declarações sobre Vorcaro (aosfatos.org) https://www.aosfatos.org/noticias/flavio-mentiu-ao-menos-43-vezes-sobre-envolvimento-com-vorcaro/ | Os registros de contato no celular do banqueiro (piaui.uol.com.br) https://piaui.uol.com.br/web/mensagens-celular-flavio-vorcaro/ | As menções a encontros presenciais (estadao.com.br) https://www.estadao.com.br/politica/celular-de-vorcaro-tinha-tres-meses-de-conversa-com-flavio-bolsonaro-e-mencao-a-seis-encontros/ | O voo no jato de Vorcaro em janeiro de 2025 (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-viajou-em-jato-de-vorcaro/ | O apartamento de Fabiano Zettel e Willer Tomaz (piaui.uol.com.br) https://piaui.uol.com.br/web/flavio-bolsonaro-zettel-tomaz-imovel-vila-nova-conceicao-sao-paulo/ | O aniversário em uma mansão gerida por empresa de Vorcaro (iclnoticias.com.br) https://iclnoticias.com.br/flavio-bolsonaro-aniversario-da-filha-em-mansao/ | E-mails sobre vínculo bancário com Willer Tomaz (noticias.uol.com.br) https://noticias.uol.com.br/colunas/fabio-serapiao/2026/10/10/flavio-dividia-conta-com-suspeito-de-lavar-dinheiro-do-inss-indicam-emails.htm | Endereço e contabilidade compartilhados em Brasília (iclnoticias.com.br) https://iclnoticias.com.br/empresas-de-flavio-bolsonaro-e-careca-do-inss/ | Cargo na Câmara, faculdade e estágio no Rio (bbc.com) https://www.bbc.com/portuguese/brasil-46828487 | A acusação de rachadinhas na Alerj (valor.globo.com) https://valor.globo.com/politica/eleicoes-2026/noticia/2026/09/01/flavio-bolsonaro-relembre-o-processo-da-rachadinha.ghtml | A acusação de rachadinhas na Alerj (folhadelondrina.com.br) https://www.folhadelondrina.com.br/ultimas-noticias/entenda-quais-provas-da-rachadinha-contra-flavio-bolsonaro-ainda-valem-3131387e.html | A investigação da loja Kopenhagen (oglobo.globo.com) https://oglobo.globo.com/politica/alvo-de-investigacao-das-rachadinhas-loja-de-flavio-bolsonaro-no-rio-vendida-1-24867874 | Imóveis comprados pela família e investigações (g1.globo.com) https://g1.globo.com/jornal-nacional/noticia/2022/08/31/reportagem-do-uol-revela-que-51-imoveis-comprados-pela-familia-bolsonaro-foram-pagos-em-dinheiro-vivo.ghtml | Imóveis comprados pela família e investigações (noticias.uol.com.br) https://noticias.uol.com.br/politica/ultimas-noticias/2022/08/30/imoveis-cla-bolsonaro-objeto-de-investigacao-suspeita-dinheiro-vivo.htm | Imóveis comprados pela família e investigações (estadao.com.br) https://www.estadao.com.br/politica/investigacao-sobre-flaviobolsonaro-alcanca-37-imoveis/ | A compra e a quitação da mansão em Brasília (oglobo.globo.com) https://oglobo.globo.com/politica/eleicoes-2026/noticia/2026/08/14/video-mansao-que-fez-patrimonio-de-flavio-disparar-fica-em-terreno-de-2400-m-e-foi-quitada-27-anos-antes-do-previsto.ghtml | A análise do MPF sobre 37 transações imobiliárias (cnnbrasil.com.br) https://www.maisgoias.com.br/politica/procurador-aponta-fortes-indicios-de-lavagem-de-dinheiro-em-bens-de-flavio-bolsonaro/ | A acusação do MP-RJ sobre organização criminosa (g1.globo.com) https://g1.globo.com/rj/rio-de-janeiro/noticia/2019/12/19/mp-do-rj-detalha-suposto-esquema-de-corrupcao-envolvendo-entao-deputado-flavio-bolsonaro.ghtml?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=g1 | Destinação de emendas e entidades questionadas (revistaforum.com.br) https://revistaforum.com.br/politica/flavio-bolsonaro-emendas-ong-fantasma-e-instituto-de-miliciano/ | Portal Porque (resume piauí, 20/10/2026) https://www.portalporque.com.br/brasil/revista-piaui-aponta-que-flavio-bolsonaro-foi-socio-indireto-de-bet/ | Notícias ao Minuto (resume piauí) https://www.noticiasaominuto.com.br/politica/2422338/flavio-bolsonaro-e-dono-de-bet-entenda-o-que-a-pf-investiga | Mais Goiás (via Folha, 16/10/2026) https://www.maisgoias.com.br/brasil/pf-descobre-voos-de-flavio-bolsonaro-pagos-por-dono-de-bet-que-e-investigado-por-fraudes-no-inss/</t>
         </is>
       </c>
       <c r="L10" s="37" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="M10" s="37" t="inlineStr">
         <is>
-          <t>Resultado do 1º turno; 2º inquérito no STF; Operação Make Up; visitas ao pai liberadas. 21/10/2026: importado do acervo a verdade. (bolsomaster.site).</t>
+          <t>Resultado do 1º turno; 2º inquérito no STF; Operação Make Up; visitas ao pai liberadas. 21/10/2026: importado do acervo a verdade. (bolsomaster.site). 22/10/2026: rodada UOL News (bets, Loterj, hangar, Weverton).</t>
         </is>
       </c>
       <c r="N10" s="24" t="inlineStr">
@@ -3765,8 +3783,78 @@
       <c r="O35" s="24" t="n"/>
       <c r="P35" s="24" t="n"/>
     </row>
+    <row r="36">
+      <c r="A36" s="37" t="inlineStr">
+        <is>
+          <t>weverton</t>
+        </is>
+      </c>
+      <c r="B36" s="38" t="inlineStr">
+        <is>
+          <t>Weverton Rocha</t>
+        </is>
+      </c>
+      <c r="C36" s="37" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D36" s="37" t="inlineStr">
+        <is>
+          <t>Senador pelo Maranhão (PDT) e vice-líder do governo Lula no Senado. Investigado na Operação Sem Desconto (caso INSS): a PF diz que ele formulava demandas e cobrava pagamentos numa estrutura ligada a Willer Tomaz, que mora numa casa de R$ 6 mi registrada na WT e que a mulher dele, Samya Rocha, recebeu mais de R$ 11 mi de empresas de Willer. Buscas em 04/08/2026, autorizadas por André Mendonça.</t>
+        </is>
+      </c>
+      <c r="E36" s="37" t="inlineStr">
+        <is>
+          <t>Maranhão (MA); mandato em Brasília</t>
+        </is>
+      </c>
+      <c r="F36" s="37" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G36" s="37" t="inlineStr">
+        <is>
+          <t>Investigado, sem denúncia. Diz que as movimentações vêm de atividades profissionais declaradas à Receita e que é alvo por suas posições políticas. Willer diz que os repasses a Samya são honorários de advogada associada.</t>
+        </is>
+      </c>
+      <c r="H36" s="39" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I36" s="37" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J36" s="37" t="inlineStr">
+        <is>
+          <t>“Braço direito” é expressão do UOL News; a PF descreve a estrutura de Willer como “hub financeiro, patrimonial e logístico” do senador.</t>
+        </is>
+      </c>
+      <c r="K36" s="37" t="inlineStr">
+        <is>
+          <t>Poder360 04/08/2026 https://www.poder360.com.br/poder-justica/pf-investiga-advogado-amigo-de-flavio-em-operacao-sobre-o-inss/ | O Povo 04/08/2026 https://www.opovo.com.br/noticias/politica/2026/08/04/pf-investiga-senador-weverton-rocha-por-suspeita-de-desvios-no-inss.html</t>
+        </is>
+      </c>
+      <c r="L36" s="37" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M36" s="37" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada UOL News (bets, Loterj, hangar, Weverton). Perfil novo.</t>
+        </is>
+      </c>
+      <c r="N36" s="24" t="n"/>
+      <c r="O36" s="24" t="n"/>
+      <c r="P36" s="24" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P35"/>
+  <autoFilter ref="A1:P36"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3779,7 +3867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -3869,7 +3957,7 @@
         </is>
       </c>
       <c r="F2" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A2)+COUNTIF(Edges!$B$2:$B$182,A2)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A2)+COUNTIF(Edges!$B$2:$B$198,A2)</f>
         <v/>
       </c>
       <c r="G2" s="24" t="n"/>
@@ -3904,7 +3992,7 @@
         </is>
       </c>
       <c r="F3" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A3)+COUNTIF(Edges!$B$2:$B$182,A3)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A3)+COUNTIF(Edges!$B$2:$B$198,A3)</f>
         <v/>
       </c>
     </row>
@@ -3935,7 +4023,7 @@
         </is>
       </c>
       <c r="F4" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A4)+COUNTIF(Edges!$B$2:$B$182,A4)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A4)+COUNTIF(Edges!$B$2:$B$198,A4)</f>
         <v/>
       </c>
     </row>
@@ -3966,7 +4054,7 @@
         </is>
       </c>
       <c r="F5" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A5)+COUNTIF(Edges!$B$2:$B$182,A5)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A5)+COUNTIF(Edges!$B$2:$B$198,A5)</f>
         <v/>
       </c>
     </row>
@@ -3997,7 +4085,7 @@
         </is>
       </c>
       <c r="F6" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A6)+COUNTIF(Edges!$B$2:$B$182,A6)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A6)+COUNTIF(Edges!$B$2:$B$198,A6)</f>
         <v/>
       </c>
     </row>
@@ -4028,7 +4116,7 @@
         </is>
       </c>
       <c r="F7" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A7)+COUNTIF(Edges!$B$2:$B$182,A7)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A7)+COUNTIF(Edges!$B$2:$B$198,A7)</f>
         <v/>
       </c>
     </row>
@@ -4059,7 +4147,7 @@
         </is>
       </c>
       <c r="F8" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A8)+COUNTIF(Edges!$B$2:$B$182,A8)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A8)+COUNTIF(Edges!$B$2:$B$198,A8)</f>
         <v/>
       </c>
       <c r="G8" s="24" t="n"/>
@@ -4094,7 +4182,7 @@
         </is>
       </c>
       <c r="F9" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A9)+COUNTIF(Edges!$B$2:$B$182,A9)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A9)+COUNTIF(Edges!$B$2:$B$198,A9)</f>
         <v/>
       </c>
       <c r="G9" s="24" t="n"/>
@@ -4129,7 +4217,7 @@
         </is>
       </c>
       <c r="F10" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A10)+COUNTIF(Edges!$B$2:$B$182,A10)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A10)+COUNTIF(Edges!$B$2:$B$198,A10)</f>
         <v/>
       </c>
     </row>
@@ -4160,7 +4248,7 @@
         </is>
       </c>
       <c r="F11" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A11)+COUNTIF(Edges!$B$2:$B$182,A11)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A11)+COUNTIF(Edges!$B$2:$B$198,A11)</f>
         <v/>
       </c>
       <c r="G11" s="24" t="n"/>
@@ -4195,7 +4283,7 @@
         </is>
       </c>
       <c r="F12" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A12)+COUNTIF(Edges!$B$2:$B$182,A12)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A12)+COUNTIF(Edges!$B$2:$B$198,A12)</f>
         <v/>
       </c>
       <c r="G12" s="24" t="inlineStr">
@@ -4242,7 +4330,7 @@
         </is>
       </c>
       <c r="F13" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A13)+COUNTIF(Edges!$B$2:$B$182,A13)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A13)+COUNTIF(Edges!$B$2:$B$198,A13)</f>
         <v/>
       </c>
     </row>
@@ -4273,7 +4361,7 @@
         </is>
       </c>
       <c r="F14" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A14)+COUNTIF(Edges!$B$2:$B$182,A14)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A14)+COUNTIF(Edges!$B$2:$B$198,A14)</f>
         <v/>
       </c>
       <c r="G14" s="24" t="n"/>
@@ -4308,7 +4396,7 @@
         </is>
       </c>
       <c r="F15" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A15)+COUNTIF(Edges!$B$2:$B$182,A15)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A15)+COUNTIF(Edges!$B$2:$B$198,A15)</f>
         <v/>
       </c>
       <c r="G15" s="24" t="n"/>
@@ -4343,7 +4431,7 @@
         </is>
       </c>
       <c r="F16" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A16)+COUNTIF(Edges!$B$2:$B$182,A16)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A16)+COUNTIF(Edges!$B$2:$B$198,A16)</f>
         <v/>
       </c>
       <c r="G16" s="24" t="inlineStr">
@@ -4390,7 +4478,7 @@
         </is>
       </c>
       <c r="F17" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A17)+COUNTIF(Edges!$B$2:$B$182,A17)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A17)+COUNTIF(Edges!$B$2:$B$198,A17)</f>
         <v/>
       </c>
       <c r="G17" s="24" t="inlineStr">
@@ -4437,7 +4525,7 @@
         </is>
       </c>
       <c r="F18" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A18)+COUNTIF(Edges!$B$2:$B$182,A18)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A18)+COUNTIF(Edges!$B$2:$B$198,A18)</f>
         <v/>
       </c>
     </row>
@@ -4468,7 +4556,7 @@
         </is>
       </c>
       <c r="F19" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A19)+COUNTIF(Edges!$B$2:$B$182,A19)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A19)+COUNTIF(Edges!$B$2:$B$198,A19)</f>
         <v/>
       </c>
     </row>
@@ -4499,7 +4587,7 @@
         </is>
       </c>
       <c r="F20" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A20)+COUNTIF(Edges!$B$2:$B$182,A20)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A20)+COUNTIF(Edges!$B$2:$B$198,A20)</f>
         <v/>
       </c>
     </row>
@@ -4530,7 +4618,7 @@
         </is>
       </c>
       <c r="F21" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A21)+COUNTIF(Edges!$B$2:$B$182,A21)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A21)+COUNTIF(Edges!$B$2:$B$198,A21)</f>
         <v/>
       </c>
     </row>
@@ -4561,7 +4649,7 @@
         </is>
       </c>
       <c r="F22" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A22)+COUNTIF(Edges!$B$2:$B$182,A22)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A22)+COUNTIF(Edges!$B$2:$B$198,A22)</f>
         <v/>
       </c>
       <c r="G22" s="24" t="n"/>
@@ -4596,7 +4684,7 @@
         </is>
       </c>
       <c r="F23" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A23)+COUNTIF(Edges!$B$2:$B$182,A23)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A23)+COUNTIF(Edges!$B$2:$B$198,A23)</f>
         <v/>
       </c>
       <c r="G23" s="24" t="n"/>
@@ -4631,7 +4719,7 @@
         </is>
       </c>
       <c r="F24" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A24)+COUNTIF(Edges!$B$2:$B$182,A24)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A24)+COUNTIF(Edges!$B$2:$B$198,A24)</f>
         <v/>
       </c>
     </row>
@@ -4662,7 +4750,7 @@
         </is>
       </c>
       <c r="F25" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A25)+COUNTIF(Edges!$B$2:$B$182,A25)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A25)+COUNTIF(Edges!$B$2:$B$198,A25)</f>
         <v/>
       </c>
     </row>
@@ -4693,7 +4781,7 @@
         </is>
       </c>
       <c r="F26" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A26)+COUNTIF(Edges!$B$2:$B$182,A26)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A26)+COUNTIF(Edges!$B$2:$B$198,A26)</f>
         <v/>
       </c>
     </row>
@@ -4724,7 +4812,7 @@
         </is>
       </c>
       <c r="F27" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A27)+COUNTIF(Edges!$B$2:$B$182,A27)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A27)+COUNTIF(Edges!$B$2:$B$198,A27)</f>
         <v/>
       </c>
     </row>
@@ -4755,7 +4843,7 @@
         </is>
       </c>
       <c r="F28" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A28)+COUNTIF(Edges!$B$2:$B$182,A28)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A28)+COUNTIF(Edges!$B$2:$B$198,A28)</f>
         <v/>
       </c>
     </row>
@@ -4786,7 +4874,7 @@
         </is>
       </c>
       <c r="F29" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A29)+COUNTIF(Edges!$B$2:$B$182,A29)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A29)+COUNTIF(Edges!$B$2:$B$198,A29)</f>
         <v/>
       </c>
     </row>
@@ -4817,7 +4905,7 @@
         </is>
       </c>
       <c r="F30" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A30)+COUNTIF(Edges!$B$2:$B$182,A30)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A30)+COUNTIF(Edges!$B$2:$B$198,A30)</f>
         <v/>
       </c>
       <c r="G30" s="24" t="n"/>
@@ -4852,7 +4940,7 @@
         </is>
       </c>
       <c r="F31" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A31)+COUNTIF(Edges!$B$2:$B$182,A31)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A31)+COUNTIF(Edges!$B$2:$B$198,A31)</f>
         <v/>
       </c>
     </row>
@@ -4883,7 +4971,7 @@
         </is>
       </c>
       <c r="F32" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A32)+COUNTIF(Edges!$B$2:$B$182,A32)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A32)+COUNTIF(Edges!$B$2:$B$198,A32)</f>
         <v/>
       </c>
     </row>
@@ -4914,7 +5002,7 @@
         </is>
       </c>
       <c r="F33" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A33)+COUNTIF(Edges!$B$2:$B$182,A33)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A33)+COUNTIF(Edges!$B$2:$B$198,A33)</f>
         <v/>
       </c>
       <c r="G33" s="24" t="n"/>
@@ -4949,7 +5037,7 @@
         </is>
       </c>
       <c r="F34" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A34)+COUNTIF(Edges!$B$2:$B$182,A34)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A34)+COUNTIF(Edges!$B$2:$B$198,A34)</f>
         <v/>
       </c>
       <c r="G34" s="24" t="n"/>
@@ -4984,7 +5072,7 @@
         </is>
       </c>
       <c r="F35" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A35)+COUNTIF(Edges!$B$2:$B$182,A35)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A35)+COUNTIF(Edges!$B$2:$B$198,A35)</f>
         <v/>
       </c>
     </row>
@@ -5015,7 +5103,7 @@
         </is>
       </c>
       <c r="F36" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A36)+COUNTIF(Edges!$B$2:$B$182,A36)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A36)+COUNTIF(Edges!$B$2:$B$198,A36)</f>
         <v/>
       </c>
     </row>
@@ -5046,7 +5134,7 @@
         </is>
       </c>
       <c r="F37" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A37)+COUNTIF(Edges!$B$2:$B$182,A37)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A37)+COUNTIF(Edges!$B$2:$B$198,A37)</f>
         <v/>
       </c>
     </row>
@@ -5077,7 +5165,7 @@
         </is>
       </c>
       <c r="F38" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A38)+COUNTIF(Edges!$B$2:$B$182,A38)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A38)+COUNTIF(Edges!$B$2:$B$198,A38)</f>
         <v/>
       </c>
       <c r="G38" s="24" t="n"/>
@@ -5112,7 +5200,7 @@
         </is>
       </c>
       <c r="F39" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A39)+COUNTIF(Edges!$B$2:$B$182,A39)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A39)+COUNTIF(Edges!$B$2:$B$198,A39)</f>
         <v/>
       </c>
       <c r="G39" s="24" t="n"/>
@@ -5147,7 +5235,7 @@
         </is>
       </c>
       <c r="F40" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A40)+COUNTIF(Edges!$B$2:$B$182,A40)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A40)+COUNTIF(Edges!$B$2:$B$198,A40)</f>
         <v/>
       </c>
       <c r="G40" s="24" t="n"/>
@@ -5182,7 +5270,7 @@
         </is>
       </c>
       <c r="F41" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A41)+COUNTIF(Edges!$B$2:$B$182,A41)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A41)+COUNTIF(Edges!$B$2:$B$198,A41)</f>
         <v/>
       </c>
       <c r="G41" s="24" t="n"/>
@@ -5217,7 +5305,7 @@
         </is>
       </c>
       <c r="F42" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A42)+COUNTIF(Edges!$B$2:$B$182,A42)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A42)+COUNTIF(Edges!$B$2:$B$198,A42)</f>
         <v/>
       </c>
       <c r="G42" s="24" t="n"/>
@@ -5252,7 +5340,7 @@
         </is>
       </c>
       <c r="F43" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A43)+COUNTIF(Edges!$B$2:$B$182,A43)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A43)+COUNTIF(Edges!$B$2:$B$198,A43)</f>
         <v/>
       </c>
     </row>
@@ -5283,7 +5371,7 @@
         </is>
       </c>
       <c r="F44" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A44)+COUNTIF(Edges!$B$2:$B$182,A44)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A44)+COUNTIF(Edges!$B$2:$B$198,A44)</f>
         <v/>
       </c>
     </row>
@@ -5314,7 +5402,7 @@
         </is>
       </c>
       <c r="F45" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A45)+COUNTIF(Edges!$B$2:$B$182,A45)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A45)+COUNTIF(Edges!$B$2:$B$198,A45)</f>
         <v/>
       </c>
     </row>
@@ -5345,7 +5433,7 @@
         </is>
       </c>
       <c r="F46" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A46)+COUNTIF(Edges!$B$2:$B$182,A46)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A46)+COUNTIF(Edges!$B$2:$B$198,A46)</f>
         <v/>
       </c>
     </row>
@@ -5376,7 +5464,7 @@
         </is>
       </c>
       <c r="F47" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A47)+COUNTIF(Edges!$B$2:$B$182,A47)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A47)+COUNTIF(Edges!$B$2:$B$198,A47)</f>
         <v/>
       </c>
     </row>
@@ -5407,7 +5495,7 @@
         </is>
       </c>
       <c r="F48" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A48)+COUNTIF(Edges!$B$2:$B$182,A48)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A48)+COUNTIF(Edges!$B$2:$B$198,A48)</f>
         <v/>
       </c>
       <c r="G48" s="24" t="n"/>
@@ -5442,7 +5530,7 @@
         </is>
       </c>
       <c r="F49" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A49)+COUNTIF(Edges!$B$2:$B$182,A49)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A49)+COUNTIF(Edges!$B$2:$B$198,A49)</f>
         <v/>
       </c>
     </row>
@@ -5473,7 +5561,7 @@
         </is>
       </c>
       <c r="F50" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A50)+COUNTIF(Edges!$B$2:$B$182,A50)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A50)+COUNTIF(Edges!$B$2:$B$198,A50)</f>
         <v/>
       </c>
     </row>
@@ -5504,7 +5592,7 @@
         </is>
       </c>
       <c r="F51" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A51)+COUNTIF(Edges!$B$2:$B$182,A51)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A51)+COUNTIF(Edges!$B$2:$B$198,A51)</f>
         <v/>
       </c>
     </row>
@@ -5535,7 +5623,7 @@
         </is>
       </c>
       <c r="F52" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A52)+COUNTIF(Edges!$B$2:$B$182,A52)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A52)+COUNTIF(Edges!$B$2:$B$198,A52)</f>
         <v/>
       </c>
       <c r="G52" s="24" t="inlineStr">
@@ -5582,7 +5670,7 @@
         </is>
       </c>
       <c r="F53" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A53)+COUNTIF(Edges!$B$2:$B$182,A53)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A53)+COUNTIF(Edges!$B$2:$B$198,A53)</f>
         <v/>
       </c>
       <c r="G53" s="24" t="inlineStr">
@@ -5629,7 +5717,7 @@
         </is>
       </c>
       <c r="F54" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A54)+COUNTIF(Edges!$B$2:$B$182,A54)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A54)+COUNTIF(Edges!$B$2:$B$198,A54)</f>
         <v/>
       </c>
       <c r="G54" s="24" t="inlineStr">
@@ -5676,7 +5764,7 @@
         </is>
       </c>
       <c r="F55" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A55)+COUNTIF(Edges!$B$2:$B$182,A55)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A55)+COUNTIF(Edges!$B$2:$B$198,A55)</f>
         <v/>
       </c>
       <c r="G55" s="24" t="inlineStr">
@@ -5723,7 +5811,7 @@
         </is>
       </c>
       <c r="F56" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A56)+COUNTIF(Edges!$B$2:$B$182,A56)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A56)+COUNTIF(Edges!$B$2:$B$198,A56)</f>
         <v/>
       </c>
     </row>
@@ -5754,7 +5842,7 @@
         </is>
       </c>
       <c r="F57" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A57)+COUNTIF(Edges!$B$2:$B$182,A57)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A57)+COUNTIF(Edges!$B$2:$B$198,A57)</f>
         <v/>
       </c>
       <c r="G57" s="24" t="inlineStr">
@@ -5801,7 +5889,7 @@
         </is>
       </c>
       <c r="F58" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A58)+COUNTIF(Edges!$B$2:$B$182,A58)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A58)+COUNTIF(Edges!$B$2:$B$198,A58)</f>
         <v/>
       </c>
       <c r="G58" s="24" t="inlineStr">
@@ -5848,7 +5936,7 @@
         </is>
       </c>
       <c r="F59" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A59)+COUNTIF(Edges!$B$2:$B$182,A59)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A59)+COUNTIF(Edges!$B$2:$B$198,A59)</f>
         <v/>
       </c>
       <c r="G59" s="24" t="n"/>
@@ -5883,7 +5971,7 @@
         </is>
       </c>
       <c r="F60" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A60)+COUNTIF(Edges!$B$2:$B$182,A60)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A60)+COUNTIF(Edges!$B$2:$B$198,A60)</f>
         <v/>
       </c>
       <c r="G60" s="24" t="n"/>
@@ -5918,7 +6006,7 @@
         </is>
       </c>
       <c r="F61" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A61)+COUNTIF(Edges!$B$2:$B$182,A61)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A61)+COUNTIF(Edges!$B$2:$B$198,A61)</f>
         <v/>
       </c>
       <c r="G61" s="24" t="n"/>
@@ -5953,7 +6041,7 @@
         </is>
       </c>
       <c r="F62" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A62)+COUNTIF(Edges!$B$2:$B$182,A62)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A62)+COUNTIF(Edges!$B$2:$B$198,A62)</f>
         <v/>
       </c>
       <c r="G62" s="24" t="n"/>
@@ -5988,7 +6076,7 @@
         </is>
       </c>
       <c r="F63" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A63)+COUNTIF(Edges!$B$2:$B$182,A63)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A63)+COUNTIF(Edges!$B$2:$B$198,A63)</f>
         <v/>
       </c>
       <c r="G63" s="24" t="n"/>
@@ -6023,7 +6111,7 @@
         </is>
       </c>
       <c r="F64" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A64)+COUNTIF(Edges!$B$2:$B$182,A64)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A64)+COUNTIF(Edges!$B$2:$B$198,A64)</f>
         <v/>
       </c>
       <c r="G64" s="24" t="n"/>
@@ -6058,7 +6146,7 @@
         </is>
       </c>
       <c r="F65" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A65)+COUNTIF(Edges!$B$2:$B$182,A65)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A65)+COUNTIF(Edges!$B$2:$B$198,A65)</f>
         <v/>
       </c>
       <c r="G65" s="24" t="n"/>
@@ -6093,7 +6181,7 @@
         </is>
       </c>
       <c r="F66" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A66)+COUNTIF(Edges!$B$2:$B$182,A66)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A66)+COUNTIF(Edges!$B$2:$B$198,A66)</f>
         <v/>
       </c>
       <c r="G66" s="24" t="n"/>
@@ -6128,7 +6216,7 @@
         </is>
       </c>
       <c r="F67" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A67)+COUNTIF(Edges!$B$2:$B$182,A67)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A67)+COUNTIF(Edges!$B$2:$B$198,A67)</f>
         <v/>
       </c>
       <c r="G67" s="24" t="n"/>
@@ -6163,7 +6251,7 @@
         </is>
       </c>
       <c r="F68" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A68)+COUNTIF(Edges!$B$2:$B$182,A68)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A68)+COUNTIF(Edges!$B$2:$B$198,A68)</f>
         <v/>
       </c>
       <c r="G68" s="24" t="n"/>
@@ -6198,7 +6286,7 @@
         </is>
       </c>
       <c r="F69" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A69)+COUNTIF(Edges!$B$2:$B$182,A69)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A69)+COUNTIF(Edges!$B$2:$B$198,A69)</f>
         <v/>
       </c>
       <c r="G69" s="24" t="n"/>
@@ -6233,7 +6321,7 @@
         </is>
       </c>
       <c r="F70" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A70)+COUNTIF(Edges!$B$2:$B$182,A70)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A70)+COUNTIF(Edges!$B$2:$B$198,A70)</f>
         <v/>
       </c>
       <c r="G70" s="24" t="n"/>
@@ -6268,7 +6356,7 @@
         </is>
       </c>
       <c r="F71" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A71)+COUNTIF(Edges!$B$2:$B$182,A71)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A71)+COUNTIF(Edges!$B$2:$B$198,A71)</f>
         <v/>
       </c>
       <c r="G71" s="24" t="n"/>
@@ -6303,7 +6391,7 @@
         </is>
       </c>
       <c r="F72" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A72)+COUNTIF(Edges!$B$2:$B$182,A72)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A72)+COUNTIF(Edges!$B$2:$B$198,A72)</f>
         <v/>
       </c>
       <c r="G72" s="24" t="n"/>
@@ -6338,7 +6426,7 @@
         </is>
       </c>
       <c r="F73" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A73)+COUNTIF(Edges!$B$2:$B$182,A73)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A73)+COUNTIF(Edges!$B$2:$B$198,A73)</f>
         <v/>
       </c>
       <c r="G73" s="24" t="n"/>
@@ -6373,7 +6461,7 @@
         </is>
       </c>
       <c r="F74" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A74)+COUNTIF(Edges!$B$2:$B$182,A74)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A74)+COUNTIF(Edges!$B$2:$B$198,A74)</f>
         <v/>
       </c>
       <c r="G74" s="24" t="n"/>
@@ -6408,7 +6496,7 @@
         </is>
       </c>
       <c r="F75" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A75)+COUNTIF(Edges!$B$2:$B$182,A75)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A75)+COUNTIF(Edges!$B$2:$B$198,A75)</f>
         <v/>
       </c>
       <c r="G75" s="24" t="n"/>
@@ -6443,7 +6531,7 @@
         </is>
       </c>
       <c r="F76" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A76)+COUNTIF(Edges!$B$2:$B$182,A76)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A76)+COUNTIF(Edges!$B$2:$B$198,A76)</f>
         <v/>
       </c>
       <c r="G76" s="24" t="n"/>
@@ -6478,7 +6566,7 @@
         </is>
       </c>
       <c r="F77" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A77)+COUNTIF(Edges!$B$2:$B$182,A77)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A77)+COUNTIF(Edges!$B$2:$B$198,A77)</f>
         <v/>
       </c>
       <c r="G77" s="24" t="n"/>
@@ -6513,7 +6601,7 @@
         </is>
       </c>
       <c r="F78" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A78)+COUNTIF(Edges!$B$2:$B$182,A78)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A78)+COUNTIF(Edges!$B$2:$B$198,A78)</f>
         <v/>
       </c>
       <c r="G78" s="24" t="n"/>
@@ -6548,7 +6636,7 @@
         </is>
       </c>
       <c r="F79" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A79)+COUNTIF(Edges!$B$2:$B$182,A79)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A79)+COUNTIF(Edges!$B$2:$B$198,A79)</f>
         <v/>
       </c>
       <c r="G79" s="24" t="n"/>
@@ -6583,7 +6671,7 @@
         </is>
       </c>
       <c r="F80" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A80)+COUNTIF(Edges!$B$2:$B$182,A80)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A80)+COUNTIF(Edges!$B$2:$B$198,A80)</f>
         <v/>
       </c>
       <c r="G80" s="24" t="n"/>
@@ -6618,7 +6706,7 @@
         </is>
       </c>
       <c r="F81" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A81)+COUNTIF(Edges!$B$2:$B$182,A81)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A81)+COUNTIF(Edges!$B$2:$B$198,A81)</f>
         <v/>
       </c>
       <c r="G81" s="24" t="n"/>
@@ -6653,7 +6741,7 @@
         </is>
       </c>
       <c r="F82" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A82)+COUNTIF(Edges!$B$2:$B$182,A82)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A82)+COUNTIF(Edges!$B$2:$B$198,A82)</f>
         <v/>
       </c>
       <c r="G82" s="24" t="n"/>
@@ -6688,7 +6776,7 @@
         </is>
       </c>
       <c r="F83" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A83)+COUNTIF(Edges!$B$2:$B$182,A83)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A83)+COUNTIF(Edges!$B$2:$B$198,A83)</f>
         <v/>
       </c>
       <c r="G83" s="24" t="n"/>
@@ -6723,13 +6811,258 @@
         </is>
       </c>
       <c r="F84" s="45">
-        <f>COUNTIF(Edges!$A$2:$A$182,A84)+COUNTIF(Edges!$B$2:$B$182,A84)</f>
+        <f>COUNTIF(Edges!$A$2:$A$198,A84)+COUNTIF(Edges!$B$2:$B$198,A84)</f>
         <v/>
       </c>
       <c r="G84" s="24" t="n"/>
       <c r="H84" s="24" t="n"/>
       <c r="I84" s="24" t="n"/>
       <c r="J84" s="24" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="45" t="inlineStr">
+        <is>
+          <t>cathedral</t>
+        </is>
+      </c>
+      <c r="B85" s="45" t="inlineStr">
+        <is>
+          <t>Cathedral Holdings</t>
+        </is>
+      </c>
+      <c r="C85" s="45" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="D85" s="45" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="E85" s="45" t="inlineStr">
+        <is>
+          <t>Offshore na Ilha da Madeira criada por Willer em jan/2023; única acionista da Rede Loto</t>
+        </is>
+      </c>
+      <c r="F85" s="45">
+        <f>COUNTIF(Edges!$A$2:$A$198,A85)+COUNTIF(Edges!$B$2:$B$198,A85)</f>
+        <v/>
+      </c>
+      <c r="G85" s="24" t="n"/>
+      <c r="H85" s="24" t="n"/>
+      <c r="I85" s="24" t="n"/>
+      <c r="J85" s="24" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="45" t="inlineStr">
+        <is>
+          <t>bestbet</t>
+        </is>
+      </c>
+      <c r="B86" s="45" t="inlineStr">
+        <is>
+          <t>Best Bet (Rede Loto)</t>
+        </is>
+      </c>
+      <c r="C86" s="45" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="D86" s="45" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="E86" s="45" t="inlineStr">
+        <is>
+          <t>Bet licenciada pela Loterj em mai/2023; a defesa diz que nunca chegou a operar</t>
+        </is>
+      </c>
+      <c r="F86" s="45">
+        <f>COUNTIF(Edges!$A$2:$A$198,A86)+COUNTIF(Edges!$B$2:$B$198,A86)</f>
+        <v/>
+      </c>
+      <c r="G86" s="24" t="n"/>
+      <c r="H86" s="24" t="n"/>
+      <c r="I86" s="24" t="n"/>
+      <c r="J86" s="24" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="45" t="inlineStr">
+        <is>
+          <t>riopag</t>
+        </is>
+      </c>
+      <c r="B87" s="45" t="inlineStr">
+        <is>
+          <t>Rio Pag</t>
+        </is>
+      </c>
+      <c r="C87" s="45" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="D87" s="45" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="E87" s="45" t="inlineStr">
+        <is>
+          <t>Processava pagamentos da Loterj; contrato rescindido pelo estado, que cobra ~R$ 4 mi</t>
+        </is>
+      </c>
+      <c r="F87" s="45">
+        <f>COUNTIF(Edges!$A$2:$A$198,A87)+COUNTIF(Edges!$B$2:$B$198,A87)</f>
+        <v/>
+      </c>
+      <c r="G87" s="24" t="n"/>
+      <c r="H87" s="24" t="n"/>
+      <c r="I87" s="24" t="n"/>
+      <c r="J87" s="24" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="45" t="inlineStr">
+        <is>
+          <t>loterj</t>
+        </is>
+      </c>
+      <c r="B88" s="45" t="inlineStr">
+        <is>
+          <t>Loterj</t>
+        </is>
+      </c>
+      <c r="C88" s="45" t="inlineStr">
+        <is>
+          <t>Instituição ou caso</t>
+        </is>
+      </c>
+      <c r="D88" s="45" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="E88" s="45" t="inlineStr">
+        <is>
+          <t>Loteria do Estado do RJ; licenciou a Best Bet e contratou a Rio Pag em 2023</t>
+        </is>
+      </c>
+      <c r="F88" s="45">
+        <f>COUNTIF(Edges!$A$2:$A$198,A88)+COUNTIF(Edges!$B$2:$B$198,A88)</f>
+        <v/>
+      </c>
+      <c r="G88" s="24" t="n"/>
+      <c r="H88" s="24" t="n"/>
+      <c r="I88" s="24" t="n"/>
+      <c r="J88" s="24" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="45" t="inlineStr">
+        <is>
+          <t>cancado</t>
+        </is>
+      </c>
+      <c r="B89" s="45" t="inlineStr">
+        <is>
+          <t>Hazenclever Cançado</t>
+        </is>
+      </c>
+      <c r="C89" s="45" t="inlineStr">
+        <is>
+          <t>Pessoa</t>
+        </is>
+      </c>
+      <c r="D89" s="45" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="E89" s="45" t="inlineStr">
+        <is>
+          <t>Ex-presidente da Loterj; assinou a licença da Best Bet</t>
+        </is>
+      </c>
+      <c r="F89" s="45">
+        <f>COUNTIF(Edges!$A$2:$A$198,A89)+COUNTIF(Edges!$B$2:$B$198,A89)</f>
+        <v/>
+      </c>
+      <c r="G89" s="24" t="n"/>
+      <c r="H89" s="24" t="n"/>
+      <c r="I89" s="24" t="n"/>
+      <c r="J89" s="24" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="45" t="inlineStr">
+        <is>
+          <t>hangar</t>
+        </is>
+      </c>
+      <c r="B90" s="45" t="inlineStr">
+        <is>
+          <t>Hangares de Willer (Aeroporto de Brasília)</t>
+        </is>
+      </c>
+      <c r="C90" s="45" t="inlineStr">
+        <is>
+          <t>Casa ou ativo</t>
+        </is>
+      </c>
+      <c r="D90" s="45" t="inlineStr">
+        <is>
+          <t>Casas e ativos</t>
+        </is>
+      </c>
+      <c r="E90" s="45" t="inlineStr">
+        <is>
+          <t>Hangares 36 e 37; PF achou sala oculta e máquina de contar, sem dinheiro; Willer diz que atende transporte de valores</t>
+        </is>
+      </c>
+      <c r="F90" s="45">
+        <f>COUNTIF(Edges!$A$2:$A$198,A90)+COUNTIF(Edges!$B$2:$B$198,A90)</f>
+        <v/>
+      </c>
+      <c r="G90" s="24" t="n"/>
+      <c r="H90" s="24" t="n"/>
+      <c r="I90" s="24" t="n"/>
+      <c r="J90" s="24" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="45" t="inlineStr">
+        <is>
+          <t>weverton</t>
+        </is>
+      </c>
+      <c r="B91" s="45" t="inlineStr">
+        <is>
+          <t>Weverton Rocha</t>
+        </is>
+      </c>
+      <c r="C91" s="45" t="inlineStr">
+        <is>
+          <t>Pessoa</t>
+        </is>
+      </c>
+      <c r="D91" s="45" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="E91" s="45" t="inlineStr">
+        <is>
+          <t>Senador (PDT-MA), vice-líder do governo Lula; investigado na Operação Sem Desconto; nega</t>
+        </is>
+      </c>
+      <c r="F91" s="45">
+        <f>COUNTIF(Edges!$A$2:$A$198,A91)+COUNTIF(Edges!$B$2:$B$198,A91)</f>
+        <v/>
+      </c>
+      <c r="G91" s="24" t="n"/>
+      <c r="H91" s="24" t="n"/>
+      <c r="I91" s="24" t="n"/>
+      <c r="J91" s="24" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F58"/>
@@ -6745,7 +7078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F182"/>
+  <dimension ref="A1:F198"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="2"/>
@@ -6808,11 +7141,11 @@
         </is>
       </c>
       <c r="E2" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A2,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A2,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F2" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B2,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B2,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -6838,11 +7171,11 @@
         </is>
       </c>
       <c r="E3" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A3,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A3,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F3" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B3,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B3,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -6868,11 +7201,11 @@
         </is>
       </c>
       <c r="E4" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A4,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A4,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F4" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B4,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B4,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -6898,11 +7231,11 @@
         </is>
       </c>
       <c r="E5" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A5,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A5,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F5" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B5,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B5,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -6928,11 +7261,11 @@
         </is>
       </c>
       <c r="E6" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A6,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A6,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F6" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B6,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B6,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -6958,11 +7291,11 @@
         </is>
       </c>
       <c r="E7" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A7,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A7,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F7" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B7,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B7,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -6988,11 +7321,11 @@
         </is>
       </c>
       <c r="E8" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A8,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A8,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F8" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B8,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B8,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7018,11 +7351,11 @@
         </is>
       </c>
       <c r="E9" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A9,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A9,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F9" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B9,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B9,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7048,11 +7381,11 @@
         </is>
       </c>
       <c r="E10" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A10,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A10,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F10" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B10,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B10,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7078,11 +7411,11 @@
         </is>
       </c>
       <c r="E11" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A11,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A11,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F11" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B11,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B11,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7108,11 +7441,11 @@
         </is>
       </c>
       <c r="E12" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A12,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A12,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F12" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B12,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B12,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7138,11 +7471,11 @@
         </is>
       </c>
       <c r="E13" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A13,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A13,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F13" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B13,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B13,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7168,11 +7501,11 @@
         </is>
       </c>
       <c r="E14" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A14,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A14,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F14" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B14,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B14,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7198,11 +7531,11 @@
         </is>
       </c>
       <c r="E15" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A15,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A15,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F15" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B15,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B15,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7228,11 +7561,11 @@
         </is>
       </c>
       <c r="E16" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A16,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A16,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F16" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B16,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B16,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7258,11 +7591,11 @@
         </is>
       </c>
       <c r="E17" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A17,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A17,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F17" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B17,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B17,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7288,11 +7621,11 @@
         </is>
       </c>
       <c r="E18" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A18,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A18,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F18" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B18,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B18,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7318,11 +7651,11 @@
         </is>
       </c>
       <c r="E19" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A19,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A19,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F19" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B19,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B19,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7348,11 +7681,11 @@
         </is>
       </c>
       <c r="E20" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A20,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A20,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F20" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B20,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B20,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7378,11 +7711,11 @@
         </is>
       </c>
       <c r="E21" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A21,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A21,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F21" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B21,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B21,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7408,11 +7741,11 @@
         </is>
       </c>
       <c r="E22" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A22,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A22,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F22" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B22,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B22,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7438,11 +7771,11 @@
         </is>
       </c>
       <c r="E23" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A23,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A23,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F23" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B23,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B23,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7468,11 +7801,11 @@
         </is>
       </c>
       <c r="E24" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A24,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A24,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F24" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B24,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B24,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7489,7 +7822,7 @@
       </c>
       <c r="C25" s="45" t="inlineStr">
         <is>
-          <t>Flávio era “usuário master”; excluído após a 1ª operação</t>
+          <t>PF/piauí: Flávio era “usuário master” da conta da Alcazar; e-mail de 22/05/2025 pediu a exclusão dele. Ele nega ter tido acesso</t>
         </is>
       </c>
       <c r="D25" s="45" t="inlineStr">
@@ -7498,11 +7831,11 @@
         </is>
       </c>
       <c r="E25" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A25,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A25,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F25" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B25,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B25,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7528,11 +7861,11 @@
         </is>
       </c>
       <c r="E26" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A26,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A26,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F26" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B26,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B26,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7558,11 +7891,11 @@
         </is>
       </c>
       <c r="E27" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A27,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A27,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F27" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B27,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B27,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7588,11 +7921,11 @@
         </is>
       </c>
       <c r="E28" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A28,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A28,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F28" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B28,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B28,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7618,11 +7951,11 @@
         </is>
       </c>
       <c r="E29" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A29,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A29,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F29" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B29,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B29,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7648,11 +7981,11 @@
         </is>
       </c>
       <c r="E30" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A30,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A30,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F30" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B30,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B30,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7678,11 +8011,11 @@
         </is>
       </c>
       <c r="E31" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A31,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A31,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F31" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B31,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B31,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7708,11 +8041,11 @@
         </is>
       </c>
       <c r="E32" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A32,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A32,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F32" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B32,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B32,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7738,11 +8071,11 @@
         </is>
       </c>
       <c r="E33" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A33,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A33,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F33" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B33,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B33,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7768,11 +8101,11 @@
         </is>
       </c>
       <c r="E34" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A34,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A34,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F34" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B34,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B34,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7798,11 +8131,11 @@
         </is>
       </c>
       <c r="E35" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A35,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A35,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F35" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B35,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B35,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7828,11 +8161,11 @@
         </is>
       </c>
       <c r="E36" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A36,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A36,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F36" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B36,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B36,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7858,11 +8191,11 @@
         </is>
       </c>
       <c r="E37" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A37,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A37,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F37" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B37,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B37,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7888,11 +8221,11 @@
         </is>
       </c>
       <c r="E38" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A38,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A38,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F38" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B38,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B38,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7918,11 +8251,11 @@
         </is>
       </c>
       <c r="E39" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A39,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A39,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F39" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B39,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B39,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7948,11 +8281,11 @@
         </is>
       </c>
       <c r="E40" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A40,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A40,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F40" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B40,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B40,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -7978,11 +8311,11 @@
         </is>
       </c>
       <c r="E41" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A41,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A41,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F41" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B41,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B41,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8008,11 +8341,11 @@
         </is>
       </c>
       <c r="E42" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A42,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A42,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F42" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B42,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B42,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8038,11 +8371,11 @@
         </is>
       </c>
       <c r="E43" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A43,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A43,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F43" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B43,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B43,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8068,11 +8401,11 @@
         </is>
       </c>
       <c r="E44" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A44,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A44,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F44" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B44,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B44,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8098,11 +8431,11 @@
         </is>
       </c>
       <c r="E45" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A45,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A45,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F45" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B45,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B45,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8128,11 +8461,11 @@
         </is>
       </c>
       <c r="E46" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A46,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A46,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F46" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B46,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B46,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8158,11 +8491,11 @@
         </is>
       </c>
       <c r="E47" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A47,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A47,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F47" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B47,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B47,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8188,11 +8521,11 @@
         </is>
       </c>
       <c r="E48" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A48,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A48,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F48" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B48,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B48,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8218,11 +8551,11 @@
         </is>
       </c>
       <c r="E49" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A49,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A49,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F49" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B49,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B49,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8248,11 +8581,11 @@
         </is>
       </c>
       <c r="E50" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A50,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A50,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F50" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B50,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B50,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8278,11 +8611,11 @@
         </is>
       </c>
       <c r="E51" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A51,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A51,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F51" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B51,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B51,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8308,11 +8641,11 @@
         </is>
       </c>
       <c r="E52" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A52,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A52,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F52" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B52,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B52,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8338,11 +8671,11 @@
         </is>
       </c>
       <c r="E53" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A53,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A53,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F53" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B53,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B53,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8368,11 +8701,11 @@
         </is>
       </c>
       <c r="E54" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A54,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A54,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F54" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B54,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B54,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8398,11 +8731,11 @@
         </is>
       </c>
       <c r="E55" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A55,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A55,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F55" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B55,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B55,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8428,11 +8761,11 @@
         </is>
       </c>
       <c r="E56" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A56,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A56,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F56" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B56,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B56,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8458,11 +8791,11 @@
         </is>
       </c>
       <c r="E57" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A57,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A57,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F57" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B57,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B57,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8488,11 +8821,11 @@
         </is>
       </c>
       <c r="E58" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A58,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A58,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F58" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B58,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B58,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8518,11 +8851,11 @@
         </is>
       </c>
       <c r="E59" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A59,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A59,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F59" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B59,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B59,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8548,11 +8881,11 @@
         </is>
       </c>
       <c r="E60" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A60,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A60,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F60" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B60,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B60,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8578,11 +8911,11 @@
         </is>
       </c>
       <c r="E61" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A61,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A61,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F61" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B61,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B61,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8608,11 +8941,11 @@
         </is>
       </c>
       <c r="E62" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A62,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A62,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F62" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B62,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B62,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8638,11 +8971,11 @@
         </is>
       </c>
       <c r="E63" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A63,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A63,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F63" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B63,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B63,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8668,11 +9001,11 @@
         </is>
       </c>
       <c r="E64" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A64,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A64,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F64" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B64,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B64,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8698,11 +9031,11 @@
         </is>
       </c>
       <c r="E65" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A65,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A65,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F65" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B65,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B65,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8728,11 +9061,11 @@
         </is>
       </c>
       <c r="E66" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A66,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A66,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F66" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B66,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B66,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8758,11 +9091,11 @@
         </is>
       </c>
       <c r="E67" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A67,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A67,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F67" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B67,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B67,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8788,11 +9121,11 @@
         </is>
       </c>
       <c r="E68" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A68,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A68,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F68" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B68,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B68,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8818,11 +9151,11 @@
         </is>
       </c>
       <c r="E69" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A69,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A69,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F69" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B69,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B69,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8848,11 +9181,11 @@
         </is>
       </c>
       <c r="E70" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A70,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A70,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F70" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B70,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B70,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8878,11 +9211,11 @@
         </is>
       </c>
       <c r="E71" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A71,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A71,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F71" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B71,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B71,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8908,11 +9241,11 @@
         </is>
       </c>
       <c r="E72" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A72,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A72,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F72" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B72,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B72,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8938,11 +9271,11 @@
         </is>
       </c>
       <c r="E73" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A73,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A73,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F73" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B73,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B73,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8968,11 +9301,11 @@
         </is>
       </c>
       <c r="E74" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A74,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A74,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F74" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B74,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B74,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -8998,11 +9331,11 @@
         </is>
       </c>
       <c r="E75" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A75,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A75,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F75" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B75,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B75,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9028,11 +9361,11 @@
         </is>
       </c>
       <c r="E76" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A76,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A76,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F76" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B76,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B76,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9058,11 +9391,11 @@
         </is>
       </c>
       <c r="E77" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A77,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A77,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F77" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B77,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B77,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9088,11 +9421,11 @@
         </is>
       </c>
       <c r="E78" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A78,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A78,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F78" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B78,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B78,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9118,11 +9451,11 @@
         </is>
       </c>
       <c r="E79" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A79,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A79,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F79" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B79,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B79,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9148,11 +9481,11 @@
         </is>
       </c>
       <c r="E80" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A80,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A80,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F80" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B80,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B80,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9178,11 +9511,11 @@
         </is>
       </c>
       <c r="E81" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A81,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A81,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F81" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B81,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B81,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9208,11 +9541,11 @@
         </is>
       </c>
       <c r="E82" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A82,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A82,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F82" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B82,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B82,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9238,11 +9571,11 @@
         </is>
       </c>
       <c r="E83" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A83,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A83,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F83" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B83,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B83,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9268,11 +9601,11 @@
         </is>
       </c>
       <c r="E84" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A84,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A84,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F84" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B84,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B84,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9298,11 +9631,11 @@
         </is>
       </c>
       <c r="E85" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A85,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A85,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F85" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B85,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B85,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9328,11 +9661,11 @@
         </is>
       </c>
       <c r="E86" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A86,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A86,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F86" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B86,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B86,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9358,11 +9691,11 @@
         </is>
       </c>
       <c r="E87" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A87,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A87,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F87" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B87,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B87,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9388,11 +9721,11 @@
         </is>
       </c>
       <c r="E88" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A88,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A88,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F88" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B88,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B88,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9418,11 +9751,11 @@
         </is>
       </c>
       <c r="E89" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A89,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A89,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F89" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B89,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B89,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9448,11 +9781,11 @@
         </is>
       </c>
       <c r="E90" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A90,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A90,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F90" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B90,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B90,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9478,11 +9811,11 @@
         </is>
       </c>
       <c r="E91" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A91,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A91,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F91" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B91,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B91,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9508,11 +9841,11 @@
         </is>
       </c>
       <c r="E92" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A92,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A92,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F92" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B92,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B92,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9538,11 +9871,11 @@
         </is>
       </c>
       <c r="E93" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A93,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A93,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F93" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B93,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B93,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9568,11 +9901,11 @@
         </is>
       </c>
       <c r="E94" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A94,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A94,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F94" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B94,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B94,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9598,11 +9931,11 @@
         </is>
       </c>
       <c r="E95" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A95,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A95,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F95" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B95,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B95,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9628,11 +9961,11 @@
         </is>
       </c>
       <c r="E96" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A96,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A96,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F96" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B96,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B96,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9658,11 +9991,11 @@
         </is>
       </c>
       <c r="E97" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A97,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A97,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F97" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B97,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B97,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9688,11 +10021,11 @@
         </is>
       </c>
       <c r="E98" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A98,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A98,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F98" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B98,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B98,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9718,11 +10051,11 @@
         </is>
       </c>
       <c r="E99" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A99,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A99,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F99" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B99,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B99,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9748,11 +10081,11 @@
         </is>
       </c>
       <c r="E100" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A100,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A100,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F100" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B100,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B100,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9778,11 +10111,11 @@
         </is>
       </c>
       <c r="E101" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A101,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A101,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F101" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B101,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B101,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9808,11 +10141,11 @@
         </is>
       </c>
       <c r="E102" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A102,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A102,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F102" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B102,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B102,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9838,11 +10171,11 @@
         </is>
       </c>
       <c r="E103" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A103,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A103,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F103" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B103,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B103,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9868,11 +10201,11 @@
         </is>
       </c>
       <c r="E104" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A104,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A104,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F104" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B104,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B104,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9898,11 +10231,11 @@
         </is>
       </c>
       <c r="E105" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A105,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A105,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F105" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B105,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B105,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9928,11 +10261,11 @@
         </is>
       </c>
       <c r="E106" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A106,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A106,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F106" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B106,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B106,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9958,11 +10291,11 @@
         </is>
       </c>
       <c r="E107" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A107,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A107,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F107" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B107,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B107,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -9988,11 +10321,11 @@
         </is>
       </c>
       <c r="E108" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A108,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A108,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F108" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B108,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B108,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10018,11 +10351,11 @@
         </is>
       </c>
       <c r="E109" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A109,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A109,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F109" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B109,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B109,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10048,11 +10381,11 @@
         </is>
       </c>
       <c r="E110" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A110,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A110,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F110" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B110,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B110,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10078,11 +10411,11 @@
         </is>
       </c>
       <c r="E111" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A111,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A111,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F111" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B111,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B111,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10108,11 +10441,11 @@
         </is>
       </c>
       <c r="E112" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A112,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A112,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F112" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B112,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B112,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10138,11 +10471,11 @@
         </is>
       </c>
       <c r="E113" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A113,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A113,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F113" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B113,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B113,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10168,11 +10501,11 @@
         </is>
       </c>
       <c r="E114" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A114,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A114,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F114" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B114,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B114,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10198,11 +10531,11 @@
         </is>
       </c>
       <c r="E115" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A115,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A115,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F115" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B115,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B115,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10228,11 +10561,11 @@
         </is>
       </c>
       <c r="E116" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A116,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A116,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F116" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B116,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B116,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10258,11 +10591,11 @@
         </is>
       </c>
       <c r="E117" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A117,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A117,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F117" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B117,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B117,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10288,11 +10621,11 @@
         </is>
       </c>
       <c r="E118" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A118,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A118,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F118" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B118,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B118,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10318,11 +10651,11 @@
         </is>
       </c>
       <c r="E119" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A119,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A119,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F119" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B119,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B119,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10348,11 +10681,11 @@
         </is>
       </c>
       <c r="E120" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A120,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A120,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F120" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B120,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B120,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10378,11 +10711,11 @@
         </is>
       </c>
       <c r="E121" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A121,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A121,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F121" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B121,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B121,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10408,11 +10741,11 @@
         </is>
       </c>
       <c r="E122" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A122,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A122,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F122" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B122,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B122,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10438,11 +10771,11 @@
         </is>
       </c>
       <c r="E123" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A123,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A123,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F123" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B123,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B123,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10468,11 +10801,11 @@
         </is>
       </c>
       <c r="E124" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A124,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A124,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F124" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B124,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B124,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10498,11 +10831,11 @@
         </is>
       </c>
       <c r="E125" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A125,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A125,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F125" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B125,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B125,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10528,11 +10861,11 @@
         </is>
       </c>
       <c r="E126" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A126,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A126,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F126" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B126,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B126,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10558,11 +10891,11 @@
         </is>
       </c>
       <c r="E127" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A127,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A127,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F127" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B127,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B127,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10588,11 +10921,11 @@
         </is>
       </c>
       <c r="E128" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A128,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A128,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F128" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B128,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B128,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10618,11 +10951,11 @@
         </is>
       </c>
       <c r="E129" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A129,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A129,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F129" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B129,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B129,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10648,11 +10981,11 @@
         </is>
       </c>
       <c r="E130" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A130,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A130,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F130" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B130,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B130,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10678,11 +11011,11 @@
         </is>
       </c>
       <c r="E131" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A131,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A131,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F131" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B131,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B131,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10708,11 +11041,11 @@
         </is>
       </c>
       <c r="E132" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A132,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A132,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F132" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B132,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B132,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10738,11 +11071,11 @@
         </is>
       </c>
       <c r="E133" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A133,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A133,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F133" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B133,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B133,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10768,11 +11101,11 @@
         </is>
       </c>
       <c r="E134" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A134,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A134,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F134" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B134,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B134,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10798,11 +11131,11 @@
         </is>
       </c>
       <c r="E135" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A135,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A135,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F135" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B135,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B135,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10828,11 +11161,11 @@
         </is>
       </c>
       <c r="E136" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A136,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A136,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F136" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B136,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B136,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10858,11 +11191,11 @@
         </is>
       </c>
       <c r="E137" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A137,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A137,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F137" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B137,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B137,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10888,11 +11221,11 @@
         </is>
       </c>
       <c r="E138" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A138,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A138,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F138" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B138,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B138,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10918,11 +11251,11 @@
         </is>
       </c>
       <c r="E139" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A139,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A139,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F139" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B139,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B139,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10948,11 +11281,11 @@
         </is>
       </c>
       <c r="E140" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A140,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A140,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F140" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B140,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B140,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -10978,11 +11311,11 @@
         </is>
       </c>
       <c r="E141" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A141,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A141,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F141" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B141,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B141,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11008,11 +11341,11 @@
         </is>
       </c>
       <c r="E142" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A142,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A142,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F142" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B142,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B142,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11038,11 +11371,11 @@
         </is>
       </c>
       <c r="E143" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A143,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A143,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F143" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B143,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B143,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11068,11 +11401,11 @@
         </is>
       </c>
       <c r="E144" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A144,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A144,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F144" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B144,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B144,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11098,11 +11431,11 @@
         </is>
       </c>
       <c r="E145" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A145,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A145,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F145" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B145,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B145,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11128,11 +11461,11 @@
         </is>
       </c>
       <c r="E146" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A146,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A146,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F146" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B146,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B146,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11158,11 +11491,11 @@
         </is>
       </c>
       <c r="E147" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A147,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A147,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F147" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B147,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B147,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11188,11 +11521,11 @@
         </is>
       </c>
       <c r="E148" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A148,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A148,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F148" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B148,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B148,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11218,11 +11551,11 @@
         </is>
       </c>
       <c r="E149" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A149,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A149,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F149" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B149,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B149,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11248,11 +11581,11 @@
         </is>
       </c>
       <c r="E150" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A150,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A150,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F150" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B150,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B150,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11278,11 +11611,11 @@
         </is>
       </c>
       <c r="E151" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A151,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A151,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F151" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B151,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B151,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11308,11 +11641,11 @@
         </is>
       </c>
       <c r="E152" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A152,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A152,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F152" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B152,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B152,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11338,11 +11671,11 @@
         </is>
       </c>
       <c r="E153" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A153,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A153,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F153" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B153,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B153,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11368,11 +11701,11 @@
         </is>
       </c>
       <c r="E154" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A154,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A154,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F154" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B154,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B154,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11398,11 +11731,11 @@
         </is>
       </c>
       <c r="E155" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A155,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A155,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F155" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B155,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B155,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11428,11 +11761,11 @@
         </is>
       </c>
       <c r="E156" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A156,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A156,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F156" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B156,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B156,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11458,11 +11791,11 @@
         </is>
       </c>
       <c r="E157" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A157,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A157,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F157" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B157,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B157,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11488,11 +11821,11 @@
         </is>
       </c>
       <c r="E158" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A158,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A158,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F158" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B158,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B158,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11518,11 +11851,11 @@
         </is>
       </c>
       <c r="E159" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A159,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A159,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F159" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B159,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B159,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11548,11 +11881,11 @@
         </is>
       </c>
       <c r="E160" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A160,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A160,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F160" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B160,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B160,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11578,11 +11911,11 @@
         </is>
       </c>
       <c r="E161" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A161,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A161,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F161" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B161,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B161,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11608,11 +11941,11 @@
         </is>
       </c>
       <c r="E162" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A162,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A162,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F162" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B162,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B162,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11638,11 +11971,11 @@
         </is>
       </c>
       <c r="E163" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A163,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A163,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F163" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B163,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B163,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11668,11 +12001,11 @@
         </is>
       </c>
       <c r="E164" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A164,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A164,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F164" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B164,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B164,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11698,11 +12031,11 @@
         </is>
       </c>
       <c r="E165" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A165,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A165,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F165" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B165,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B165,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11728,11 +12061,11 @@
         </is>
       </c>
       <c r="E166" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A166,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A166,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F166" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B166,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B166,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11758,11 +12091,11 @@
         </is>
       </c>
       <c r="E167" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A167,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A167,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F167" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B167,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B167,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11788,11 +12121,11 @@
         </is>
       </c>
       <c r="E168" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A168,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A168,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F168" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B168,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B168,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11818,11 +12151,11 @@
         </is>
       </c>
       <c r="E169" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A169,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A169,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F169" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B169,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B169,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11848,11 +12181,11 @@
         </is>
       </c>
       <c r="E170" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A170,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A170,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F170" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B170,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B170,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11878,11 +12211,11 @@
         </is>
       </c>
       <c r="E171" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A171,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A171,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F171" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B171,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B171,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11908,11 +12241,11 @@
         </is>
       </c>
       <c r="E172" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A172,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A172,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F172" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B172,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B172,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11938,11 +12271,11 @@
         </is>
       </c>
       <c r="E173" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A173,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A173,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F173" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B173,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B173,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11968,11 +12301,11 @@
         </is>
       </c>
       <c r="E174" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A174,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A174,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F174" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B174,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B174,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -11998,11 +12331,11 @@
         </is>
       </c>
       <c r="E175" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A175,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A175,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F175" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B175,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B175,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -12028,11 +12361,11 @@
         </is>
       </c>
       <c r="E176" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A176,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A176,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F176" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B176,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B176,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -12058,11 +12391,11 @@
         </is>
       </c>
       <c r="E177" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A177,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A177,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F177" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B177,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B177,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -12088,11 +12421,11 @@
         </is>
       </c>
       <c r="E178" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A178,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A178,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F178" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B178,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B178,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -12118,11 +12451,11 @@
         </is>
       </c>
       <c r="E179" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A179,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A179,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F179" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B179,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B179,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -12148,11 +12481,11 @@
         </is>
       </c>
       <c r="E180" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A180,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A180,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F180" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B180,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B180,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -12178,11 +12511,11 @@
         </is>
       </c>
       <c r="E181" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A181,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A181,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F181" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B181,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B181,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -12208,11 +12541,491 @@
         </is>
       </c>
       <c r="E182" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(A182,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A182,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
       <c r="F182" s="45">
-        <f>INDEX(Nodes!$B$2:$B$84,MATCH(B182,Nodes!$A$2:$A$84,0))</f>
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B182,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="45" t="inlineStr">
+        <is>
+          <t>willer</t>
+        </is>
+      </c>
+      <c r="B183" s="45" t="inlineStr">
+        <is>
+          <t>cathedral</t>
+        </is>
+      </c>
+      <c r="C183" s="45" t="inlineStr">
+        <is>
+          <t>Criou em jan/2023; sócio com Jorge Barbosa Dias</t>
+        </is>
+      </c>
+      <c r="D183" s="45" t="inlineStr">
+        <is>
+          <t>Documentado</t>
+        </is>
+      </c>
+      <c r="E183" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A183,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F183" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B183,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="45" t="inlineStr">
+        <is>
+          <t>cathedral</t>
+        </is>
+      </c>
+      <c r="B184" s="45" t="inlineStr">
+        <is>
+          <t>bestbet</t>
+        </is>
+      </c>
+      <c r="C184" s="45" t="inlineStr">
+        <is>
+          <t>Única acionista da Rede Loto (nome fantasia Best Bet)</t>
+        </is>
+      </c>
+      <c r="D184" s="45" t="inlineStr">
+        <is>
+          <t>Documentado</t>
+        </is>
+      </c>
+      <c r="E184" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A184,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F184" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B184,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="45" t="inlineStr">
+        <is>
+          <t>cathedral</t>
+        </is>
+      </c>
+      <c r="B185" s="45" t="inlineStr">
+        <is>
+          <t>alcazar</t>
+        </is>
+      </c>
+      <c r="C185" s="45" t="inlineStr">
+        <is>
+          <t>Mesmo dono, administrador e endereço no Funchal; auditor ouvido pela piauí vê possível financiamento</t>
+        </is>
+      </c>
+      <c r="D185" s="45" t="inlineStr">
+        <is>
+          <t>Alegado ou contestado</t>
+        </is>
+      </c>
+      <c r="E185" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A185,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F185" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B185,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="45" t="inlineStr">
+        <is>
+          <t>flavio</t>
+        </is>
+      </c>
+      <c r="B186" s="45" t="inlineStr">
+        <is>
+          <t>bestbet</t>
+        </is>
+      </c>
+      <c r="C186" s="45" t="inlineStr">
+        <is>
+          <t>piauí/PF: possível sócio oculto, via acesso à conta da Alcazar; ele e Willer negam</t>
+        </is>
+      </c>
+      <c r="D186" s="45" t="inlineStr">
+        <is>
+          <t>Alegado ou contestado</t>
+        </is>
+      </c>
+      <c r="E186" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A186,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F186" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B186,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="45" t="inlineStr">
+        <is>
+          <t>loterj</t>
+        </is>
+      </c>
+      <c r="B187" s="45" t="inlineStr">
+        <is>
+          <t>bestbet</t>
+        </is>
+      </c>
+      <c r="C187" s="45" t="inlineStr">
+        <is>
+          <t>Licença de mai/2023</t>
+        </is>
+      </c>
+      <c r="D187" s="45" t="inlineStr">
+        <is>
+          <t>Documentado</t>
+        </is>
+      </c>
+      <c r="E187" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A187,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F187" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B187,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="45" t="inlineStr">
+        <is>
+          <t>cancado</t>
+        </is>
+      </c>
+      <c r="B188" s="45" t="inlineStr">
+        <is>
+          <t>bestbet</t>
+        </is>
+      </c>
+      <c r="C188" s="45" t="inlineStr">
+        <is>
+          <t>Assinou a licença como presidente da Loterj</t>
+        </is>
+      </c>
+      <c r="D188" s="45" t="inlineStr">
+        <is>
+          <t>Documentado</t>
+        </is>
+      </c>
+      <c r="E188" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A188,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F188" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B188,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="45" t="inlineStr">
+        <is>
+          <t>flavio</t>
+        </is>
+      </c>
+      <c r="B189" s="45" t="inlineStr">
+        <is>
+          <t>cancado</t>
+        </is>
+      </c>
+      <c r="C189" s="45" t="inlineStr">
+        <is>
+          <t>Teria indicado à presidência da Loterj (Folha)</t>
+        </is>
+      </c>
+      <c r="D189" s="45" t="inlineStr">
+        <is>
+          <t>Alegado ou contestado</t>
+        </is>
+      </c>
+      <c r="E189" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A189,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F189" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B189,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="45" t="inlineStr">
+        <is>
+          <t>castro</t>
+        </is>
+      </c>
+      <c r="B190" s="45" t="inlineStr">
+        <is>
+          <t>loterj</t>
+        </is>
+      </c>
+      <c r="C190" s="45" t="inlineStr">
+        <is>
+          <t>Loteria do governo dele; contratos de 2023</t>
+        </is>
+      </c>
+      <c r="D190" s="45" t="inlineStr">
+        <is>
+          <t>Documentado</t>
+        </is>
+      </c>
+      <c r="E190" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A190,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F190" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B190,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="45" t="inlineStr">
+        <is>
+          <t>cathedral</t>
+        </is>
+      </c>
+      <c r="B191" s="45" t="inlineStr">
+        <is>
+          <t>flavio</t>
+        </is>
+      </c>
+      <c r="C191" s="45" t="inlineStr">
+        <is>
+          <t>PF: canhotos de voos Lisboa–Nice e Cascais–Nice–Paris (2025) em nome da empresa; a defesa diz que Willer pagou e que eram passeios entre famílias</t>
+        </is>
+      </c>
+      <c r="D191" s="45" t="inlineStr">
+        <is>
+          <t>Alegado ou contestado</t>
+        </is>
+      </c>
+      <c r="E191" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A191,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F191" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B191,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="45" t="inlineStr">
+        <is>
+          <t>willer</t>
+        </is>
+      </c>
+      <c r="B192" s="45" t="inlineStr">
+        <is>
+          <t>riopag</t>
+        </is>
+      </c>
+      <c r="C192" s="45" t="inlineStr">
+        <is>
+          <t>E-mail achado pela PF: se apresentou como sócio; antes negava, depois admitiu participação indireta (O Globo)</t>
+        </is>
+      </c>
+      <c r="D192" s="45" t="inlineStr">
+        <is>
+          <t>Documentado</t>
+        </is>
+      </c>
+      <c r="E192" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A192,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F192" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B192,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="45" t="inlineStr">
+        <is>
+          <t>loterj</t>
+        </is>
+      </c>
+      <c r="B193" s="45" t="inlineStr">
+        <is>
+          <t>riopag</t>
+        </is>
+      </c>
+      <c r="C193" s="45" t="inlineStr">
+        <is>
+          <t>Contratou em 2023; o estado rescindiu e cobra ~R$ 4 mi, a empresa contesta</t>
+        </is>
+      </c>
+      <c r="D193" s="45" t="inlineStr">
+        <is>
+          <t>Documentado</t>
+        </is>
+      </c>
+      <c r="E193" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A193,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F193" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B193,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="45" t="inlineStr">
+        <is>
+          <t>willer</t>
+        </is>
+      </c>
+      <c r="B194" s="45" t="inlineStr">
+        <is>
+          <t>hangar</t>
+        </is>
+      </c>
+      <c r="C194" s="45" t="inlineStr">
+        <is>
+          <t>Ocupados por duas empresas de aviação dele</t>
+        </is>
+      </c>
+      <c r="D194" s="45" t="inlineStr">
+        <is>
+          <t>Documentado</t>
+        </is>
+      </c>
+      <c r="E194" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A194,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F194" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B194,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="45" t="inlineStr">
+        <is>
+          <t>pf</t>
+        </is>
+      </c>
+      <c r="B195" s="45" t="inlineStr">
+        <is>
+          <t>hangar</t>
+        </is>
+      </c>
+      <c r="C195" s="45" t="inlineStr">
+        <is>
+          <t>Busca em ago/2026: sala oculta, máquina de contar e malas vazias, sem dinheiro (Estadão); Willer nega uso irregular</t>
+        </is>
+      </c>
+      <c r="D195" s="45" t="inlineStr">
+        <is>
+          <t>Alegado ou contestado</t>
+        </is>
+      </c>
+      <c r="E195" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A195,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F195" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B195,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="45" t="inlineStr">
+        <is>
+          <t>pf</t>
+        </is>
+      </c>
+      <c r="B196" s="45" t="inlineStr">
+        <is>
+          <t>weverton</t>
+        </is>
+      </c>
+      <c r="C196" s="45" t="inlineStr">
+        <is>
+          <t>Operação Sem Desconto (04/08/2026), autorizada por Mendonça</t>
+        </is>
+      </c>
+      <c r="D196" s="45" t="inlineStr">
+        <is>
+          <t>Documentado</t>
+        </is>
+      </c>
+      <c r="E196" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A196,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F196" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B196,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="45" t="inlineStr">
+        <is>
+          <t>willer</t>
+        </is>
+      </c>
+      <c r="B197" s="45" t="inlineStr">
+        <is>
+          <t>weverton</t>
+        </is>
+      </c>
+      <c r="C197" s="45" t="inlineStr">
+        <is>
+          <t>PF: a estrutura dele era “hub financeiro” do senador; a mulher do senador recebeu R$ 11 mi de empresas dele. Ambos negam</t>
+        </is>
+      </c>
+      <c r="D197" s="45" t="inlineStr">
+        <is>
+          <t>Alegado ou contestado</t>
+        </is>
+      </c>
+      <c r="E197" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A197,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F197" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B197,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="45" t="inlineStr">
+        <is>
+          <t>weverton</t>
+        </is>
+      </c>
+      <c r="B198" s="45" t="inlineStr">
+        <is>
+          <t>wt</t>
+        </is>
+      </c>
+      <c r="C198" s="45" t="inlineStr">
+        <is>
+          <t>PF: mora em casa de R$ 6 mi registrada na WT; Willer diz que é negócio regular da imobiliária</t>
+        </is>
+      </c>
+      <c r="D198" s="45" t="inlineStr">
+        <is>
+          <t>Alegado ou contestado</t>
+        </is>
+      </c>
+      <c r="E198" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(A198,Nodes!$A$2:$A$91,0))</f>
+        <v/>
+      </c>
+      <c r="F198" s="45">
+        <f>INDEX(Nodes!$B$2:$B$91,MATCH(B198,Nodes!$A$2:$A$91,0))</f>
         <v/>
       </c>
     </row>
@@ -12230,7 +13043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="110" customWidth="1" style="24" min="1" max="1"/>
@@ -12335,9 +13148,16 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>Checagem final (21/10/2026): 111 links testados (91 abrem; 19 bloqueiam robôs, como UOL, Intercept e Folha; 1 link da CNN quebrado foi trocado por Mais Goiás). Conferidas contra a fonte 22 matérias das conexões mais sensíveis. Corrigidos: Zettel foi o 2º doador de Jair, não o maior; o advogado morto em 2024 representava a WT, não Richarlison; a posse de Willer reconhecida pelo STJ não foi confirmada; Mendonça teve uma reunião reservada confirmada (14/03/2025), não duas; o voo de Marçal foi pago pela Prime You (R$ 1,17 mi). Respostas dos citados foram adicionadas (Flávio sobre o BRB e a emenda, Ciro, Faria, Marçal, Gaspar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada a partir do UOL News (Dani Lima, 21/10). Entraram só itens com reportagem escrita: Best Bet/Cathedral (piauí), voos pagos pela Cathedral (Folha), Rio Pag (O Globo), sala no hangar (Estadão) e Operação Sem Desconto (Poder360, O Povo). Ficaram de fora, sem texto publicado: a festa no hangar em 2024 com Flávio e Valdemar, as tratativas da indicação de Nunes no rancho de Willer e a origem em loja de informática em Taguatinga. O comunicado de relatores da ONU sobre a Meta, no mesmo vídeo, não tem relação com o mapa.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Incorpora logos do Santander e do Banco Master; atualiza README
Traz para o main os dois commits que estavam só no clone local da Isis
(267ef81, 1ac7153), refeitos sobre a planilha atual para evitar conflito
no xlsx. README passa a citar o acervo a verdade. e as reportagens.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011rQv2fzfb4Xj3f3AYjm2Yf
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -971,7 +971,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="25">
       <c r="A4" s="28" t="inlineStr">
         <is>
@@ -1080,23 +1079,6 @@
         <v/>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
     <row r="28" ht="15" customHeight="1" s="25">
       <c r="A28" s="35" t="inlineStr">
         <is>
@@ -4436,17 +4418,17 @@
       </c>
       <c r="G16" s="24" t="inlineStr">
         <is>
-          <t>santander.jpg</t>
+          <t>santander.png</t>
         </is>
       </c>
       <c r="H16" s="24" t="inlineStr">
         <is>
-          <t>Simplus Menegati · CC BY-SA 4.0</t>
+          <t>Interbrand · domínio público (logo simples, sem direito autoral)</t>
         </is>
       </c>
       <c r="I16" s="24" t="inlineStr">
         <is>
-          <t>https://commons.wikimedia.org/wiki/File:Agencia_Banco_Santander_de_Telemaco_Borba.jpg</t>
+          <t>https://commons.wikimedia.org/wiki/File:Banco_Santander_Logotipo.svg</t>
         </is>
       </c>
       <c r="J16" s="24" t="inlineStr"/>
@@ -4908,9 +4890,21 @@
         <f>COUNTIF(Edges!$A$2:$A$198,A30)+COUNTIF(Edges!$B$2:$B$198,A30)</f>
         <v/>
       </c>
-      <c r="G30" s="24" t="n"/>
-      <c r="H30" s="24" t="n"/>
-      <c r="I30" s="24" t="n"/>
+      <c r="G30" s="24" t="inlineStr">
+        <is>
+          <t>master.png</t>
+        </is>
+      </c>
+      <c r="H30" s="24" t="inlineStr">
+        <is>
+          <t>Banco Master · domínio público (logo simples, sem direito autoral)</t>
+        </is>
+      </c>
+      <c r="I30" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Logotipo_do_Banco_Master.svg</t>
+        </is>
+      </c>
       <c r="J30" s="24" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
@@ -13155,7 +13149,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>22/10/2026: rodada a partir do UOL News (Dani Lima, 21/10). Entraram só itens com reportagem escrita: Best Bet/Cathedral (piauí), voos pagos pela Cathedral (Folha), Rio Pag (O Globo), sala no hangar (Estadão) e Operação Sem Desconto (Poder360, O Povo). Ficaram de fora, sem texto publicado: a festa no hangar em 2024 com Flávio e Valdemar, as tratativas da indicação de Nunes no rancho de Willer e a origem em loja de informática em Taguatinga. O comunicado de relatores da ONU sobre a Meta, no mesmo vídeo, não tem relação com o mapa.</t>
         </is>

</xml_diff>

<commit_message>
Redesign C: regiões por grupo, linhas recuadas e nomes por zoom
- Cada grupo vira uma região num anel; a ordem garante que regiões
  vizinhas tenham cores distinguíveis (validado para daltonismo).
- 'Poder e Justiça' dividido em 'Justiça e investigação' (violeta) e
  'Política e governo' (verde).
- Linhas recuadas por padrão; as que cruzam grupos ficam mais claras.
  Hover e seleção continuam destacando.
- Visão geral mostra só nomes com 5+ conexões; aproximar revela o resto.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011rQv2fzfb4Xj3f3AYjm2Yf
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -3021,7 +3021,7 @@
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="D26" s="37" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="C27" s="37" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="D27" s="37" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="C28" s="37" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="D28" s="37" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="C29" s="37" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="D29" s="37" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="C30" s="37" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="D30" s="37" t="inlineStr">
@@ -3416,7 +3416,7 @@
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="D31" s="37" t="inlineStr">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="C32" s="37" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="D32" s="37" t="inlineStr">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="C36" s="37" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="D36" s="37" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="D45" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E45" s="45" t="inlineStr">
@@ -5418,7 +5418,7 @@
       </c>
       <c r="D46" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E46" s="45" t="inlineStr">
@@ -5449,7 +5449,7 @@
       </c>
       <c r="D47" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E47" s="45" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="D48" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E48" s="45" t="inlineStr">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="D49" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E49" s="45" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="D50" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E50" s="45" t="inlineStr">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="D51" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E51" s="45" t="inlineStr">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="D52" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E52" s="45" t="inlineStr">
@@ -5655,7 +5655,7 @@
       </c>
       <c r="D53" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E53" s="45" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="D54" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E54" s="45" t="inlineStr">
@@ -5749,7 +5749,7 @@
       </c>
       <c r="D55" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E55" s="45" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="D56" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E56" s="45" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="D57" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E57" s="45" t="inlineStr">
@@ -5874,7 +5874,7 @@
       </c>
       <c r="D58" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E58" s="45" t="inlineStr">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="D59" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E59" s="45" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="D60" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E60" s="45" t="inlineStr">
@@ -6026,7 +6026,7 @@
       </c>
       <c r="D62" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E62" s="45" t="inlineStr">
@@ -6061,7 +6061,7 @@
       </c>
       <c r="D63" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E63" s="45" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="D64" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E64" s="45" t="inlineStr">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="D65" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E65" s="45" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D66" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E66" s="45" t="inlineStr">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="D67" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Justiça e investigação</t>
         </is>
       </c>
       <c r="E67" s="45" t="inlineStr">
@@ -6376,7 +6376,7 @@
       </c>
       <c r="D72" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E72" s="45" t="inlineStr">
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D88" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E88" s="45" t="inlineStr">
@@ -6971,7 +6971,7 @@
       </c>
       <c r="D89" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E89" s="45" t="inlineStr">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="D91" s="45" t="inlineStr">
         <is>
-          <t>Poder e Justiça</t>
+          <t>Política e governo</t>
         </is>
       </c>
       <c r="E91" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Rodada contexto e imagens: 55 perfis novos, 15 imagens, rótulos para não-pessoas, Allure Eventos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018rccqzzxrj3q4wcvp7v91m
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -1150,7 +1150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P91"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3548,12 +3548,24 @@
       </c>
       <c r="M32" s="37" t="inlineStr">
         <is>
-          <t>21/10/2026: importado do acervo a verdade. (bolsomaster.site) (perfil novo).</t>
-        </is>
-      </c>
-      <c r="N32" s="24" t="n"/>
-      <c r="O32" s="24" t="n"/>
-      <c r="P32" s="24" t="n"/>
+          <t>21/10/2026: importado do acervo a verdade. (bolsomaster.site) (perfil novo). 22/10/2026: foto adicionada.</t>
+        </is>
+      </c>
+      <c r="N32" s="24" t="inlineStr">
+        <is>
+          <t>mendonca.jpg</t>
+        </is>
+      </c>
+      <c r="O32" s="24" t="inlineStr">
+        <is>
+          <t>Luis Macedo/Câmara dos Deputados · CC BY 3.0</t>
+        </is>
+      </c>
+      <c r="P32" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Andr%C3%A9_Luiz_de_Almeida_Mendon%C3%A7a_(cropped).jpg</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="37" t="inlineStr">
@@ -3618,12 +3630,24 @@
       </c>
       <c r="M33" s="37" t="inlineStr">
         <is>
-          <t>21/10/2026: importado do acervo a verdade. (bolsomaster.site) (perfil novo).</t>
-        </is>
-      </c>
-      <c r="N33" s="24" t="n"/>
-      <c r="O33" s="24" t="n"/>
-      <c r="P33" s="24" t="n"/>
+          <t>21/10/2026: importado do acervo a verdade. (bolsomaster.site) (perfil novo). 22/10/2026: foto adicionada.</t>
+        </is>
+      </c>
+      <c r="N33" s="24" t="inlineStr">
+        <is>
+          <t>faria.jpg</t>
+        </is>
+      </c>
+      <c r="O33" s="24" t="inlineStr">
+        <is>
+          <t>Luis Macedo/Câmara dos Deputados · CC BY 3.0</t>
+        </is>
+      </c>
+      <c r="P33" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:F%C3%A1bio_Faria_(cropped).jpg</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="37" t="inlineStr">
@@ -3688,12 +3712,24 @@
       </c>
       <c r="M34" s="37" t="inlineStr">
         <is>
-          <t>21/10/2026: importado do acervo a verdade. (bolsomaster.site) (perfil novo).</t>
-        </is>
-      </c>
-      <c r="N34" s="24" t="n"/>
-      <c r="O34" s="24" t="n"/>
-      <c r="P34" s="24" t="n"/>
+          <t>21/10/2026: importado do acervo a verdade. (bolsomaster.site) (perfil novo). 22/10/2026: foto adicionada.</t>
+        </is>
+      </c>
+      <c r="N34" s="24" t="inlineStr">
+        <is>
+          <t>frias.jpg</t>
+        </is>
+      </c>
+      <c r="O34" s="24" t="inlineStr">
+        <is>
+          <t>Isac Nóbrega/PR · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="P34" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:M%C3%A1rio_Frias_em_2020.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="37" t="inlineStr">
@@ -3758,12 +3794,24 @@
       </c>
       <c r="M35" s="37" t="inlineStr">
         <is>
-          <t>21/10/2026: importado do acervo a verdade. (bolsomaster.site) (perfil novo).</t>
-        </is>
-      </c>
-      <c r="N35" s="24" t="n"/>
-      <c r="O35" s="24" t="n"/>
-      <c r="P35" s="24" t="n"/>
+          <t>21/10/2026: importado do acervo a verdade. (bolsomaster.site) (perfil novo). 22/10/2026: foto adicionada.</t>
+        </is>
+      </c>
+      <c r="N35" s="24" t="inlineStr">
+        <is>
+          <t>gaspar.jpg</t>
+        </is>
+      </c>
+      <c r="O35" s="24" t="inlineStr">
+        <is>
+          <t>Kayo Magalhães/Câmara dos Deputados · CC BY 3.0</t>
+        </is>
+      </c>
+      <c r="P35" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Alfredo_Gaspar_Deputado_Federal_(cropped).jpg</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="37" t="inlineStr">
@@ -3828,12 +3876,4009 @@
       </c>
       <c r="M36" s="37" t="inlineStr">
         <is>
-          <t>22/10/2026: rodada UOL News (bets, Loterj, hangar, Weverton). Perfil novo.</t>
-        </is>
-      </c>
-      <c r="N36" s="24" t="n"/>
-      <c r="O36" s="24" t="n"/>
-      <c r="P36" s="24" t="n"/>
+          <t>22/10/2026: rodada UOL News (bets, Loterj, hangar, Weverton). Perfil novo. 22/10/2026: foto adicionada.</t>
+        </is>
+      </c>
+      <c r="N36" s="24" t="inlineStr">
+        <is>
+          <t>weverton.jpg</t>
+        </is>
+      </c>
+      <c r="O36" s="24" t="inlineStr">
+        <is>
+          <t>Rodrigo Viana/Senado Federal · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="P36" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Senadores_da_56%C2%AA_Legislatura_-_Weverton_Rocha_(32121443327).jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>pf</t>
+        </is>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>Polícia Federal</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>Polícia judiciária da União. Conduz as duas frentes centrais do mapa: a Operação Compliance Zero (Banco Master; prendeu Daniel Vorcaro em 17/11/2025 e teve várias fases em 2026) e a Operação Sem Desconto (descontos ilegais em aposentadorias do INSS; deflagrada com a CGU em abr/2025, com nova fase em 04/08/2026 contra Willer Tomaz e familiares de Weverton Rocha). Em out/2026 enviou ao STF um segundo inquérito sobre Flávio Bolsonaro, por suspeita de lavagem ligada a Willer.</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>Sede em Brasília (DF); atuação nacional</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="24" t="inlineStr">
+        <is>
+          <t>Em 08/09/2026 o ministro André Mendonça afastou o diretor-geral Andrei Rodrigues e o diretor de Inteligência, sem ouvir a PGR; a AGU contestou a decisão.</t>
+        </is>
+      </c>
+      <c r="H37" s="24" t="inlineStr">
+        <is>
+          <t>Órgão público</t>
+        </is>
+      </c>
+      <c r="I37" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J37" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="inlineStr">
+        <is>
+          <t>Entenda a operação que prendeu Vorcaro (cnnbrasil.com.br) https://www.cnnbrasil.com.br/economia/mercado/entenda-operacao-que-prendeu-daniel-vorcaro-dono-do-banco-master/ | Nova fase da Sem Desconto mira Weverton e Willer (congressoemfoco.com.br) https://www.congressoemfoco.com.br/noticia/120986/fraudes-no-inss-pf-mira-weverton-rocha-e-advogado-willer-tomaz | Afastamento do diretor-geral da PF (cnnbrasil.com.br) https://www.cnnbrasil.com.br/blogs/teo-cury/politica/mendonca-ordenou-afastamento-de-diretor-geral-da-pf-sem-ouvir-pgr/ | Segundo inquérito contra Flávio no STF (oliberal.com) https://www.oliberal.com/politica/flavio-e-investigado-em-2-inquerito-no-stf-para-apurar-suspeitas-de-lavagem-com-advogado-1.1183991</t>
+        </is>
+      </c>
+      <c r="L37" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M37" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N37" s="24" t="inlineStr">
+        <is>
+          <t>pf.jpg</t>
+        </is>
+      </c>
+      <c r="O37" s="24" t="inlineStr">
+        <is>
+          <t>Agência Senado · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="P37" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Sede_da_Pol%C3%ADcia_Federal_(52830107256).jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>angra</t>
+        </is>
+      </c>
+      <c r="B38" s="24" t="inlineStr">
+        <is>
+          <t>Mansão em Angra dos Reis</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="inlineStr">
+        <is>
+          <t>Casas e ativos</t>
+        </is>
+      </c>
+      <c r="D38" s="24" t="inlineStr">
+        <is>
+          <t>Mansão na Ilha Comprida, em Angra dos Reis, avaliada em cerca de R$ 10 mi. Foi comprada em 2020 pela empresa de Richarlison e de seu empresário; em 2022 a posse foi transferida na Justiça à WT Administração de Imóveis, de Willer Tomaz, que diz ter pago pendências da antiga dona (M Locadora) por sub-rogação. O processo terminou em 2025, favorável a Willer. A Prime You, de que Vorcaro era sócio, administrou o imóvel, e Flávio fez lá o aniversário da filha.</t>
+        </is>
+      </c>
+      <c r="E38" s="24" t="inlineStr">
+        <is>
+          <t>Ilha Comprida, Angra dos Reis (RJ)</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="24" t="inlineStr">
+        <is>
+          <t>Disputa civil encerrada em favor da WT. Em out/2026 Richarlison pediu à PF que investigue o caso; não há inquérito específico sobre o imóvel nas fontes.</t>
+        </is>
+      </c>
+      <c r="H38" s="24" t="inlineStr">
+        <is>
+          <t>Bem citado</t>
+        </is>
+      </c>
+      <c r="I38" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J38" s="24" t="inlineStr">
+        <is>
+          <t>Flávio diz não ter relação com o imóvel e chamou a associação de "factualmente infundada e eleitoralmente motivada". Willer chama os antigos ocupantes de "invasores".</t>
+        </is>
+      </c>
+      <c r="K38" s="24" t="inlineStr">
+        <is>
+          <t>Richarlison disputa imóvel com amigo de Flávio (poder360.com.br) https://www.poder360.com.br/justica/richarlison-briga-na-justica-com-amigo-de-flavio-bolsonaro/ | Richarlison pede apuração à PF (sbtnews.sbt.com.br) https://sbtnews.sbt.com.br/noticia/brasil/richarlison-apuracao-pf-disputa-ilha-flavio-bolsonaro | Empresas e imóveis em nome de Lídia Mazelli (iclnoticias.com.br) https://iclnoticias.com.br/domestica-preside-empresas-fraude-flavio/</t>
+        </is>
+      </c>
+      <c r="L38" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M38" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>master</t>
+        </is>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>Banco Master</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>Vorcaro e o Banco Master</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>Banco de Daniel Vorcaro. Cresceu vendendo CDBs com rendimento acima do mercado, apoiados na garantia do FGC. O Banco Central decretou a liquidação extrajudicial em 18/11/2025, no dia da Operação Compliance Zero (Vorcaro foi preso na noite anterior, em Guarulhos), que apura gestão fraudulenta e venda de carteiras de crédito sem lastro. O BRB, banco público do DF, pôs cerca de R$ 12 bi no Master comprando carteiras que a investigação aponta como fraudulentas.</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="24" t="inlineStr">
+        <is>
+          <t>Em liquidação extrajudicial pelo BC desde nov/2025. Ex-dirigentes investigados no STF (relator André Mendonça); Vorcaro preso.</t>
+        </is>
+      </c>
+      <c r="H39" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I39" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J39" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>Banco Master tem liquidação decretada (bloomberglinea.com.br) https://www.bloomberglinea.com.br/negocios/banco-master-tem-liquidacao-decretada-e-daniel-vorcaro-e-preso-pela-policia-federal/ | Entenda a operação que prendeu Vorcaro (cnnbrasil.com.br) https://www.cnnbrasil.com.br/economia/mercado/entenda-operacao-que-prendeu-daniel-vorcaro-dono-do-banco-master/ | PF prende ex-presidente do BRB (timesbrasil.com.br) https://timesbrasil.com.br/brasil/operacoes-da-pf/pf-prende-paulo-henrique-costa-ex-presidente-do-brb-em-nova-fase-da-compliance-zero/</t>
+        </is>
+      </c>
+      <c r="L39" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M39" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N39" s="24" t="inlineStr">
+        <is>
+          <t>master.png</t>
+        </is>
+      </c>
+      <c r="O39" s="24" t="inlineStr">
+        <is>
+          <t>Banco Master · domínio público (logo simples, sem direito autoral)</t>
+        </is>
+      </c>
+      <c r="P39" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Logotipo_do_Banco_Master.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
+          <t>coaf</t>
+        </is>
+      </c>
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>Caso rachadinha / COAF</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>Investigação do MP-RJ sobre devolução de salários ("rachadinha") no gabinete de Flávio na Alerj. Começou com relatório do Coaf de 2018 que apontou R$ 1,2 mi em movimentações atípicas de Fabrício Queiroz. Em nov/2020 Flávio foi denunciado por peculato, lavagem e organização criminosa (desvio estimado em cerca de R$ 6 mi). O STJ anulou quebras de sigilo em fev/2021, e em 30/11/2021 a Segunda Turma do STF anulou quatro relatórios do Coaf (3 a 1, com voto de Nunes Marques).</t>
+        </is>
+      </c>
+      <c r="E40" s="24" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="24" t="inlineStr">
+        <is>
+          <t>Com as anulações, a denúncia original ficou sem efeito e o caso voltou praticamente à estaca zero. Flávio sempre negou irregularidades.</t>
+        </is>
+      </c>
+      <c r="H40" s="24" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+      <c r="I40" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J40" s="24" t="inlineStr">
+        <is>
+          <t>O primeiro relatório do Coaf, sobre Queiroz, foi mantido; os anulados são os posteriores.</t>
+        </is>
+      </c>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>STF anula 4 relatórios do Coaf (poder360.com.br) https://www.poder360.com.br/justica/stf-anula-4-relatorios-do-coaf-que-miravam-flavio-no-caso-das-rachadinhas/ | Segunda Turma anula provas contra Flávio (correiobraziliense.com.br) https://www.correiobraziliense.com.br/politica/2021/11/4967209-segunda-turma-anula-provas-contra-flavio-bolsonaro-no-inquerito-das-rachadinhas.html</t>
+        </is>
+      </c>
+      <c r="L40" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M40" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>jato</t>
+        </is>
+      </c>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>Jato (3 cotistas)</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="inlineStr">
+        <is>
+          <t>Casas e ativos</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>Embraer Legacy 650, prefixo PP-NLR, dividido em três cotas: Alcazar Holdings (de Willer Tomaz), Prime You (de que Vorcaro era sócio) e Laerte Cosentino. Flávio voou nele com Willer em jan/2025, entre Brasília e a Flórida, segundo a piauí. Segundo O Globo, Alexandre de Moraes e a esposa também desembarcaram desse jato em ago/2025.</t>
+        </is>
+      </c>
+      <c r="E41" s="24" t="inlineStr">
+        <is>
+          <t>Base no Brasil (DF/SP)</t>
+        </is>
+      </c>
+      <c r="F41" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="24" t="inlineStr">
+        <is>
+          <t>O jato aparece em inquéritos da PF sobre Willer e Flávio; não há processo sobre a aeronave em si.</t>
+        </is>
+      </c>
+      <c r="H41" s="24" t="inlineStr">
+        <is>
+          <t>Bem citado</t>
+        </is>
+      </c>
+      <c r="I41" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J41" s="24" t="inlineStr">
+        <is>
+          <t>As fontes divergem sobre o registro: uma cita a Fraction 024 Administração de Bem Próprio, outra a Prime Aviation. Flávio diz que voou de carona, por amizade; Willer diz que não sabia que a Prime You era de Vorcaro.</t>
+        </is>
+      </c>
+      <c r="K41" s="24" t="inlineStr">
+        <is>
+          <t>Flávio era usuário master de conta de offshore sócia do jato (maisgoias.com.br) https://www.maisgoias.com.br/brasil/flavio-bolsonaro-era-usuario-master-de-conta-de-offshore-socia-do-jato-usado-por-vorcaro/ | Moraes flagrado desembarcando do PP-NLR (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/09/11724483-alexandre-de-moraes-foi-flagrado-desembarcando-de-jatinho-de-vorcaro.html</t>
+        </is>
+      </c>
+      <c r="L41" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M41" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="24" t="inlineStr">
+        <is>
+          <t>primeu</t>
+        </is>
+      </c>
+      <c r="B42" s="24" t="inlineStr">
+        <is>
+          <t>Prime U</t>
+        </is>
+      </c>
+      <c r="C42" s="24" t="inlineStr">
+        <is>
+          <t>Vorcaro e o Banco Master</t>
+        </is>
+      </c>
+      <c r="D42" s="24" t="inlineStr">
+        <is>
+          <t>Prime You: empresa de compartilhamento e gestão de bens de alto padrão (cotas de aviões, barcos, casas e carros). Vorcaro foi sócio até set/2025, quando a participação passou a um fundo. Administra mansões, um hotel em Campos do Jordão e jatos; era cotista do jato usado por Flávio e administrou a mansão de Angra. Segundo o Valor, pagou em 2025 um voo de R$ 1,17 mi usado por Pablo Marçal.</t>
+        </is>
+      </c>
+      <c r="E42" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F42" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G42" s="24" t="inlineStr">
+        <is>
+          <t>Sem acusação formal contra a empresa nas fontes.</t>
+        </is>
+      </c>
+      <c r="H42" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I42" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J42" s="24" t="inlineStr">
+        <is>
+          <t>A empresa diz que administrar um bem "não implica necessariamente propriedade direta" de Vorcaro.</t>
+        </is>
+      </c>
+      <c r="K42" s="24" t="inlineStr">
+        <is>
+          <t>Mansões, hotel e jatos administrados pela Prime You (jornalgrandebahia.com.br) https://jornalgrandebahia.com.br/2026/03/ex-banqueiro-daniel-vorcaro-tem-mansoes-hotel-de-luxo-e-jatos-administrados-pela-prime-you-empresa-da-qual-foi-socio/ | Empresa de Vorcaro pagou voo de Marçal (gp1.com.br) https://www.gp1.com.br/brasil/noticia/2026/10/2/empresa-ligada-a-daniel-vorcaro-pagou-voo-de-r-117-milhao-usado-por-pablo-marcal-633016.html</t>
+        </is>
+      </c>
+      <c r="L42" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M42" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="24" t="inlineStr">
+        <is>
+          <t>alcazar</t>
+        </is>
+      </c>
+      <c r="B43" s="24" t="inlineStr">
+        <is>
+          <t>Alcazar Holdings</t>
+        </is>
+      </c>
+      <c r="C43" s="24" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="D43" s="24" t="inlineStr">
+        <is>
+          <t>Offshore registrada na Ilha da Madeira (Portugal) em 2023, que tem Willer Tomaz como único sócio. É cotista do jato PP-NLR e tinha conta no Santander em que, segundo a PF, Flávio aparecia como "usuário master"; a conta teria movimentado cerca de R$ 130 mi entre mar e mai/2025. Divide dono, administrador e endereço no Funchal com a Cathedral Holdings, dona da Best Bet.</t>
+        </is>
+      </c>
+      <c r="E43" s="24" t="inlineStr">
+        <is>
+          <t>Funchal, Ilha da Madeira (Portugal)</t>
+        </is>
+      </c>
+      <c r="F43" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G43" s="24" t="inlineStr">
+        <is>
+          <t>Citada no inquérito da PF enviado ao STF em out/2026 (relator Alexandre de Moraes) sobre suspeita de lavagem envolvendo Flávio e Willer.</t>
+        </is>
+      </c>
+      <c r="H43" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I43" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J43" s="24" t="inlineStr">
+        <is>
+          <t>Willer atribui o vínculo de Flávio à conta a um erro cadastral do Santander, já corrigido. Flávio nega ter tido conta com Willer.</t>
+        </is>
+      </c>
+      <c r="K43" s="24" t="inlineStr">
+        <is>
+          <t>Flávio era usuário master de conta de offshore (maisgoias.com.br) https://www.maisgoias.com.br/brasil/flavio-bolsonaro-era-usuario-master-de-conta-de-offshore-socia-do-jato-usado-por-vorcaro/ | Offshore ligada a Flávio e o mercado de bets (jornalopcao.com.br) https://www.jornalopcao.com.br/ultimas-noticias/offshore-ligada-a-flavio-bolsonaro-reune-conexoes-com-o-mercado-de-bets-879306/ | Segundo inquérito contra Flávio no STF (oliberal.com) https://www.oliberal.com/politica/flavio-e-investigado-em-2-inquerito-no-stf-para-apurar-suspeitas-de-lavagem-com-advogado-1.1183991</t>
+        </is>
+      </c>
+      <c r="L43" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M43" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="24" t="inlineStr">
+        <is>
+          <t>wt</t>
+        </is>
+      </c>
+      <c r="B44" s="24" t="inlineStr">
+        <is>
+          <t>WT (e outras 13 empresas)</t>
+        </is>
+      </c>
+      <c r="C44" s="24" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="D44" s="24" t="inlineStr">
+        <is>
+          <t>WT Administração de Imóveis e Bens, empresa de Willer Tomaz. Ficou com a mansão de Angra e comprou de Fabiano Zettel um apartamento em SP. É uma de cerca de 14 empresas ligadas a Willer (Jet Line, Ícaro Aviation, Friponor, RioPag/Capital Pretium, Alcazar etc.) que tiveram Lídia Mazelli como diretora; a WT até jul/2024. A PF diz que Weverton Rocha mora numa casa de R$ 6 mi registrada na WT.</t>
+        </is>
+      </c>
+      <c r="E44" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F44" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="24" t="inlineStr">
+        <is>
+          <t>Citada na Operação Sem Desconto (ago/2026). Willer diz que os negócios da imobiliária são regulares.</t>
+        </is>
+      </c>
+      <c r="H44" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I44" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J44" s="24" t="inlineStr">
+        <is>
+          <t>A reportagem do ICL fala em 14 empresas, mas nomeia 13.</t>
+        </is>
+      </c>
+      <c r="K44" s="24" t="inlineStr">
+        <is>
+          <t>Doméstica preside no papel empresas de Willer (iclnoticias.com.br) https://iclnoticias.com.br/domestica-preside-empresas-fraude-flavio/ | Apartamento usado por Flávio foi vendido à WT (diariodocomercio.com.br) https://diariodocomercio.com.br/politica/flavio-bolsonaro-apartamento-pf/ | Nova fase da Sem Desconto (congressoemfoco.com.br) https://www.congressoemfoco.com.br/noticia/120986/fraudes-no-inss-pf-mira-weverton-rocha-e-advogado-willer-tomaz</t>
+        </is>
+      </c>
+      <c r="L44" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M44" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="24" t="inlineStr">
+        <is>
+          <t>iter</t>
+        </is>
+      </c>
+      <c r="B45" s="24" t="inlineStr">
+        <is>
+          <t>Instituto ITER</t>
+        </is>
+      </c>
+      <c r="C45" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D45" s="24" t="inlineStr">
+        <is>
+          <t>Instituto de ensino jurídico em São Paulo de que André Mendonça era sócio. Recebeu ao menos 52 contratos sem licitação de prefeituras, estados e tribunais (R$ 8,2 mi em dois anos, segundo a Revista Fórum), entre eles o governo de SP (R$ 1,6 mi), a Prefeitura de SP (R$ 380 mil) e o governo do RJ (R$ 518 mil). Em jan/2026 recebeu R$ 5,2 mi de empresa de um ex-parceiro de negócios de Vorcaro. Mendonça recebeu Vorcaro na sede do instituto em 14/03/2025.</t>
+        </is>
+      </c>
+      <c r="E45" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F45" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="24" t="inlineStr">
+        <is>
+          <t>Alvo de representações de parlamentares do PSOL ao TCM-SP, ao TCE-SP e ao MP-SP (set/2026). Mendonça anunciou que deixaria a sociedade.</t>
+        </is>
+      </c>
+      <c r="H45" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I45" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J45" s="24" t="inlineStr">
+        <is>
+          <t>Os levantamentos de contratos (52 e R$ 8,2 mi; 55 e R$ 10,8 mi) são recortes diferentes e não se somam.</t>
+        </is>
+      </c>
+      <c r="K45" s="24" t="inlineStr">
+        <is>
+          <t>Instituto de Mendonça é alvo de representações (apublica.org) https://apublica.org/nota/instituto-de-andre-mendonca-e-alvo-de-representacoes-para-investigar-irregularidades/ | Ex-parceiro de Vorcaro pôs R$ 5 mi no instituto (noticias.uol.com.br) https://noticias.uol.com.br/ultimas-noticias/redacao/2026/09/17/ex-parceiro-de-vorcaro-pos-r-5-milhoes-em-instituto-de-mendonca.htm | Mendonça diz que deixará sociedade (dgabc.com.br) https://www.dgabc.com.br/Noticia/4344940/mendonca-diz-que-deixara-sociedade-no-instituto-iter</t>
+        </is>
+      </c>
+      <c r="L45" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M45" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="24" t="inlineStr">
+        <is>
+          <t>triplex</t>
+        </is>
+      </c>
+      <c r="B46" s="24" t="inlineStr">
+        <is>
+          <t>Triplex de Vorcaro</t>
+        </is>
+      </c>
+      <c r="C46" s="24" t="inlineStr">
+        <is>
+          <t>Casas e ativos</t>
+        </is>
+      </c>
+      <c r="D46" s="24" t="inlineStr">
+        <is>
+          <t>Apartamento de Daniel Vorcaro no Itaim Bibi, em São Paulo. Segundo a piauí, com base em relatos de promoters e mensagens, recebia às quartas e quintas festas fechadas com garotas de programa. A reportagem cita entre os frequentadores o ministro Nunes Marques e o filho Kevin, e o ex-ministro Fábio Faria.</t>
+        </is>
+      </c>
+      <c r="E46" s="24" t="inlineStr">
+        <is>
+          <t>Itaim Bibi, São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F46" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G46" s="24" t="inlineStr">
+        <is>
+          <t>Não há processo sobre o imóvel nas fontes. As festas aparecem em mensagens obtidas pela PF e em reportagens.</t>
+        </is>
+      </c>
+      <c r="H46" s="24" t="inlineStr">
+        <is>
+          <t>Bem citado</t>
+        </is>
+      </c>
+      <c r="I46" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J46" s="24" t="inlineStr">
+        <is>
+          <t>O gabinete de Nunes Marques nega contato com Vorcaro. Os relatos não foram verificados de forma independente pela imprensa que os reproduziu.</t>
+        </is>
+      </c>
+      <c r="K46" s="24" t="inlineStr">
+        <is>
+          <t>A semana de festas fechadas de Vorcaro (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/10/11725610-terca-no-bar-quarta-e-quinta-no-triplex-a-semana-de-festas-fechadas-de-vorcaro.html | Vorcaro coordenou noitada para Nunes Marques (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/10/11726793-vorcaro-coordenou-noitada-em-triplex-para-ministro-kassio-nunes-marques.html</t>
+        </is>
+      </c>
+      <c r="L46" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M46" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="24" t="inlineStr">
+        <is>
+          <t>tarcisio</t>
+        </is>
+      </c>
+      <c r="B47" s="24" t="inlineStr">
+        <is>
+          <t>Tarcísio de Freitas</t>
+        </is>
+      </c>
+      <c r="C47" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D47" s="24" t="inlineStr">
+        <is>
+          <t>Governador de São Paulo (Republicanos) desde 2023 e ex-ministro da Infraestrutura de Jair Bolsonaro. Na campanha de 2022 recebeu R$ 2 mi de Fabiano Zettel, cunhado de Vorcaro, a maior doação de pessoa física. O governo dele contratou o Instituto ITER, de Mendonça, sem licitação (R$ 1,6 mi), e ele financiou 24% da campanha do deputado Cezinha de Madureira.</t>
+        </is>
+      </c>
+      <c r="E47" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F47" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G47" s="24" t="inlineStr">
+        <is>
+          <t>Não há investigação contra ele nas fontes.</t>
+        </is>
+      </c>
+      <c r="H47" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I47" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J47" s="24" t="inlineStr">
+        <is>
+          <t>O governo de SP diz que a campanha seguiu a lei, teve mais de 600 doadores e contas aprovadas, e que Tarcísio não tem vínculo com Zettel.</t>
+        </is>
+      </c>
+      <c r="K47" s="24" t="inlineStr">
+        <is>
+          <t>Alvo da PF doou R$ 5 mi a Bolsonaro e Tarcísio (cnnbrasil.com.br) https://www.cnnbrasil.com.br/politica/alvo-da-pf-doou-r-5-mi-para-campanhas-de-bolsonaro-e-tarcisio-em-2022/ | Contratos do ITER com governos (apublica.org) https://apublica.org/nota/instituto-de-andre-mendonca-e-alvo-de-representacoes-para-investigar-irregularidades/ | Financiamento da campanha de Cezinha (iclnoticias.com.br) https://iclnoticias.com.br/tarcisio-campanha-deputado-mendonca-vorcaro/</t>
+        </is>
+      </c>
+      <c r="L47" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M47" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N47" s="24" t="inlineStr">
+        <is>
+          <t>tarcisio.jpg</t>
+        </is>
+      </c>
+      <c r="O47" s="24" t="inlineStr">
+        <is>
+          <t>Ciete Silvério/Governo do Estado de SP · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="P47" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Governador_do_Estado_de_S%C3%A3o_Paulo,_Tarc%C3%ADsio_de_Freitas_-_Foto_Oficial.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="24" t="inlineStr">
+        <is>
+          <t>castro</t>
+        </is>
+      </c>
+      <c r="B48" s="24" t="inlineStr">
+        <is>
+          <t>Cláudio Castro</t>
+        </is>
+      </c>
+      <c r="C48" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D48" s="24" t="inlineStr">
+        <is>
+          <t>Ex-governador do Rio de Janeiro (PL), no cargo de 2021 a mar/2026. O governo dele contratou o ITER, de Mendonça (R$ 518 mil), e nomeou Hazenclever Cançado para a Loterj, que licenciou a Best Bet e contratou a RioPag. Renunciou em 23/03/2026 e foi tornado inelegível pelo TSE no dia seguinte. Em mai/2026 desistiu de concorrer ao Senado, depois de ser citado em fase da Operação Compliance Zero sobre aportes do Rio Previdência no Master.</t>
+        </is>
+      </c>
+      <c r="E48" s="24" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F48" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G48" s="24" t="inlineStr">
+        <is>
+          <t>Inelegível até 2030 por abuso de poder político e econômico na eleição de 2022 (TSE, 5 a 2, 24/03/2026); disse que recorreria. Mendonça escreveu que há indícios, "em tese", de vínculo próximo dele com Vorcaro.</t>
+        </is>
+      </c>
+      <c r="H48" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I48" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J48" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K48" s="24" t="inlineStr">
+        <is>
+          <t>TSE torna Castro inelegível (jovempan.com.br) https://jovempan.com.br/politica/tse-forma-maioria-para-tornar-castro-inelegivel-por-8-anos/ | Castro desiste do Senado após operações (oantagonista.com.br) https://oantagonista.com.br/brasil/claudio-castro-comunica-ao-pl-desistencia-de-candidatura-ao-senado-apos-operacoes/ | Mendonça votou a favor de Castro 4 vezes (iclnoticias.com.br) https://iclnoticias.com.br/mendonca-votou-a-favor-de-castro-4-vezes/</t>
+        </is>
+      </c>
+      <c r="L48" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M48" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N48" s="24" t="inlineStr">
+        <is>
+          <t>castro.jpg</t>
+        </is>
+      </c>
+      <c r="O48" s="24" t="inlineStr">
+        <is>
+          <t>Alan Santos/PR · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="P48" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Cl%C3%A1udio_Castro,_governador_do_Rio_de_Janeiro.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="24" t="inlineStr">
+        <is>
+          <t>moraes</t>
+        </is>
+      </c>
+      <c r="B49" s="24" t="inlineStr">
+        <is>
+          <t>Alexandre de Moraes</t>
+        </is>
+      </c>
+      <c r="C49" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D49" s="24" t="inlineStr">
+        <is>
+          <t>Ministro do STF desde 2017 e ex-presidente do TSE. É relator do segundo inquérito da PF contra Flávio Bolsonaro, sobre suspeita de lavagem com Willer Tomaz (out/2026). Segundo O Globo, ele e a esposa, a advogada Viviane Barci, desembarcaram em ago/2025 do jato PP-NLR, o mesmo usado por Flávio. O escritório dela tinha contratos com o Banco Master. A PF diz que Fábio Faria intermediou contatos entre Vorcaro e Moraes.</t>
+        </is>
+      </c>
+      <c r="E49" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F49" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G49" s="24" t="inlineStr">
+        <is>
+          <t>Não é investigado nas fontes. O PGR Paulo Gonet sustenta que Mendonça o investigou antes de aval do plenário.</t>
+        </is>
+      </c>
+      <c r="H49" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I49" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J49" s="24" t="inlineStr">
+        <is>
+          <t>Moraes tinha dito que nunca viajou em aviões de Vorcaro e nega que tenha existido o acordo de pagamento em cotas de jato citado pela PF.</t>
+        </is>
+      </c>
+      <c r="K49" s="24" t="inlineStr">
+        <is>
+          <t>Moraes flagrado desembarcando de jatinho de Vorcaro (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/09/11724483-alexandre-de-moraes-foi-flagrado-desembarcando-de-jatinho-de-vorcaro.html | Segundo inquérito contra Flávio no STF (oliberal.com) https://www.oliberal.com/politica/flavio-e-investigado-em-2-inquerito-no-stf-para-apurar-suspeitas-de-lavagem-com-advogado-1.1183991 | Gonet diz que Mendonça investigou Moraes (iclnoticias.com.br) https://iclnoticias.com.br/gonet-diz-que-mendonca-investigou-moraes/</t>
+        </is>
+      </c>
+      <c r="L49" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M49" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N49" s="24" t="inlineStr">
+        <is>
+          <t>moraes.jpg</t>
+        </is>
+      </c>
+      <c r="O49" s="24" t="inlineStr">
+        <is>
+          <t>Isac Nóbrega · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="P49" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Ministro_Alexandre_de_Moraes_como_presidente_do_TSE.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="24" t="inlineStr">
+        <is>
+          <t>rnunes</t>
+        </is>
+      </c>
+      <c r="B50" s="24" t="inlineStr">
+        <is>
+          <t>Ricardo Nunes</t>
+        </is>
+      </c>
+      <c r="C50" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D50" s="24" t="inlineStr">
+        <is>
+          <t>Prefeito de São Paulo (MDB) desde 2021, reeleito em 2024. A prefeitura contratou o ITER, de Mendonça (R$ 380 mil). Segundo o ICL, o irmão do ministro, Alexandre de Almeida Mendonça, chegou a secretário-executivo da SP Regula em jun/2026, por portaria de Nunes, depois de Mendonça votar na direção defendida pela prefeitura no caso das concessões funerárias no STF.</t>
+        </is>
+      </c>
+      <c r="E50" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F50" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G50" s="24" t="inlineStr">
+        <is>
+          <t>Não há investigação contra ele nas fontes.</t>
+        </is>
+      </c>
+      <c r="H50" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I50" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J50" s="24" t="inlineStr">
+        <is>
+          <t>A prefeitura diz que não houve promoção (mesmo nível, mesma remuneração), que a mudança veio mais de um ano após o voto e chama a insinuação de "irresponsável e sem fundamento".</t>
+        </is>
+      </c>
+      <c r="K50" s="24" t="inlineStr">
+        <is>
+          <t>Irmão de Mendonça foi promovido por Nunes (iclnoticias.com.br) https://iclnoticias.com.br/irmao-de-mendonca-foi-promovido-por-nunes/ | Contratos do ITER (apublica.org) https://apublica.org/nota/instituto-de-andre-mendonca-e-alvo-de-representacoes-para-investigar-irregularidades/</t>
+        </is>
+      </c>
+      <c r="L50" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M50" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N50" s="24" t="inlineStr">
+        <is>
+          <t>rnunes.jpg</t>
+        </is>
+      </c>
+      <c r="O50" s="24" t="inlineStr">
+        <is>
+          <t>Celso Silva/Governo do Estado de SP · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="P50" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Ricardo_Nunes,_December_2024.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="24" t="inlineStr">
+        <is>
+          <t>cezinha</t>
+        </is>
+      </c>
+      <c r="B51" s="24" t="inlineStr">
+        <is>
+          <t>Cezinha de Madureira</t>
+        </is>
+      </c>
+      <c r="C51" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D51" s="24" t="inlineStr">
+        <is>
+          <t>Deputado federal por São Paulo, no terceiro mandato, e liderança da Assembleia de Deus Ministério de Madureira. Mensagens obtidas pela PF mostram que ele e o advogado Ciro Rocha Soares articularam os encontros de Vorcaro com Mendonça em fev e mar/2025; em 13/03/2025 marcou a reunião do dia seguinte, na sede do ITER. Tarcísio financiou 24% da campanha dele.</t>
+        </is>
+      </c>
+      <c r="E51" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP); mandato em Brasília</t>
+        </is>
+      </c>
+      <c r="F51" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G51" s="24" t="inlineStr">
+        <is>
+          <t>Alvo de operação autorizada pelo ministro Flávio Dino (2026). Sem denúncia nas fontes.</t>
+        </is>
+      </c>
+      <c r="H51" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I51" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J51" s="24" t="inlineStr">
+        <is>
+          <t>As reportagens não trazem resposta dele.</t>
+        </is>
+      </c>
+      <c r="K51" s="24" t="inlineStr">
+        <is>
+          <t>Mensagens e áudios inéditos sobre Mendonça (iclnoticias.com.br) https://iclnoticias.com.br/vaza-mendonca-mensagens-e-audios-ineditos/ | Áudios revelam encontro entre Vorcaro e Mendonça (bahianoticias.com.br) https://www.bahianoticias.com.br/justica/noticia/75274-audios-e-mensagens-revelam-encontro-entre-vorcaro-e-mendonca-ministro-admite-e-diz-que-se-limitou-a-ouvi-lo | Operação de Dino e afastamento na PF (iclnoticias.com.br) https://iclnoticias.com.br/mendonca-cesinha-madureira-vorcaro-dino/</t>
+        </is>
+      </c>
+      <c r="L51" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M51" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N51" s="24" t="inlineStr">
+        <is>
+          <t>cezinha.jpg</t>
+        </is>
+      </c>
+      <c r="O51" s="24" t="inlineStr">
+        <is>
+          <t>Câmara dos Deputados · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="P51" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Cezinha_de_Madureira.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="24" t="inlineStr">
+        <is>
+          <t>cancado</t>
+        </is>
+      </c>
+      <c r="B52" s="24" t="inlineStr">
+        <is>
+          <t>Hazenclever Cançado</t>
+        </is>
+      </c>
+      <c r="C52" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D52" s="24" t="inlineStr">
+        <is>
+          <t>Hazenclever Lopes Cançado, advogado e servidor federal, ex-assessor do senador Magno Malta. Foi nomeado presidente da Loterj por Cláudio Castro em jul/2022 e, nessa função, assinou em 25/05/2023 a licença da Rede Loto (Best Bet), a primeira bet autorizada pelo estado.</t>
+        </is>
+      </c>
+      <c r="E52" s="24" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F52" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G52" s="24" t="inlineStr">
+        <is>
+          <t>Não há investigação contra ele nas fontes.</t>
+        </is>
+      </c>
+      <c r="H52" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I52" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J52" s="24" t="inlineStr">
+        <is>
+          <t>A indicação dele por Flávio é atribuída à Folha ("teria"). Ele não comentou até a publicação das reportagens.</t>
+        </is>
+      </c>
+      <c r="K52" s="24" t="inlineStr">
+        <is>
+          <t>Loterj tem novo presidente (bnldata.com.br) https://bnldata.com.br/?p=105308 | Bet de investigado pagou voos de Flávio (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/10/11726788-bet-de-investigado-por-fraude-no-inss-pagou-voos-de-flavio-bolsonaro-na-europa-aponta-pf.html</t>
+        </is>
+      </c>
+      <c r="L52" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M52" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="24" t="inlineStr">
+        <is>
+          <t>motta</t>
+        </is>
+      </c>
+      <c r="B53" s="24" t="inlineStr">
+        <is>
+          <t>Hugo Motta</t>
+        </is>
+      </c>
+      <c r="C53" s="24" t="inlineStr">
+        <is>
+          <t>Vorcaro e o Banco Master</t>
+        </is>
+      </c>
+      <c r="D53" s="24" t="inlineStr">
+        <is>
+          <t>Deputado federal pela Paraíba (Republicanos) e presidente da Câmara desde fev/2025. Integrava com Vorcaro, Ciro Nogueira e Fábio Faria um grupo de mensagens criado em abr/2024 para combinar jantares, viagens e encontros; as últimas mensagens são da noite da prisão de Vorcaro (17/11/2025). Segundo a reportagem, Ciro o apresentou a Vorcaro para uma possível sociedade num terreno em João Pessoa.</t>
+        </is>
+      </c>
+      <c r="E53" s="24" t="inlineStr">
+        <is>
+          <t>Paraíba (PB); mandato em Brasília</t>
+        </is>
+      </c>
+      <c r="F53" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G53" s="24" t="inlineStr">
+        <is>
+          <t>Não é investigado nas fontes.</t>
+        </is>
+      </c>
+      <c r="H53" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I53" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J53" s="24" t="inlineStr">
+        <is>
+          <t>A assessoria de Motta disse que não se pronunciaria.</t>
+        </is>
+      </c>
+      <c r="K53" s="24" t="inlineStr">
+        <is>
+          <t>Grupo com Motta, Ciro e Faria organizava encontros (gazetadopovo.com.br) https://www.gazetadopovo.com.br/republica/vorcaro-grupo-motta-ciro-nogueira-fabio-faria-organizar-encontros/ | Vorcaro cita encontros com Hugo Motta (poder360.com.br) https://www.poder360.com.br/poder-economia/vorcaro-cita-encontros-com-hugo-motta-e-elogia-emenda-de-ciro-nogueira/</t>
+        </is>
+      </c>
+      <c r="L53" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M53" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N53" s="24" t="inlineStr">
+        <is>
+          <t>motta.jpg</t>
+        </is>
+      </c>
+      <c r="O53" s="24" t="inlineStr">
+        <is>
+          <t>Gilclécio Lucena · CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="P53" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Deputado_Federal_Hugo_Motta_(cropped).jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="24" t="inlineStr">
+        <is>
+          <t>marcal</t>
+        </is>
+      </c>
+      <c r="B54" s="24" t="inlineStr">
+        <is>
+          <t>Pablo Marçal</t>
+        </is>
+      </c>
+      <c r="C54" s="24" t="inlineStr">
+        <is>
+          <t>Vorcaro e o Banco Master</t>
+        </is>
+      </c>
+      <c r="D54" s="24" t="inlineStr">
+        <is>
+          <t>Empresário e influenciador, ex-coach; foi candidato a prefeito de São Paulo em 2024. Segundo o Valor, com base em mensagens do celular de Vorcaro, a Prime You pagou um voo de R$ 1,17 mi de São Paulo a Nova York usado por ele entre mai e jun/2025.</t>
+        </is>
+      </c>
+      <c r="E54" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F54" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G54" s="24" t="inlineStr">
+        <is>
+          <t>Não é investigado no caso Master nas fontes.</t>
+        </is>
+      </c>
+      <c r="H54" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I54" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J54" s="24" t="inlineStr">
+        <is>
+          <t>Marçal confirmou o voo e disse que se ofereceu para pagar; segundo ele, Vorcaro sugeriu que testasse o avião antes de comprar um parecido.</t>
+        </is>
+      </c>
+      <c r="K54" s="24" t="inlineStr">
+        <is>
+          <t>Empresa de Vorcaro pagou voo de Marçal (gp1.com.br) https://www.gp1.com.br/brasil/noticia/2026/10/2/empresa-ligada-a-daniel-vorcaro-pagou-voo-de-r-117-milhao-usado-por-pablo-marcal-633016.html | Vorcaro bancou voo e mandou ocultar valor (revistaforum.com.br) https://revistaforum.com.br/politica/vorcaro-voo-pablo-marcal/</t>
+        </is>
+      </c>
+      <c r="L54" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M54" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N54" s="24" t="inlineStr">
+        <is>
+          <t>marcal.jpg</t>
+        </is>
+      </c>
+      <c r="O54" s="24" t="inlineStr">
+        <is>
+          <t>TV Brasil Central · CC BY 3.0</t>
+        </is>
+      </c>
+      <c r="P54" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Pablo_Mar%C3%A7al_(cropped).png</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="24" t="inlineStr">
+        <is>
+          <t>bianco</t>
+        </is>
+      </c>
+      <c r="B55" s="24" t="inlineStr">
+        <is>
+          <t>Bruno Bianco Leal</t>
+        </is>
+      </c>
+      <c r="C55" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D55" s="24" t="inlineStr">
+        <is>
+          <t>Advogado-geral da União de ago/2021 a jan/2023, sucessor de Mendonça no governo Jair Bolsonaro. Depois atuou na iniciativa privada ligado ao Banco Master e passou a integrar a defesa de Vorcaro. Mensagens mostram o advogado Ciro Rocha Soares pedindo que ele fosse convidado para a reunião com Mendonça de 19/02/2025.</t>
+        </is>
+      </c>
+      <c r="E55" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F55" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G55" s="24" t="inlineStr">
+        <is>
+          <t>Não é investigado nas fontes.</t>
+        </is>
+      </c>
+      <c r="H55" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I55" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J55" s="24" t="inlineStr">
+        <is>
+          <t>As mensagens mostram o convite, mas não se ele compareceu.</t>
+        </is>
+      </c>
+      <c r="K55" s="24" t="inlineStr">
+        <is>
+          <t>Mensagens e áudios inéditos sobre Mendonça (iclnoticias.com.br) https://iclnoticias.com.br/vaza-mendonca-mensagens-e-audios-ineditos/ | Áudios revelam encontro entre Vorcaro e Mendonça (bahianoticias.com.br) https://www.bahianoticias.com.br/justica/noticia/75274-audios-e-mensagens-revelam-encontro-entre-vorcaro-e-mendonca-ministro-admite-e-diz-que-se-limitou-a-ouvi-lo</t>
+        </is>
+      </c>
+      <c r="L55" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M55" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N55" s="24" t="inlineStr">
+        <is>
+          <t>bianco.jpg</t>
+        </is>
+      </c>
+      <c r="O55" s="24" t="inlineStr">
+        <is>
+          <t>Marcos Corrêa/PR · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="P55" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Bruno_Bianco.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="24" t="inlineStr">
+        <is>
+          <t>jbcarvalho</t>
+        </is>
+      </c>
+      <c r="B56" s="24" t="inlineStr">
+        <is>
+          <t>Bispo JB Carvalho</t>
+        </is>
+      </c>
+      <c r="C56" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D56" s="24" t="inlineStr">
+        <is>
+          <t>João Batista Araújo Carvalho Lima, bispo fundador da Comunidade das Nações, igreja com mais de 50 unidades no Brasil, nos EUA e em Portugal. Flávio e a mulher, Fernanda, foram batizados na igreja, em Brasília, em jan/2024. Em livro de 2001 ele defendeu tirar de Nossa Senhora Aparecida o título de padroeira; os trechos voltaram a circular em set/2026.</t>
+        </is>
+      </c>
+      <c r="E56" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F56" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G56" s="24" t="inlineStr">
+        <is>
+          <t>Não há processo contra ele nas fontes. Uma associação pediu à Justiça Federal a retirada do livro.</t>
+        </is>
+      </c>
+      <c r="H56" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I56" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J56" s="24" t="inlineStr">
+        <is>
+          <t>As reportagens não trazem resposta dele.</t>
+        </is>
+      </c>
+      <c r="K56" s="24" t="inlineStr">
+        <is>
+          <t>A ligação de Flávio com o bispo (tvtnews.com.br) https://tvtnews.com.br/?p=804749 | Bispo que batizou Flávio criticou Nossa Senhora (poder360.com.br) https://www.poder360.com.br/poder-gente/bispo-que-batizou-flavio-criticou-nossa-senhora-em-livro/</t>
+        </is>
+      </c>
+      <c r="L56" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M56" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N56" s="24" t="inlineStr">
+        <is>
+          <t>jbcarvalho.jpg</t>
+        </is>
+      </c>
+      <c r="O56" s="24" t="inlineStr">
+        <is>
+          <t>Povoselinguas · CC BY 3.0</t>
+        </is>
+      </c>
+      <c r="P56" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:JB_Carvalho_(3x4_cropped).webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="24" t="inlineStr">
+        <is>
+          <t>stf</t>
+        </is>
+      </c>
+      <c r="B57" s="24" t="inlineStr">
+        <is>
+          <t>STF</t>
+        </is>
+      </c>
+      <c r="C57" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D57" s="24" t="inlineStr">
+        <is>
+          <t>Supremo Tribunal Federal. Concentra os casos do mapa que envolvem autoridades com foro: o caso Master (relator André Mendonça desde fev/2026), o inquérito sobre o dinheiro de Vorcaro para o filme Dark Horse (Mendonça) e o inquérito sobre suspeita de lavagem de Flávio com Willer Tomaz (Alexandre de Moraes, out/2026). Em 2021 a Segunda Turma anulou relatórios do Coaf do caso da rachadinha.</t>
+        </is>
+      </c>
+      <c r="E57" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F57" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G57" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H57" s="24" t="inlineStr">
+        <is>
+          <t>Órgão público</t>
+        </is>
+      </c>
+      <c r="I57" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J57" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K57" s="24" t="inlineStr">
+        <is>
+          <t>STF anula 4 relatórios do Coaf (poder360.com.br) https://www.poder360.com.br/justica/stf-anula-4-relatorios-do-coaf-que-miravam-flavio-no-caso-das-rachadinhas/ | Segundo inquérito contra Flávio no STF (oliberal.com) https://www.oliberal.com/politica/flavio-e-investigado-em-2-inquerito-no-stf-para-apurar-suspeitas-de-lavagem-com-advogado-1.1183991</t>
+        </is>
+      </c>
+      <c r="L57" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M57" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N57" s="24" t="inlineStr">
+        <is>
+          <t>stf.jpg</t>
+        </is>
+      </c>
+      <c r="O57" s="24" t="inlineStr">
+        <is>
+          <t>Daderot · CC0 (domínio público)</t>
+        </is>
+      </c>
+      <c r="P57" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Supremo_Tribunal_Federal_building_in_Brasilia_-_DSC00288.JPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="24" t="inlineStr">
+        <is>
+          <t>abin</t>
+        </is>
+      </c>
+      <c r="B58" s="24" t="inlineStr">
+        <is>
+          <t>Abin</t>
+        </is>
+      </c>
+      <c r="C58" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D58" s="24" t="inlineStr">
+        <is>
+          <t>Agência Brasileira de Inteligência. Na investigação da "Abin paralela", a PF achou o áudio de uma reunião de 25/08/2020 entre Jair Bolsonaro, Augusto Heleno e o então diretor Alexandre Ramagem, possivelmente com uma advogada de Flávio, em que Ramagem sugere processos contra auditores da Receita para blindar Flávio no caso da rachadinha.</t>
+        </is>
+      </c>
+      <c r="E58" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F58" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="24" t="inlineStr">
+        <is>
+          <t>O episódio faz parte do inquérito sobre uso ilegal do sistema First Mile por servidores da Abin.</t>
+        </is>
+      </c>
+      <c r="H58" s="24" t="inlineStr">
+        <is>
+          <t>Órgão público</t>
+        </is>
+      </c>
+      <c r="I58" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J58" s="24" t="inlineStr">
+        <is>
+          <t>Flávio diz não ter "nenhuma relação" com a Abin.</t>
+        </is>
+      </c>
+      <c r="K58" s="24" t="inlineStr">
+        <is>
+          <t>Áudio de Ramagem sugere investigar auditores (poder360.com.br) https://www.poder360.com.br/poder-justica/audio-de-ramagem-sugere-investigar-auditores-para-blindar-flavio/ | PF investiga se Abin ajudou defesa de Flávio (congressoemfoco.com.br) https://congressoemfoco.com.br/noticia/7623/pf-investiga-se-abin-ajudou-defesa-de-flavio-bolsonaro-senador-nega</t>
+        </is>
+      </c>
+      <c r="L58" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M58" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N58" s="24" t="inlineStr">
+        <is>
+          <t>abin.jpg</t>
+        </is>
+      </c>
+      <c r="O58" s="24" t="inlineStr">
+        <is>
+          <t>Antonio Cruz/Agência Brasil · CC BY 3.0 BR</t>
+        </is>
+      </c>
+      <c r="P58" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Pr%C3%A9dio_da_Abin.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="24" t="inlineStr">
+        <is>
+          <t>cpi</t>
+        </is>
+      </c>
+      <c r="B59" s="24" t="inlineStr">
+        <is>
+          <t>CPI da pandemia (Covaxin)</t>
+        </is>
+      </c>
+      <c r="C59" s="24" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="D59" s="24" t="inlineStr">
+        <is>
+          <t>CPI da Pandemia do Senado (abr a out/2021), relatada por Renan Calheiros. Investigou, entre outros pontos, a compra da vacina Covaxin pelo Ministério da Saúde. Flávio, então senador do Patriota, atuou na comissão como defensor do governo do pai.</t>
+        </is>
+      </c>
+      <c r="E59" s="24" t="inlineStr">
+        <is>
+          <t>Senado Federal, Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F59" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G59" s="24" t="inlineStr">
+        <is>
+          <t>O relatório final pediu indiciamentos; a CPI foi encerrada em out/2021.</t>
+        </is>
+      </c>
+      <c r="H59" s="24" t="inlineStr">
+        <is>
+          <t>Órgão público</t>
+        </is>
+      </c>
+      <c r="I59" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J59" s="24" t="inlineStr">
+        <is>
+          <t>A citação de Willer Tomaz no caso Covaxin e o cancelamento da quebra do sigilo dele vêm do vídeo de origem e não foram reverificados nesta rodada.</t>
+        </is>
+      </c>
+      <c r="K59" s="24" t="inlineStr">
+        <is>
+          <t>Flávio Bolsonaro na CPI da Pandemia (congressoemfoco.com.br) https://congressoemfoco.com.br/artigo/14228/flavio-bolsonaro-na-cpi-da-pandemia | CPI aprova convocações e quebras de sigilo (senado.leg.br) https://www12.senado.leg.br/radio/1/noticia/2021/06/23/cpi-da-pandemia-aprovou-novas-convocacoes-quebras-de-sigilos-e-pedidos-de-informacoes</t>
+        </is>
+      </c>
+      <c r="L59" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M59" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N59" s="24" t="inlineStr">
+        <is>
+          <t>cpi.jpg</t>
+        </is>
+      </c>
+      <c r="O59" s="24" t="inlineStr">
+        <is>
+          <t>Agência Senado · CC BY 2.0</t>
+        </is>
+      </c>
+      <c r="P59" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:CPIPANDEMIA_-_Comiss%C3%A3o_Parlamentar_de_Inqu%C3%A9rito_da_Pandemia_(1).jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="24" t="inlineStr">
+        <is>
+          <t>loterj</t>
+        </is>
+      </c>
+      <c r="B60" s="24" t="inlineStr">
+        <is>
+          <t>Loterj</t>
+        </is>
+      </c>
+      <c r="C60" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D60" s="24" t="inlineStr">
+        <is>
+          <t>Loteria do Estado do Rio de Janeiro, autarquia estadual. Em mai/2023, sob a presidência de Hazenclever Cançado, licenciou a Rede Loto (Best Bet), a primeira bet autorizada no país, sem exigir a identificação dos beneficiários finais. Em 2023 contratou a RioPag para intermediar os pagamentos das bets; a empresa faturou R$ 187,8 mi em taxas entre jun/2023 e ago/2026.</t>
+        </is>
+      </c>
+      <c r="E60" s="24" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F60" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" s="24" t="inlineStr">
+        <is>
+          <t>Rescindiu o contrato da RioPag em 22/09/2026 e cobra R$ 9,4 mi; uma liminar suspendeu a rescisão.</t>
+        </is>
+      </c>
+      <c r="H60" s="24" t="inlineStr">
+        <is>
+          <t>Órgão público</t>
+        </is>
+      </c>
+      <c r="I60" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J60" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K60" s="24" t="inlineStr">
+        <is>
+          <t>Loterj licencia a Rede Loto (lotterydaily.com) https://lotterydaily.com/2023/06/06/retail/rios-loterj-achieves-2023-betting-ambitions-with-rede-loto-contract/ | Bet de investigado pagou voos de Flávio (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/10/11726788-bet-de-investigado-por-fraude-no-inss-pagou-voos-de-flavio-bolsonaro-na-europa-aponta-pf.html | Loterj rescinde contrato com a RioPag (bnldata.com.br) https://bnldata.com.br/loterj-rescinde-contrato-com-riopag-e-cobra-r-94-mi-da-empresa/</t>
+        </is>
+      </c>
+      <c r="L60" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M60" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="24" t="inlineStr">
+        <is>
+          <t>pgr</t>
+        </is>
+      </c>
+      <c r="B61" s="24" t="inlineStr">
+        <is>
+          <t>Procuradoria-Geral (PGR)</t>
+        </is>
+      </c>
+      <c r="C61" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D61" s="24" t="inlineStr">
+        <is>
+          <t>Procuradoria-Geral da República, chefiada por Paulo Gonet. Cabe a ela denunciar autoridades com foro no STF, como os investigados do caso Master. Em 2026 negociava com a PF a delação de Vorcaro e sustentou que Mendonça investigou Alexandre de Moraes sem aval do plenário. Não foi ouvida antes do afastamento do diretor-geral da PF.</t>
+        </is>
+      </c>
+      <c r="E61" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F61" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G61" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H61" s="24" t="inlineStr">
+        <is>
+          <t>Órgão público</t>
+        </is>
+      </c>
+      <c r="I61" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J61" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K61" s="24" t="inlineStr">
+        <is>
+          <t>Afastamento do diretor-geral da PF sem ouvir a PGR (cnnbrasil.com.br) https://www.cnnbrasil.com.br/blogs/teo-cury/politica/mendonca-ordenou-afastamento-de-diretor-geral-da-pf-sem-ouvir-pgr/ | Gonet diz que Mendonça investigou Moraes (iclnoticias.com.br) https://iclnoticias.com.br/gonet-diz-que-mendonca-investigou-moraes/ | Delação de Vorcaro em negociação (timesbrasil.com.br) https://timesbrasil.com.br/brasil/operacoes-da-pf/pf-prende-paulo-henrique-costa-ex-presidente-do-brb-em-nova-fase-da-compliance-zero/</t>
+        </is>
+      </c>
+      <c r="L61" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M61" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N61" s="24" t="inlineStr">
+        <is>
+          <t>pgr.jpg</t>
+        </is>
+      </c>
+      <c r="O61" s="24" t="inlineStr">
+        <is>
+          <t>Webysther · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="P61" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Webysther_20180212174501_-_PGR_-_Procuradoria_Geral_da_Rep%C3%BAblica.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="24" t="inlineStr">
+        <is>
+          <t>receita</t>
+        </is>
+      </c>
+      <c r="B62" s="24" t="inlineStr">
+        <is>
+          <t>Receita Federal</t>
+        </is>
+      </c>
+      <c r="C62" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D62" s="24" t="inlineStr">
+        <is>
+          <t>Receita Federal. O secretário José Barroso Tostes Neto teve três reuniões com Flávio em ago e set/2020, a pedido do senador e com a advogada dele no caso Queiroz; a última teria sido na casa de Flávio. Os temas declarados foram a situação fiscal de pessoas e empresas ligadas a ele e supostas condutas irregulares de servidores do órgão.</t>
+        </is>
+      </c>
+      <c r="E62" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F62" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="24" t="inlineStr">
+        <is>
+          <t>Órgão público</t>
+        </is>
+      </c>
+      <c r="I62" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J62" s="24" t="inlineStr">
+        <is>
+          <t>O local da última reunião é relatado com "teria".</t>
+        </is>
+      </c>
+      <c r="K62" s="24" t="inlineStr">
+        <is>
+          <t>Receita confirma visita de secretário a Flávio (poder360.com.br) https://www.poder360.com.br/governo/receita-federal-confirma-visita-de-secretario-do-fisco-a-flavio-bolsonaro/ | Chefe da Receita foi à casa de Flávio (infomoney.com.br) https://www.infomoney.com.br/?p=2535322</t>
+        </is>
+      </c>
+      <c r="L62" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M62" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N62" s="24" t="inlineStr">
+        <is>
+          <t>receita.jpg</t>
+        </is>
+      </c>
+      <c r="O62" s="24" t="inlineStr">
+        <is>
+          <t>Academia de Letras de Campo Maior · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="P62" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Ag%C3%AAncia_da_Receita_Federal_de_Campo_Maior,_Piau%C3%AD,_Brasil.JPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="24" t="inlineStr">
+        <is>
+          <t>tse</t>
+        </is>
+      </c>
+      <c r="B63" s="24" t="inlineStr">
+        <is>
+          <t>TSE</t>
+        </is>
+      </c>
+      <c r="C63" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D63" s="24" t="inlineStr">
+        <is>
+          <t>Tribunal Superior Eleitoral. Kassio Nunes Marques assumiu a presidência em mai/2026 e conduz as eleições de 2026. Em mar/2026 o tribunal tornou Cláudio Castro inelegível; Nunes Marques votou pela absolvição.</t>
+        </is>
+      </c>
+      <c r="E63" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F63" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H63" s="24" t="inlineStr">
+        <is>
+          <t>Órgão público</t>
+        </is>
+      </c>
+      <c r="I63" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J63" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K63" s="24" t="inlineStr">
+        <is>
+          <t>Nunes Marques assume a presidência do TSE (poder360.com.br) https://www.poder360.com.br/brasil/nunes-marques-assume-presidencia-do-tse/ | TSE torna Castro inelegível (jovempan.com.br) https://jovempan.com.br/politica/tse-forma-maioria-para-tornar-castro-inelegivel-por-8-anos/</t>
+        </is>
+      </c>
+      <c r="L63" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M63" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N63" s="24" t="inlineStr">
+        <is>
+          <t>tse.jpg</t>
+        </is>
+      </c>
+      <c r="O63" s="24" t="inlineStr">
+        <is>
+          <t>Alexandresena · CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="P63" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Sede_do_Tribunal_Superior_Eleitoral,_em_Bras%C3%ADlia.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="24" t="inlineStr">
+        <is>
+          <t>brb</t>
+        </is>
+      </c>
+      <c r="B64" s="24" t="inlineStr">
+        <is>
+          <t>BRB (Banco de Brasília)</t>
+        </is>
+      </c>
+      <c r="C64" s="24" t="inlineStr">
+        <is>
+          <t>Vorcaro e o Banco Master</t>
+        </is>
+      </c>
+      <c r="D64" s="24" t="inlineStr">
+        <is>
+          <t>Banco de Brasília, banco público controlado pelo governo do DF. Pôs cerca de R$ 12 bi no Master comprando carteiras de crédito consignado que a investigação aponta como fraudulentas, e tentou comprar o próprio Master em 2025. O ex-presidente Paulo Henrique Costa foi afastado em nov/2025 e preso em 16/04/2026 na Compliance Zero. Em 2021 financiou R$ 3,1 mi da mansão de Flávio em Brasília.</t>
+        </is>
+      </c>
+      <c r="E64" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F64" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G64" s="24" t="inlineStr">
+        <is>
+          <t>Ex-dirigentes investigados no inquérito do caso Master. A PF também apura as condições do empréstimo a Flávio.</t>
+        </is>
+      </c>
+      <c r="H64" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I64" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J64" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K64" s="24" t="inlineStr">
+        <is>
+          <t>PF prende ex-presidente do BRB (timesbrasil.com.br) https://timesbrasil.com.br/brasil/operacoes-da-pf/pf-prende-paulo-henrique-costa-ex-presidente-do-brb-em-nova-fase-da-compliance-zero/ | PF apura financiamento do BRB a Flávio (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/10/11725606-pf-apura-condicoes-de-financiamento-do-brb-a-flavio-bolsonaro-para-mansao-de-rs-6-milhoes.html</t>
+        </is>
+      </c>
+      <c r="L64" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M64" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N64" s="24" t="inlineStr">
+        <is>
+          <t>brb.png</t>
+        </is>
+      </c>
+      <c r="O64" s="24" t="inlineStr">
+        <is>
+          <t>Banco de Brasília · domínio público (logo simples, sem direito autoral)</t>
+        </is>
+      </c>
+      <c r="P64" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Logotipo_do_Banco_de_Bras%C3%ADlia.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="24" t="inlineStr">
+        <is>
+          <t>govlula</t>
+        </is>
+      </c>
+      <c r="B65" s="24" t="inlineStr">
+        <is>
+          <t>Governo Lula (Haddad, Gleisi, Mercadante)</t>
+        </is>
+      </c>
+      <c r="C65" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D65" s="24" t="inlineStr">
+        <is>
+          <t>Ministros do governo Lula citados em mensagens do celular de Vorcaro. Em 29/10/2025, enquanto a compra do Master pelo BRB estava em análise no Banco Central, Vorcaro escreveu que Fernando Haddad era "um dos meus maiores opositores". A planilha também registra pedido de ajuda para "bloquear" Gleisi Hoffmann e Aloizio Mercadante.</t>
+        </is>
+      </c>
+      <c r="E65" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F65" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G65" s="24" t="inlineStr">
+        <is>
+          <t>Nenhum dos ministros é investigado nas fontes.</t>
+        </is>
+      </c>
+      <c r="H65" s="24" t="inlineStr">
+        <is>
+          <t>Órgão público</t>
+        </is>
+      </c>
+      <c r="I65" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J65" s="24" t="inlineStr">
+        <is>
+          <t>Haddad diz que nunca recebeu Vorcaro e que recusou "diversas vezes" encontrá-lo. O trecho sobre Gleisi e Mercadante não foi reverificado nesta rodada.</t>
+        </is>
+      </c>
+      <c r="K65" s="24" t="inlineStr">
+        <is>
+          <t>Vorcaro sobre Haddad: um de meus maiores opositores (em.com.br) https://www.em.com.br/politica/2026/10/7513704-vorcaro-sobre-haddad-um-de-meus-maiores-opositores.html | Haddad nega ter recebido Vorcaro (dgabc.com.br) https://www.dgabc.com.br/Noticia/4346805/haddad-nega-ter-recebido-vorcaro-ou-estado-no-mesmo-ambiente-que-ele</t>
+        </is>
+      </c>
+      <c r="L65" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M65" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="24" t="inlineStr">
+        <is>
+          <t>adriano</t>
+        </is>
+      </c>
+      <c r="B66" s="24" t="inlineStr">
+        <is>
+          <t>Adriano da Nóbrega</t>
+        </is>
+      </c>
+      <c r="C66" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D66" s="24" t="inlineStr">
+        <is>
+          <t>Adriano Magalhães da Nóbrega, ex-capitão do Bope apontado pelo MP-RJ como chefe do Escritório do Crime e da milícia de Rio das Pedras. Flávio o homenageou com moção de louvor em 2003 e com a Medalha Tiradentes em jun/2005, quando ele estava preso por homicídio (depois absolvido, em 2007). A mãe e a mulher dele trabalharam no gabinete de Flávio na Alerj.</t>
+        </is>
+      </c>
+      <c r="E66" s="24" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F66" s="24" t="inlineStr">
+        <is>
+          <t>Morto (fev/2020)</t>
+        </is>
+      </c>
+      <c r="G66" s="24" t="inlineStr">
+        <is>
+          <t>Foragido desde a Operação Os Intocáveis (jan/2019); morto pela polícia na Bahia em fev/2020.</t>
+        </is>
+      </c>
+      <c r="H66" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I66" s="24" t="inlineStr">
+        <is>
+          <t>Apontado pelo MP-RJ como chefe da milícia de Rio das Pedras e do Escritório do Crime.</t>
+        </is>
+      </c>
+      <c r="J66" s="24" t="inlineStr">
+        <is>
+          <t>Mesmo sendo uma figura notória, fica sem foto porque não era pessoa pública por escolha.</t>
+        </is>
+      </c>
+      <c r="K66" s="24" t="inlineStr">
+        <is>
+          <t>Ex-PM estava preso quando Flávio o homenageou (agazeta.com.br) https://www.agazeta.com.br/brasil/ex-pm-estava-preso-por-homicidio-quando-flavio-bolsonaro-o-homenageou-0119 | Miliciano ligado a Flávio é morto (congressoemfoco.com.br) https://www.congressoemfoco.com.br/governo/miliciano-ligado-a-flavio-bolsonaro-e-morto-durante-operacao/ | Entre medalhas e milícias (vermelho.org.br) https://vermelho.org.br/?p=740865</t>
+        </is>
+      </c>
+      <c r="L66" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M66" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="24" t="inlineStr">
+        <is>
+          <t>ronald</t>
+        </is>
+      </c>
+      <c r="B67" s="24" t="inlineStr">
+        <is>
+          <t>Ronald Paulo Alves Pereira</t>
+        </is>
+      </c>
+      <c r="C67" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D67" s="24" t="inlineStr">
+        <is>
+          <t>Major da PM do Rio. Flávio apresentou em 2004 uma moção de louvor a ele na Alerj. Foi preso em jan/2019 na Operação Os Intocáveis, contra a milícia de Rio das Pedras, e em fev/2026 condenado pela Primeira Turma do STF a 56 anos de prisão no caso Marielle Franco e Anderson Gomes.</t>
+        </is>
+      </c>
+      <c r="E67" s="24" t="inlineStr">
+        <is>
+          <t>Cumpre pena na Penitenciária Federal de Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F67" s="24" t="inlineStr">
+        <is>
+          <t>Vivo (preso)</t>
+        </is>
+      </c>
+      <c r="G67" s="24" t="inlineStr">
+        <is>
+          <t>Condenado pelo STF (56 anos); trânsito em julgado declarado em 13/07/2026.</t>
+        </is>
+      </c>
+      <c r="H67" s="24" t="inlineStr">
+        <is>
+          <t>Condenado</t>
+        </is>
+      </c>
+      <c r="I67" s="24" t="inlineStr">
+        <is>
+          <t>Preso na operação contra a milícia de Rio das Pedras e Muzema.</t>
+        </is>
+      </c>
+      <c r="J67" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K67" s="24" t="inlineStr">
+        <is>
+          <t>Moraes determina cumprimento das penas no caso Marielle (agenciabrasil.ebc.com.br) https://agenciabrasil.ebc.com.br/justica/noticia/2026-07/caso-marielle-moraes-determina-cumprimento-imediato-de-penas | Flávio homenageou em 2004 suspeito do caso Marielle (jb.com.br) https://www.jb.com.br/rio/2019/01/974171-flavio-bolsonaro-homenageou-em-2004-suspeito-de-participar-da-morte-de-marielle.html</t>
+        </is>
+      </c>
+      <c r="L67" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M67" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="24" t="inlineStr">
+        <is>
+          <t>orelha</t>
+        </is>
+      </c>
+      <c r="B68" s="24" t="inlineStr">
+        <is>
+          <t>Luís Carlos Felipe Martins (“Orelha”)</t>
+        </is>
+      </c>
+      <c r="C68" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D68" s="24" t="inlineStr">
+        <is>
+          <t>Não consegui confirmar em fonte pública a identidade nem o histórico de "Orelha" como descritos na planilha (ex-PM ligado à milícia de Rio das Pedras, homenageado por Flávio e morto em 2021). O nó fica sem perfil detalhado até haver fonte.</t>
+        </is>
+      </c>
+      <c r="E68" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F68" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G68" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H68" s="24" t="inlineStr">
+        <is>
+          <t>Não pesquisado</t>
+        </is>
+      </c>
+      <c r="I68" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J68" s="24" t="inlineStr">
+        <is>
+          <t>Identidade não confirmada: mais vale faltar do que atribuir algo à pessoa errada.</t>
+        </is>
+      </c>
+      <c r="K68" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L68" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M68" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="24" t="inlineStr">
+        <is>
+          <t>peixe</t>
+        </is>
+      </c>
+      <c r="B69" s="24" t="inlineStr">
+        <is>
+          <t>Robson Calixto (“Peixe”)</t>
+        </is>
+      </c>
+      <c r="C69" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D69" s="24" t="inlineStr">
+        <is>
+          <t>Robson Calixto da Fonseca, PM da reserva e ex-assessor de Domingos Brazão na Alerj e no TCE-RJ. Em fev/2026 o STF o condenou a 9 anos por integrar organização criminosa armada ligada ao assassinato de Marielle Franco; não foi condenado pelos homicídios. Segundo a PF, em out/2023 pediu a uma assessora de Flávio uma emenda de R$ 199 mil para o Instituto Ifop, paga em nov/2023.</t>
+        </is>
+      </c>
+      <c r="E69" s="24" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F69" s="24" t="inlineStr">
+        <is>
+          <t>Vivo (preso)</t>
+        </is>
+      </c>
+      <c r="G69" s="24" t="inlineStr">
+        <is>
+          <t>Condenado pelo STF a 9 anos (organização criminosa armada); trânsito em julgado em jul/2026. A PF apura a emenda.</t>
+        </is>
+      </c>
+      <c r="H69" s="24" t="inlineStr">
+        <is>
+          <t>Condenado</t>
+        </is>
+      </c>
+      <c r="I69" s="24" t="inlineStr">
+        <is>
+          <t>A PGR o descreveu como operador e intermediário dos irmãos Brazão.</t>
+        </is>
+      </c>
+      <c r="J69" s="24" t="inlineStr">
+        <is>
+          <t>Flávio diz que a emenda seguiu critérios técnicos e que a execução cabe ao beneficiário.</t>
+        </is>
+      </c>
+      <c r="K69" s="24" t="inlineStr">
+        <is>
+          <t>Quem é Peixe (tvtnews.com.br) https://tvtnews.com.br/?p=804271 | PF apura emenda de Flávio para ONG dos Brazão (infomoney.com.br) https://www.infomoney.com.br/politica/pf-apura-emenda-de-flavio-para-ong-suspeita-de-integrar-esquema-dos-irmaos-brazao/ | Penas do caso Marielle (agenciabrasil.ebc.com.br) https://agenciabrasil.ebc.com.br/justica/noticia/2026-07/caso-marielle-moraes-determina-cumprimento-imediato-de-penas</t>
+        </is>
+      </c>
+      <c r="L69" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M69" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="24" t="inlineStr">
+        <is>
+          <t>pms16</t>
+        </is>
+      </c>
+      <c r="B70" s="24" t="inlineStr">
+        <is>
+          <t>16 PMs denunciados</t>
+        </is>
+      </c>
+      <c r="C70" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D70" s="24" t="inlineStr">
+        <is>
+          <t>Grupo de policiais militares que receberam homenagens de Flávio e Carlos Bolsonaro e depois foram denunciados por organização criminosa ou ligação com milícias. Entre os casos documentados estão quatro PMs da Operação Quarto Elemento, denunciados por extorsão de comerciantes e mototaxistas. Os nomes individuais não são listados aqui.</t>
+        </is>
+      </c>
+      <c r="E70" s="24" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F70" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G70" s="24" t="inlineStr">
+        <is>
+          <t>Denunciados pelo MP-RJ; a situação varia caso a caso.</t>
+        </is>
+      </c>
+      <c r="H70" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I70" s="24" t="inlineStr">
+        <is>
+          <t>Parte do grupo é ligada a milícias, segundo o MP-RJ.</t>
+        </is>
+      </c>
+      <c r="J70" s="24" t="inlineStr">
+        <is>
+          <t>O total de 16 vem do vídeo de origem. A fonte reverificada nomeia seis homenageados denunciados e não confirma o total.</t>
+        </is>
+      </c>
+      <c r="K70" s="24" t="inlineStr">
+        <is>
+          <t>Entre medalhas e milícias (vermelho.org.br) https://vermelho.org.br/?p=740865 | Milicianos presos foram homenageados por Flávio na Alerj (istoe.com.br) https://istoe.com.br/milicianos-presos-no-rio-foram-homenageados-por-flavio-bolsonaro-na-alerj/</t>
+        </is>
+      </c>
+      <c r="L70" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M70" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="24" t="inlineStr">
+        <is>
+          <t>pmacusado</t>
+        </is>
+      </c>
+      <c r="B71" s="24" t="inlineStr">
+        <is>
+          <t>PM acusado de matar menina de 5 anos</t>
+        </is>
+      </c>
+      <c r="C71" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="inlineStr">
+        <is>
+          <t>Policial militar denunciado pelo MP-RJ por um disparo de fuzil que matou uma criança de 5 anos durante patrulha em Niterói, em fev/2021. Flávio integrou a defesa e assinou um recurso ao STJ em 2024 para evitar o júri popular. O STJ negou o recurso, e o PM aguarda o júri.</t>
+        </is>
+      </c>
+      <c r="E71" s="24" t="inlineStr">
+        <is>
+          <t>Niterói (RJ)</t>
+        </is>
+      </c>
+      <c r="F71" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G71" s="24" t="inlineStr">
+        <is>
+          <t>Réu; pronunciado a júri popular, sem mais recursos. A prisão preventiva foi revogada em nov/2021.</t>
+        </is>
+      </c>
+      <c r="H71" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I71" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J71" s="24" t="inlineStr">
+        <is>
+          <t>Por envolver uma criança, o mapa não traz o nome da vítima. A defesa do PM diz que ele reagiu a um ataque; o MP-RJ diz que não houve confronto.</t>
+        </is>
+      </c>
+      <c r="K71" s="24" t="inlineStr">
+        <is>
+          <t>Flávio atuou na defesa de PM acusado (iclnoticias.com.br) https://iclnoticias.com.br/flavio-bolsonaro-defesa-pm-acusado-matar-menina/ | Flávio advogou para PM (eshoje.com.br) https://eshoje.com.br/brasil/2026/10/flavio-advogou-para-pm/</t>
+        </is>
+      </c>
+      <c r="L71" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M71" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="24" t="inlineStr">
+        <is>
+          <t>cirorocha</t>
+        </is>
+      </c>
+      <c r="B72" s="24" t="inlineStr">
+        <is>
+          <t>Ciro Rocha Soares</t>
+        </is>
+      </c>
+      <c r="C72" s="24" t="inlineStr">
+        <is>
+          <t>Vorcaro e o Banco Master</t>
+        </is>
+      </c>
+      <c r="D72" s="24" t="inlineStr">
+        <is>
+          <t>Advogado baiano, sócio da Rocha Soares Advogados Associados (Salvador) e ex-ouvidor do Ministério do Turismo (2016-2017). Em mensagens obtidas pela PF aparece articulando, com Cezinha de Madureira, a aproximação de Vorcaro com Mendonça: em 08/02/2025 mandou foto e áudio dizendo que levara o ministro a uma alfaiataria "trabalhando por você".</t>
+        </is>
+      </c>
+      <c r="E72" s="24" t="inlineStr">
+        <is>
+          <t>Salvador (BA)</t>
+        </is>
+      </c>
+      <c r="F72" s="24" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="G72" s="24" t="inlineStr">
+        <is>
+          <t>Não há acusação contra ele nas fontes.</t>
+        </is>
+      </c>
+      <c r="H72" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I72" s="24" t="inlineStr">
+        <is>
+          <t>Nada nas fontes.</t>
+        </is>
+      </c>
+      <c r="J72" s="24" t="inlineStr">
+        <is>
+          <t>Ele diz que não há irregularidade em pedir conversas com magistrados e que Vorcaro não era investigado em fev/2025.</t>
+        </is>
+      </c>
+      <c r="K72" s="24" t="inlineStr">
+        <is>
+          <t>Mensagens e áudios inéditos sobre Mendonça (iclnoticias.com.br) https://iclnoticias.com.br/vaza-mendonca-mensagens-e-audios-ineditos/ | Áudios revelam encontro entre Vorcaro e Mendonça (bahianoticias.com.br) https://www.bahianoticias.com.br/justica/noticia/75274-audios-e-mensagens-revelam-encontro-entre-vorcaro-e-mendonca-ministro-admite-e-diz-que-se-limitou-a-ouvi-lo</t>
+        </is>
+      </c>
+      <c r="L72" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M72" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="24" t="inlineStr">
+        <is>
+          <t>ong</t>
+        </is>
+      </c>
+      <c r="B73" s="24" t="inlineStr">
+        <is>
+          <t>ONG e produtora do filme</t>
+        </is>
+      </c>
+      <c r="C73" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D73" s="24" t="inlineStr">
+        <is>
+          <t>Entidades ligadas a Karina Ferreira da Gama, sócia da GoUp, produtora do filme Dark Horse, sobre Jair Bolsonaro: o Instituto Conhecer Brasil e a Associação (ou Academia) Nacional de Cultura. Receberam emendas de deputados paulistas. Segundo o Intercept, houve negociação de US$ 24 mi de Vorcaro para o filme; Flávio admitiu ter recebido mais de US$ 12 mi, que chama de "patrocínio".</t>
+        </is>
+      </c>
+      <c r="E73" s="24" t="inlineStr">
+        <is>
+          <t>Av. Paulista, São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F73" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="24" t="inlineStr">
+        <is>
+          <t>Flávio é investigado no STF pelo dinheiro do filme (relator André Mendonça). A Prefeitura de SP pediu explicações a uma das entidades sobre despesas.</t>
+        </is>
+      </c>
+      <c r="H73" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I73" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J73" s="24" t="inlineStr">
+        <is>
+          <t>Karina diz que Vorcaro foi intermediário e que o dinheiro veio do fundo Heavengate, do Texas. O papel de tesoureiro de fachada atribuído ao eletricista vem do vídeo e não foi reverificado.</t>
+        </is>
+      </c>
+      <c r="K73" s="24" t="inlineStr">
+        <is>
+          <t>Produtora diz que filme já custou R$ 65,7 mi (oliberal.com) https://www.oliberal.com/politica/produtora-diz-que-filme-de-bolsonaro-ja-custou-r-65-7-milhoes-vorcaro-bancou-90-do-custo-1.1123519 | Deputados indicaram R$ 700 mil a entidades da produtora (cnnbrasil.com.br) https://www.cnnbrasil.com.br/politica/deputados-de-sp-indicaram-r-700-mil-a-entidades-da-produtora-de-dark-horse/ | Prefeitura pede explicações a ONG ligada a Dark Horse (dgabc.com.br) https://www.dgabc.com.br/Noticia/4334231/prefeitura-de-sp-pede-explicacoes-a-ong-ligada-a-dark-horse-por-despesas-de-rs-13-4-milhoes</t>
+        </is>
+      </c>
+      <c r="L73" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M73" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="24" t="inlineStr">
+        <is>
+          <t>bestbet</t>
+        </is>
+      </c>
+      <c r="B74" s="24" t="inlineStr">
+        <is>
+          <t>Best Bet (Rede Loto)</t>
+        </is>
+      </c>
+      <c r="C74" s="24" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="D74" s="24" t="inlineStr">
+        <is>
+          <t>Nome fantasia da Rede Loto, registrada em SP em fev/2023 e licenciada pela Loterj em 25/05/2023, a primeira bet autorizada no país. A única acionista é a Cathedral Holdings, de Willer Tomaz e sócios. A PF apura se Willer controla a empresa de fato e encontrou canhotos de voos de Flávio na Europa (2025) pagos via Cathedral.</t>
+        </is>
+      </c>
+      <c r="E74" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F74" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="24" t="inlineStr">
+        <is>
+          <t>Citada no inquérito enviado ao STF em out/2026 (relator Moraes).</t>
+        </is>
+      </c>
+      <c r="H74" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I74" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J74" s="24" t="inlineStr">
+        <is>
+          <t>A defesa diz que a bet nunca chegou a operar e que os voos foram pagos por Willer, como passeios entre famílias.</t>
+        </is>
+      </c>
+      <c r="K74" s="24" t="inlineStr">
+        <is>
+          <t>Bet de investigado pagou voos de Flávio (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/10/11726788-bet-de-investigado-por-fraude-no-inss-pagou-voos-de-flavio-bolsonaro-na-europa-aponta-pf.html | Segundo inquérito contra Flávio no STF (oliberal.com) https://www.oliberal.com/politica/flavio-e-investigado-em-2-inquerito-no-stf-para-apurar-suspeitas-de-lavagem-com-advogado-1.1183991</t>
+        </is>
+      </c>
+      <c r="L74" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M74" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="24" t="inlineStr">
+        <is>
+          <t>cathedral</t>
+        </is>
+      </c>
+      <c r="B75" s="24" t="inlineStr">
+        <is>
+          <t>Cathedral Holdings</t>
+        </is>
+      </c>
+      <c r="C75" s="24" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="D75" s="24" t="inlineStr">
+        <is>
+          <t>Cathedral Holdings S.A., aberta na Ilha da Madeira (Portugal) em jan/2023 só com sócios brasileiros: Willer Tomaz, a mulher e a irmã dele, Jorge Barbosa Dias e um parente de Dias. É a única acionista da Rede Loto (Best Bet). Segundo a PF, pagou voos de Flávio e da mulher entre Lisboa, Cascais, Nice e Paris em abr e mai/2025.</t>
+        </is>
+      </c>
+      <c r="E75" s="24" t="inlineStr">
+        <is>
+          <t>Funchal, Ilha da Madeira (Portugal)</t>
+        </is>
+      </c>
+      <c r="F75" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G75" s="24" t="inlineStr">
+        <is>
+          <t>Citada no inquérito da PF sobre Flávio e Willer (STF, out/2026).</t>
+        </is>
+      </c>
+      <c r="H75" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I75" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J75" s="24" t="inlineStr">
+        <is>
+          <t>Dias foi processado por jogo ilegal e lavagem em 2022 e absolvido em 2023. A defesa diz que os voos foram pagos por Willer.</t>
+        </is>
+      </c>
+      <c r="K75" s="24" t="inlineStr">
+        <is>
+          <t>Bet de investigado pagou voos de Flávio (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/10/11726788-bet-de-investigado-por-fraude-no-inss-pagou-voos-de-flavio-bolsonaro-na-europa-aponta-pf.html | Bet de investigado pagou voos de Flávio, aponta PF (bahianoticias.com.br) https://www.bahianoticias.com.br/folha/noticia/412847-bet-de-investigado-por-fraude-do-inss-pagou-voos-de-flavio-bolsonaro-na-europa</t>
+        </is>
+      </c>
+      <c r="L75" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M75" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="24" t="inlineStr">
+        <is>
+          <t>bravo</t>
+        </is>
+      </c>
+      <c r="B76" s="24" t="inlineStr">
+        <is>
+          <t>Bravo Grafeno</t>
+        </is>
+      </c>
+      <c r="C76" s="24" t="inlineStr">
+        <is>
+          <t>Esquema do INSS</t>
+        </is>
+      </c>
+      <c r="D76" s="24" t="inlineStr">
+        <is>
+          <t>Fábrica de capacetes aberta em jun/2024, com capital de R$ 100 mil, que tem como sócios Flávio e Carlos Bolsonaro (Jair já foi sócio e é garoto-propaganda). Está registrada na sala 2601 de um edifício em Águas Claras (DF), mesmo endereço de ao menos 16 empresas ligadas ao Careca do INSS, e usa o mesmo contador, Alexandre Caetano dos Reis.</t>
+        </is>
+      </c>
+      <c r="E76" s="24" t="inlineStr">
+        <is>
+          <t>Águas Claras (DF)</t>
+        </is>
+      </c>
+      <c r="F76" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G76" s="24" t="inlineStr">
+        <is>
+          <t>Não há acusação contra a empresa nas fontes.</t>
+        </is>
+      </c>
+      <c r="H76" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I76" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J76" s="24" t="inlineStr">
+        <is>
+          <t>O escritório do contador diz que a sala é um coworking de outra empresa. Flávio nega envolvimento com o caso INSS.</t>
+        </is>
+      </c>
+      <c r="K76" s="24" t="inlineStr">
+        <is>
+          <t>Empresas de Flávio e do Careca dividem a mesma sala (brasildefato.com.br) https://www.brasildefato.com.br/2026/09/11/empresas-de-flavio-bolsonaro-e-careca-do-inss-dividem-a-mesma-sala-em-brasilia/ | Mesma sala e mesmo contador (bahianoticias.com.br) https://www.bahianoticias.com.br/noticia/321055-empresas-de-flavio-bolsonaro-e-do-careca-do-inss-dividem-a-mesma-sala-e-possuem-o-mesmo-contador</t>
+        </is>
+      </c>
+      <c r="L76" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M76" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="24" t="inlineStr">
+        <is>
+          <t>escf</t>
+        </is>
+      </c>
+      <c r="B77" s="24" t="inlineStr">
+        <is>
+          <t>Escritório de advocacia de Flávio</t>
+        </is>
+      </c>
+      <c r="C77" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D77" s="24" t="inlineStr">
+        <is>
+          <t>Banca de advocacia de Flávio, ativa desde 2021 e com sede na casa do senador, em Brasília. É administrada à distância por Letícia Caetano dos Reis, e a contabilidade é feita pelo escritório do irmão dela, Alexandre. Em abr/2025 emitiu nota de R$ 500 mil por "assessoria jurídica" a uma empresa ligada a uma consultoria que recebeu R$ 58 mi do Master.</t>
+        </is>
+      </c>
+      <c r="E77" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F77" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G77" s="24" t="inlineStr">
+        <is>
+          <t>Não há acusação contra o escritório nas fontes. Figura em ao menos 18 processos.</t>
+        </is>
+      </c>
+      <c r="H77" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I77" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J77" s="24" t="inlineStr">
+        <is>
+          <t>Flávio alega sigilo profissional e não revela os clientes.</t>
+        </is>
+      </c>
+      <c r="K77" s="24" t="inlineStr">
+        <is>
+          <t>Escritório de Flávio que emitiu nota de R$ 500 mil (tribunadosertao.com.br) https://www.tribunadosertao.com.br/poder-e-governo/2026/07/26/946935-escritorio-de-advocacia-de-flavio-que-emitiu-nota-de-r-500-mil-tem-atuacao-discreta-e-gestao-a-distancia | Firma de advocacia de Flávio (apublica.org) https://apublica.org/2022/06/firma-de-advocacia-de-flavio-bolsonaro-tem-contratos-consideraveis-diz-administradora/</t>
+        </is>
+      </c>
+      <c r="L77" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M77" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="24" t="inlineStr">
+        <is>
+          <t>consult</t>
+        </is>
+      </c>
+      <c r="B78" s="24" t="inlineStr">
+        <is>
+          <t>Consultoria do amigo de Nunes</t>
+        </is>
+      </c>
+      <c r="C78" s="24" t="inlineStr">
+        <is>
+          <t>Poder e Justiça</t>
+        </is>
+      </c>
+      <c r="D78" s="24" t="inlineStr">
+        <is>
+          <t>Consult Inteligência Tributária. Segundo relatório do Coaf, recebeu R$ 6,6 mi do Banco Master e R$ 11,3 mi da JBS entre 2024 e 2025, e repassou R$ 281,6 mil, em 11 parcelas, ao escritório de Kevin Marques, filho do ministro Nunes Marques.</t>
+        </is>
+      </c>
+      <c r="E78" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G78" s="24" t="inlineStr">
+        <is>
+          <t>Aparece em relatório do Coaf sobre movimentações atípicas; sem acusação formal nas fontes.</t>
+        </is>
+      </c>
+      <c r="H78" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I78" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J78" s="24" t="inlineStr">
+        <is>
+          <t>As reportagens não nomeiam o dono, e a ligação "amigo de Nunes" vem do vídeo de origem, sem confirmação. A defesa de Kevin diz que ele prestou serviços tributários e nunca recebeu direto das empresas. A JBS diz que contrata consultorias pela complexidade tributária.</t>
+        </is>
+      </c>
+      <c r="K78" s="24" t="inlineStr">
+        <is>
+          <t>Quem é Kevin Nunes Marques (istoe.com.br) https://istoe.com.br/quem-e-kelvin-nunes-marques-filho-do-ministro-do-stf-que-diz | Consultoria ligada ao Master e à JBS contratou filho de Nunes Marques (metropoles.com) https://www.metropoles.com/brasil/consultoria-ligada-ao-master-e-a-jbs-contratou-filho-de-nunes-marques</t>
+        </is>
+      </c>
+      <c r="L78" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M78" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="24" t="inlineStr">
+        <is>
+          <t>riopag</t>
+        </is>
+      </c>
+      <c r="B79" s="24" t="inlineStr">
+        <is>
+          <t>Rio Pag</t>
+        </is>
+      </c>
+      <c r="C79" s="24" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="D79" s="24" t="inlineStr">
+        <is>
+          <t>Intermediadora de pagamentos (depósitos e saques) das bets licenciadas pela Loterj, contratada em 2023. Faturou R$ 187,8 mi em taxas entre jun/2023 e ago/2026. A única acionista é a Capital Pretium, representada por Lídia Mazelli. Em e-mail achado pela PF, Willer se apresentou como sócio.</t>
+        </is>
+      </c>
+      <c r="E79" s="24" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F79" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="24" t="inlineStr">
+        <is>
+          <t>A Loterj rescindiu o contrato em 22/09/2026 e cobra R$ 9,4 mi, acusando a empresa de reter R$ 20,9 mi; três dias depois uma liminar suspendeu a rescisão.</t>
+        </is>
+      </c>
+      <c r="H79" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I79" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J79" s="24" t="inlineStr">
+        <is>
+          <t>Willer nega ser sócio ou gestor e diz que a relação é só de advogado. Antes dizia não ter participação; depois admitiu participação indireta (O Globo).</t>
+        </is>
+      </c>
+      <c r="K79" s="24" t="inlineStr">
+        <is>
+          <t>Empresa ligada a amigo de Flávio faturou R$ 187,8 mi (ncnews.com.br) https://ncnews.com.br/?p=55340 | Loterj rescinde contrato com a RioPag (bnldata.com.br) https://bnldata.com.br/loterj-rescinde-contrato-com-riopag-e-cobra-r-94-mi-da-empresa/</t>
+        </is>
+      </c>
+      <c r="L79" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M79" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="24" t="inlineStr">
+        <is>
+          <t>luri</t>
+        </is>
+      </c>
+      <c r="B80" s="24" t="inlineStr">
+        <is>
+          <t>Allure Eventos</t>
+        </is>
+      </c>
+      <c r="C80" s="24" t="inlineStr">
+        <is>
+          <t>Vorcaro e o Banco Master</t>
+        </is>
+      </c>
+      <c r="D80" s="24" t="inlineStr">
+        <is>
+          <t>Allure Eventos, agência de eventos de Felipe Nisti Cataldo. Segundo o UOL, recrutava mulheres, inclusive estrangeiras, para festas privadas de Vorcaro no Brasil e no exterior. Mensagens indicam Vorcaro como sócio oculto, e um contrato de dez/2023 previa a compra de 50% da agência por R$ 1,5 mi.</t>
+        </is>
+      </c>
+      <c r="E80" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F80" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G80" s="24" t="inlineStr">
+        <is>
+          <t>A PF abriu inquérito em mai/2026 sobre a contratação das estrangeiras.</t>
+        </is>
+      </c>
+      <c r="H80" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I80" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J80" s="24" t="inlineStr">
+        <is>
+          <t>O nó se chamava "Luri Eventos", provável erro de transcrição do vídeo; as reportagens grafam Allure Eventos (confirmado em 22/10/2026). O dono confirma o interesse de Vorcaro, mas nega que a compra tenha avançado e contesta a versão das mensagens. Uma das reportagens não afirma explicitamente que a Allure é a agência usada no recrutamento.</t>
+        </is>
+      </c>
+      <c r="K80" s="24" t="inlineStr">
+        <is>
+          <t>Mensagens apontam Vorcaro como sócio de agência (maisgoias.com.br) https://www.maisgoias.com.br/brasil/justica/mensagens-apontam-vorcaro-como-socio-de-agencia-que-recrutava-refugiadas-para-prostituicao/ | Mensagens ligam Vorcaro a recrutamento (jornalopcao.com.br) https://www.jornalopcao.com.br/ultimas-noticias/daniel-vorcaro-esquema-prostituicao-878361/ | Mensagens ligam Vorcaro a esquema de recrutamento (acritica.net) https://acritica.net/policia/mensagens-ligam-daniel-vorcaro-a-esquema-de-prostituicao-e-recrutamento-de-refugiadas/</t>
+        </is>
+      </c>
+      <c r="L80" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M80" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo). 22/10/2026: renomeado de "Luri Eventos" para "Allure Eventos".</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="24" t="inlineStr">
+        <is>
+          <t>ongbrazao</t>
+        </is>
+      </c>
+      <c r="B81" s="24" t="inlineStr">
+        <is>
+          <t>ONG ligada aos irmãos Brazão</t>
+        </is>
+      </c>
+      <c r="C81" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D81" s="24" t="inlineStr">
+        <is>
+          <t>Instituto de Formação Profissional José Carlos Procópio (Ifop), numa sala comercial em Taquara, Zona Oeste do Rio, área de influência dos Brazão. Recebeu R$ 199 mil de emenda de Flávio em 29/11/2023 para um projeto de futebol infantil. A PF apura se o repasse fez parte de um esquema de desvio de verbas de entidades ligadas aos Brazão, que teriam recebido R$ 268 mi entre 2020 e 2024.</t>
+        </is>
+      </c>
+      <c r="E81" s="24" t="inlineStr">
+        <is>
+          <t>Taquara, Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F81" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G81" s="24" t="inlineStr">
+        <is>
+          <t>Investigação da PF em andamento; sem denúncia nas fontes.</t>
+        </is>
+      </c>
+      <c r="H81" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I81" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J81" s="24" t="inlineStr">
+        <is>
+          <t>O Ifop nega relação com Peixe ou com os Brazão e diz que prestou contas ao Ministério do Esporte e devolveu o que sobrou.</t>
+        </is>
+      </c>
+      <c r="K81" s="24" t="inlineStr">
+        <is>
+          <t>PF apura emenda de Flávio para ONG dos Brazão (infomoney.com.br) https://www.infomoney.com.br/politica/pf-apura-emenda-de-flavio-para-ong-suspeita-de-integrar-esquema-dos-irmaos-brazao/ | Quem é Peixe (tvtnews.com.br) https://tvtnews.com.br/?p=804271</t>
+        </is>
+      </c>
+      <c r="L81" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M81" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="24" t="inlineStr">
+        <is>
+          <t>kopenhagen</t>
+        </is>
+      </c>
+      <c r="B82" s="24" t="inlineStr">
+        <is>
+          <t>Loja Kopenhagen de Flávio</t>
+        </is>
+      </c>
+      <c r="C82" s="24" t="inlineStr">
+        <is>
+          <t>Flávio e família</t>
+        </is>
+      </c>
+      <c r="D82" s="24" t="inlineStr">
+        <is>
+          <t>Franquia de chocolates no Shopping Via Parque (Barra da Tijuca), da empresa Bolsotini Chocolates e Café, de Flávio e do sócio Alexandre Santini, comprada entre 2014 e 2015. O MP-RJ suspeitou que a loja servia para lavar dinheiro da rachadinha, com até R$ 2,1 mi "legalizados" e depósitos em espécie desproporcionais ao faturamento. A operação foi repassada ao grupo CRM em fev/2021.</t>
+        </is>
+      </c>
+      <c r="E82" s="24" t="inlineStr">
+        <is>
+          <t>Barra da Tijuca, Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="F82" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G82" s="24" t="inlineStr">
+        <is>
+          <t>Fazia parte da denúncia da rachadinha, que perdeu efeito com as anulações de provas.</t>
+        </is>
+      </c>
+      <c r="H82" s="24" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+      <c r="I82" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J82" s="24" t="inlineStr">
+        <is>
+          <t>Flávio nega crime e diz que as operações da loja eram legais. A marca Kopenhagen não é parte do caso; por isso o nó fica sem logo.</t>
+        </is>
+      </c>
+      <c r="K82" s="24" t="inlineStr">
+        <is>
+          <t>Flávio entrega loja investigada pelo MP (poder360.com.br) https://www.poder360.com.br/brasil/flavio-bolsonaro-entrega-loja-de-chocolates-investigada-pelo-mp/ | Investigação apura se loja lavou R$ 2,1 mi (opovo.com.br) https://www.opovo.com.br/noticias/politica/2020/08/20/investigacao-apura-se-loja-de-flavio-bolsonaro--lavou--r--2-1-milhoes.html</t>
+        </is>
+      </c>
+      <c r="L82" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M82" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="24" t="inlineStr">
+        <is>
+          <t>santander</t>
+        </is>
+      </c>
+      <c r="B83" s="24" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="C83" s="24" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="D83" s="24" t="inlineStr">
+        <is>
+          <t>Banco onde a Alcazar Holdings, de Willer Tomaz, mantinha conta. Segundo a PF e a piauí, Flávio aparecia como "usuário master" dessa conta, e um e-mail da secretária de Willer em 22/05/2025 pediu ao banco a exclusão dele, confirmada no mesmo dia.</t>
+        </is>
+      </c>
+      <c r="E83" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F83" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G83" s="24" t="inlineStr">
+        <is>
+          <t>O banco não é investigado; a conta é citada no inquérito sobre Flávio e Willer.</t>
+        </is>
+      </c>
+      <c r="H83" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I83" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J83" s="24" t="inlineStr">
+        <is>
+          <t>Willer atribui o vínculo a um erro cadastral do banco.</t>
+        </is>
+      </c>
+      <c r="K83" s="24" t="inlineStr">
+        <is>
+          <t>Flávio era usuário master de conta de offshore (maisgoias.com.br) https://www.maisgoias.com.br/brasil/flavio-bolsonaro-era-usuario-master-de-conta-de-offshore-socia-do-jato-usado-por-vorcaro/ | Offshore ligada a Flávio (jornalopcao.com.br) https://www.jornalopcao.com.br/ultimas-noticias/offshore-ligada-a-flavio-bolsonaro-reune-conexoes-com-o-mercado-de-bets-879306/</t>
+        </is>
+      </c>
+      <c r="L83" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M83" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N83" s="24" t="inlineStr">
+        <is>
+          <t>santander.png</t>
+        </is>
+      </c>
+      <c r="O83" s="24" t="inlineStr">
+        <is>
+          <t>Interbrand · domínio público (logo simples, sem direito autoral)</t>
+        </is>
+      </c>
+      <c r="P83" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Banco_Santander_Logotipo.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="24" t="inlineStr">
+        <is>
+          <t>bets</t>
+        </is>
+      </c>
+      <c r="B84" s="24" t="inlineStr">
+        <is>
+          <t>Blaze e sites de apostas</t>
+        </is>
+      </c>
+      <c r="C84" s="24" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="D84" s="24" t="inlineStr">
+        <is>
+          <t>Plataforma de apostas Blaze. Segundo o Metrópoles, Willer Tomaz movimentou cerca de R$ 5 bi em apostas de cassino on-line nela em 2025, com prejuízo líquido de R$ 163 mi. Ele foi à Justiça de SP alegando vício e cobrando a plataforma. A PF abriu frente de investigação sobre possível lavagem por apostas.</t>
+        </is>
+      </c>
+      <c r="E84" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F84" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G84" s="24" t="inlineStr">
+        <is>
+          <t>A plataforma não é acusada nas fontes. A Justiça de SP negou o pedido de ressarcimento de Willer.</t>
+        </is>
+      </c>
+      <c r="H84" s="24" t="inlineStr">
+        <is>
+          <t>Citado, sem acusação</t>
+        </is>
+      </c>
+      <c r="I84" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J84" s="24" t="inlineStr">
+        <is>
+          <t>Willer nega lavagem e diz que tudo passou pela própria conta, de forma rastreável. As fontes divergem sobre o valor cobrado na ação (R$ 20 mi ou R$ 163 mi).</t>
+        </is>
+      </c>
+      <c r="K84" s="24" t="inlineStr">
+        <is>
+          <t>Willer movimenta R$ 5 bi em apostas (bahianoticias.com.br) https://www.bahianoticias.com.br/noticia/321709-advogado-willer-tomaz-movimenta-r-5-bi-em-apostas-e-registra-prejuizo-de-r-163-mi | Justiça de SP nega ressarcimento a Willer (bnldata.com.br) https://bnldata.com.br/?p=189317</t>
+        </is>
+      </c>
+      <c r="L84" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M84" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+      <c r="N84" s="24" t="inlineStr">
+        <is>
+          <t>bets.png</t>
+        </is>
+      </c>
+      <c r="O84" s="24" t="inlineStr">
+        <is>
+          <t>blaze.com · domínio público (logo simples, sem direito autoral)</t>
+        </is>
+      </c>
+      <c r="P84" s="24" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Blaze_apostas_logo.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="24" t="inlineStr">
+        <is>
+          <t>aptosp</t>
+        </is>
+      </c>
+      <c r="B85" s="24" t="inlineStr">
+        <is>
+          <t>Apartamento de luxo em SP</t>
+        </is>
+      </c>
+      <c r="C85" s="24" t="inlineStr">
+        <is>
+          <t>Casas e ativos</t>
+        </is>
+      </c>
+      <c r="D85" s="24" t="inlineStr">
+        <is>
+          <t>Apartamento de 159 m² em São Paulo. Fabiano Zettel, cunhado de Vorcaro, comprou em abr/2025 por R$ 5,5 mi e vendeu em fev/2026 à WT, de Willer, por R$ 3,5 mi. Segundo a piauí, Flávio ficou lá por vários dias em ago/2026, onde se reuniu com a equipe e gravou vídeos de campanha.</t>
+        </is>
+      </c>
+      <c r="E85" s="24" t="inlineStr">
+        <is>
+          <t>São Paulo (SP)</t>
+        </is>
+      </c>
+      <c r="F85" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G85" s="24" t="inlineStr">
+        <is>
+          <t>Não há processo sobre o imóvel nas fontes.</t>
+        </is>
+      </c>
+      <c r="H85" s="24" t="inlineStr">
+        <is>
+          <t>Bem citado</t>
+        </is>
+      </c>
+      <c r="I85" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J85" s="24" t="inlineStr">
+        <is>
+          <t>Flávio disse à piauí que só se hospedou em hotéis da região. Willer diz não conhecer Zettel nem Vorcaro.</t>
+        </is>
+      </c>
+      <c r="K85" s="24" t="inlineStr">
+        <is>
+          <t>Flávio usou em campanha imóvel de advogado alvo da PF (diariodocomercio.com.br) https://diariodocomercio.com.br/politica/flavio-bolsonaro-apartamento-pf/ | Apartamento pertenceu a cunhado de Vorcaro (timesbrasil.com.br) https://timesbrasil.com.br/brasil/apartamento-usado-por-flavio-bolsonaro-durante-campanha-eleitoral-pertenceu-a-cunhado-de-daniel-vorcaro/</t>
+        </is>
+      </c>
+      <c r="L85" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M85" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="24" t="inlineStr">
+        <is>
+          <t>atibaia</t>
+        </is>
+      </c>
+      <c r="B86" s="24" t="inlineStr">
+        <is>
+          <t>Casa de Wassef em Atibaia</t>
+        </is>
+      </c>
+      <c r="C86" s="24" t="inlineStr">
+        <is>
+          <t>Casas e ativos</t>
+        </is>
+      </c>
+      <c r="D86" s="24" t="inlineStr">
+        <is>
+          <t>Casa do advogado Frederick Wassef, que defendia Flávio e Jair Bolsonaro, em Atibaia (SP). Fabrício Queiroz foi preso lá em 18/06/2020, na Operação Anjo, desdobramento da Furna da Onça.</t>
+        </is>
+      </c>
+      <c r="E86" s="24" t="inlineStr">
+        <is>
+          <t>Atibaia (SP)</t>
+        </is>
+      </c>
+      <c r="F86" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G86" s="24" t="inlineStr">
+        <is>
+          <t>Não há processo sobre o imóvel.</t>
+        </is>
+      </c>
+      <c r="H86" s="24" t="inlineStr">
+        <is>
+          <t>Bem citado</t>
+        </is>
+      </c>
+      <c r="I86" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J86" s="24" t="inlineStr">
+        <is>
+          <t>Wassef negou ter escondido Queiroz.</t>
+        </is>
+      </c>
+      <c r="K86" s="24" t="inlineStr">
+        <is>
+          <t>Queiroz é preso em Atibaia (poder360.com.br) https://www.poder360.com.br/justica/fabricio-queiroz-ex-assessor-de-flavio-bolsonaro-e-preso/ | Advogado de Bolsonaro diz que não escondeu Queiroz (poder360.com.br) https://poder360.com.br/justica/advogado-de-bolsonaro-diz-que-nao-escondeu-queiroz-e-nega-ser-o-anjo/</t>
+        </is>
+      </c>
+      <c r="L86" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M86" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="24" t="inlineStr">
+        <is>
+          <t>mansaobsb</t>
+        </is>
+      </c>
+      <c r="B87" s="24" t="inlineStr">
+        <is>
+          <t>Mansão de Flávio em Brasília</t>
+        </is>
+      </c>
+      <c r="C87" s="24" t="inlineStr">
+        <is>
+          <t>Casas e ativos</t>
+        </is>
+      </c>
+      <c r="D87" s="24" t="inlineStr">
+        <is>
+          <t>Casa comprada por Flávio em 2021 por R$ 6 mi, num terreno de 2.400 m² no Setor de Mansões Dom Bosco (Lago Sul). Foram R$ 2,87 mi de entrada e R$ 3,1 mi financiados pelo BRB a 3,71% ao ano, abaixo da média do banco; ele quitou em cerca de três anos. Também abriga o escritório de advocacia dele.</t>
+        </is>
+      </c>
+      <c r="E87" s="24" t="inlineStr">
+        <is>
+          <t>Lago Sul, Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F87" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G87" s="24" t="inlineStr">
+        <is>
+          <t>A PF apura as condições do empréstimo dentro do inquérito BRB-Master.</t>
+        </is>
+      </c>
+      <c r="H87" s="24" t="inlineStr">
+        <is>
+          <t>Bem citado</t>
+        </is>
+      </c>
+      <c r="I87" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J87" s="24" t="inlineStr">
+        <is>
+          <t>Flávio diz que a compra foi legal, paga com a venda de outro imóvel e da loja de chocolates.</t>
+        </is>
+      </c>
+      <c r="K87" s="24" t="inlineStr">
+        <is>
+          <t>PF apura financiamento do BRB a Flávio (diariodepernambuco.com.br) https://www.diariodepernambuco.com.br/politica/2026/10/11725606-pf-apura-condicoes-de-financiamento-do-brb-a-flavio-bolsonaro-para-mansao-de-rs-6-milhoes.html | PF investiga financiamento de mansão de Flávio (jb.com.br) https://www.jb.com.br/brasil/policia/2026/10/1061098-pf-investiga-financiamento-de-mansao-de-flavio-bolsonaro-em-brasilia.html</t>
+        </is>
+      </c>
+      <c r="L87" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M87" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="24" t="inlineStr">
+        <is>
+          <t>hangar</t>
+        </is>
+      </c>
+      <c r="B88" s="24" t="inlineStr">
+        <is>
+          <t>Hangares de Willer (Aeroporto de Brasília)</t>
+        </is>
+      </c>
+      <c r="C88" s="24" t="inlineStr">
+        <is>
+          <t>Casas e ativos</t>
+        </is>
+      </c>
+      <c r="D88" s="24" t="inlineStr">
+        <is>
+          <t>Hangares 36 e 37 do Aeroporto de Brasília, operados por empresas de aviação de Willer Tomaz (Ícaro Aviation e Jet Line). Na busca de ago/2026 da Operação Sem Desconto, a PF encontrou uma sala oculta, máquina de contar e malas vazias, sem dinheiro.</t>
+        </is>
+      </c>
+      <c r="E88" s="24" t="inlineStr">
+        <is>
+          <t>Aeroporto de Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F88" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G88" s="24" t="inlineStr">
+        <is>
+          <t>Alvo de busca na Operação Sem Desconto (ago/2026).</t>
+        </is>
+      </c>
+      <c r="H88" s="24" t="inlineStr">
+        <is>
+          <t>Bem citado</t>
+        </is>
+      </c>
+      <c r="I88" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J88" s="24" t="inlineStr">
+        <is>
+          <t>Willer nega uso irregular e diz que o espaço atende transporte de valores.</t>
+        </is>
+      </c>
+      <c r="K88" s="24" t="inlineStr">
+        <is>
+          <t>Empresas e hangar de Willer (iclnoticias.com.br) https://iclnoticias.com.br/domestica-preside-empresas-fraude-flavio/ | PF mira advogado camaleão de Brasília (opovo.com.br) https://www.opovo.com.br/noticias/economia/2026/08/04/fraudes-do-inss-pf-mira-advogado-camaleao-de-brasilia-por-suspeita-de-lavagem-para-senador.html</t>
+        </is>
+      </c>
+      <c r="L88" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M88" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="24" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B89" s="24" t="inlineStr">
+        <is>
+          <t>Sala em Águas Claras (DF)</t>
+        </is>
+      </c>
+      <c r="C89" s="24" t="inlineStr">
+        <is>
+          <t>Esquema do INSS</t>
+        </is>
+      </c>
+      <c r="D89" s="24" t="inlineStr">
+        <is>
+          <t>Sala 2601 de um edifício comercial em Águas Claras (DF). É o endereço de ao menos 16 empresas ligadas ao Careca do INSS, oito delas abertas no mesmo dia (05/10/2023), e da Bravo Grafeno, de Flávio e Carlos. Uma das empresas do Careca, a Prospect, recebeu R$ 204,2 mi de entidades, segundo a CPMI do INSS.</t>
+        </is>
+      </c>
+      <c r="E89" s="24" t="inlineStr">
+        <is>
+          <t>Águas Claras (DF)</t>
+        </is>
+      </c>
+      <c r="F89" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G89" s="24" t="inlineStr">
+        <is>
+          <t>Várias empresas do endereço são investigadas no caso INSS; algumas foram baixadas.</t>
+        </is>
+      </c>
+      <c r="H89" s="24" t="inlineStr">
+        <is>
+          <t>Bem citado</t>
+        </is>
+      </c>
+      <c r="I89" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J89" s="24" t="inlineStr">
+        <is>
+          <t>O escritório do contador diz que a sala é um coworking de outra empresa.</t>
+        </is>
+      </c>
+      <c r="K89" s="24" t="inlineStr">
+        <is>
+          <t>Empresas de Flávio e do Careca dividem a mesma sala (brasildefato.com.br) https://www.brasildefato.com.br/2026/09/11/empresas-de-flavio-bolsonaro-e-careca-do-inss-dividem-a-mesma-sala-em-brasilia/ | Mesma sala e mesmo contador (bahianoticias.com.br) https://www.bahianoticias.com.br/noticia/321055-empresas-de-flavio-bolsonaro-e-do-careca-do-inss-dividem-a-mesma-sala-e-possuem-o-mesmo-contador</t>
+        </is>
+      </c>
+      <c r="L89" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M89" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="24" t="inlineStr">
+        <is>
+          <t>escw</t>
+        </is>
+      </c>
+      <c r="B90" s="24" t="inlineStr">
+        <is>
+          <t>Escritório de Willer</t>
+        </is>
+      </c>
+      <c r="C90" s="24" t="inlineStr">
+        <is>
+          <t>Willer Tomaz e sua rede</t>
+        </is>
+      </c>
+      <c r="D90" s="24" t="inlineStr">
+        <is>
+          <t>Escritório de advocacia de Willer Tomaz em Brasília. Foi alvo de busca da PF em 04/08/2026, na nova fase da Operação Sem Desconto, quando os agentes encontraram uma máquina de contar cédulas.</t>
+        </is>
+      </c>
+      <c r="E90" s="24" t="inlineStr">
+        <is>
+          <t>Brasília (DF)</t>
+        </is>
+      </c>
+      <c r="F90" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G90" s="24" t="inlineStr">
+        <is>
+          <t>Alvo de busca e apreensão autorizada por André Mendonça.</t>
+        </is>
+      </c>
+      <c r="H90" s="24" t="inlineStr">
+        <is>
+          <t>Bem citado</t>
+        </is>
+      </c>
+      <c r="I90" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J90" s="24" t="inlineStr">
+        <is>
+          <t>O dinheiro escondido em livros-cofre vem do vídeo de origem; as reportagens reverificadas citam a máquina de contar, mas não os livros-cofre. A defesa diz que a busca se deve ao empréstimo pessoal do avião a Weverton.</t>
+        </is>
+      </c>
+      <c r="K90" s="24" t="inlineStr">
+        <is>
+          <t>PF acha máquina de contar cédulas (metropoles.com) https://www.metropoles.com/colunas/mirelle-pinheiro/fraude-no-inss-pf-acha-maquina-de-contar-cedulas-e-pilhas-de-dinheiro | Uma máquina de dinheiro no escritório do advogado (oantagonista.com.br) https://oantagonista.com.br/brasil/uma-maquina-de-dinheiro-no-escritorio-do-advogado-ligado-a-weverton-rocha/</t>
+        </is>
+      </c>
+      <c r="L90" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M90" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="24" t="inlineStr">
+        <is>
+          <t>assoc</t>
+        </is>
+      </c>
+      <c r="B91" s="24" t="inlineStr">
+        <is>
+          <t>Associações de aposentados</t>
+        </is>
+      </c>
+      <c r="C91" s="24" t="inlineStr">
+        <is>
+          <t>Esquema do INSS</t>
+        </is>
+      </c>
+      <c r="D91" s="24" t="inlineStr">
+        <is>
+          <t>Entidades que descontavam mensalidades direto de aposentadorias e pensões do INSS. PF e CGU estimam R$ 6,3 bi descontados entre 2019 e 2024; em pesquisa da CGU, 97% dos beneficiários ouvidos disseram não ter autorizado. A Operação Sem Desconto (abr/2025) derrubou o presidente do INSS, e o dinheiro passava pelo esquema atribuído ao Careca do INSS.</t>
+        </is>
+      </c>
+      <c r="E91" s="24" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="F91" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G91" s="24" t="inlineStr">
+        <is>
+          <t>Convênios suspensos; o governo prometeu ressarcir os aposentados.</t>
+        </is>
+      </c>
+      <c r="H91" s="24" t="inlineStr">
+        <is>
+          <t>Investigado / alvo (sem denúncia)</t>
+        </is>
+      </c>
+      <c r="I91" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J91" s="24" t="inlineStr">
+        <is>
+          <t>Nem todo o valor é ilegal: parte dos segurados autorizou os descontos.</t>
+        </is>
+      </c>
+      <c r="K91" s="24" t="inlineStr">
+        <is>
+          <t>Como funcionava o esquema de fraude no INSS (opovo.com.br) https://www.opovo.com.br/noticias/brasil/2025/04/30/como-funcionava-o-esquema-bilionario-de-fraude-no-inss.html | Crise no INSS (congressoemfoco.com.br) https://www.congressoemfoco.com.br/noticia/108221/crise-no-inss-entenda-escandalo-que-derrubou-ministro-da-previdencia</t>
+        </is>
+      </c>
+      <c r="L91" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="M91" s="24" t="inlineStr">
+        <is>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:P36"/>
@@ -5012,7 +9057,7 @@
       </c>
       <c r="B34" s="45" t="inlineStr">
         <is>
-          <t>Luri Eventos</t>
+          <t>Allure Eventos</t>
         </is>
       </c>
       <c r="C34" s="45" t="inlineStr">
@@ -6661,7 +10706,7 @@
       </c>
       <c r="E80" s="45" t="inlineStr">
         <is>
-          <t>Robson Calixto, PM da reserva condenado no caso Marielle; PF diz que intermediou emenda de Flávio</t>
+          <t>PM da reserva condenado no caso Marielle (organização criminosa); PF diz que intermediou emenda de Flávio</t>
         </is>
       </c>
       <c r="F80" s="45">
@@ -6906,7 +10951,7 @@
       </c>
       <c r="E87" s="45" t="inlineStr">
         <is>
-          <t>Processava pagamentos da Loterj; contrato rescindido pelo estado, que cobra ~R$ 4 mi</t>
+          <t>Processava pagamentos das bets da Loterj; o estado rescindiu em set/2026 e cobra R$ 9,4 mi (liminar suspendeu)</t>
         </is>
       </c>
       <c r="F87" s="45">
@@ -12856,7 +16901,7 @@
       </c>
       <c r="C193" s="45" t="inlineStr">
         <is>
-          <t>Contratou em 2023; o estado rescindiu e cobra ~R$ 4 mi, a empresa contesta</t>
+          <t>Contratou em 2023; o estado rescindiu em set/2026 e cobra R$ 9,4 mi (liminar suspendeu); a empresa contesta</t>
         </is>
       </c>
       <c r="D193" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Remove menção ao nome antigo (Luri) do perfil da Allure Eventos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018rccqzzxrj3q4wcvp7v91m
</commit_message>
<xml_diff>
--- a/data/mapa.xlsx
+++ b/data/mapa.xlsx
@@ -7094,7 +7094,7 @@
       </c>
       <c r="J80" s="24" t="inlineStr">
         <is>
-          <t>O nó se chamava "Luri Eventos", provável erro de transcrição do vídeo; as reportagens grafam Allure Eventos (confirmado em 22/10/2026). O dono confirma o interesse de Vorcaro, mas nega que a compra tenha avançado e contesta a versão das mensagens. Uma das reportagens não afirma explicitamente que a Allure é a agência usada no recrutamento.</t>
+          <t>O dono confirma o interesse de Vorcaro, mas nega que a compra tenha avançado e contesta a versão das mensagens. Uma das reportagens não afirma explicitamente que a Allure é a agência usada no recrutamento.</t>
         </is>
       </c>
       <c r="K80" s="24" t="inlineStr">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="M80" s="24" t="inlineStr">
         <is>
-          <t>22/10/2026: rodada contexto e imagens (perfil novo). 22/10/2026: renomeado de "Luri Eventos" para "Allure Eventos".</t>
+          <t>22/10/2026: rodada contexto e imagens (perfil novo).</t>
         </is>
       </c>
     </row>

</xml_diff>